<commit_message>
monitor: high run 2026-05-21T14:25Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -3775,7 +3775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3975,9 +3975,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4005,9 +4002,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4035,9 +4029,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4065,9 +4056,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4095,9 +4083,6 @@
           <t>New 8-K filed 2026-05-08 (accession 0001594805-26-000022)</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4125,9 +4110,6 @@
           <t>New 144 filed 2026-05-05 (accession 0001950047-26-004066)</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4155,9 +4137,6 @@
           <t>New S-8 POS filed 2026-05-05 (accession 0001594805-26-000020)</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4185,9 +4164,6 @@
           <t>New 10-Q filed 2026-05-05 (accession 0001594805-26-000019)</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4215,9 +4191,6 @@
           <t>New 8-K filed 2026-05-05 (accession 0001594805-26-000018)</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4245,9 +4218,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4275,9 +4245,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4305,9 +4272,6 @@
           <t>New 4 filed 2026-05-19 (accession 0001731746-26-000002)</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4335,9 +4299,6 @@
           <t>New 144 filed 2026-05-15 (accession 0001969223-26-000559)</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4365,9 +4326,6 @@
           <t>New 4 filed 2026-05-05 (accession 0002068229-26-000009)</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4395,9 +4353,6 @@
           <t>New 4 filed 2026-05-05 (accession 0001525358-26-000012)</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4425,9 +4380,6 @@
           <t>New 4 filed 2026-05-05 (accession 0002047113-26-000006)</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4455,9 +4407,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4485,9 +4434,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4515,9 +4461,6 @@
           <t>New SCHEDULE 13G/A filed 2026-05-15 (accession 0000905148-26-002425)</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4545,9 +4488,6 @@
           <t>New SCHEDULE 13G filed 2026-05-14 (accession 0001167557-26-000087)</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4575,9 +4515,6 @@
           <t>New 4 filed 2026-05-05 (accession 0001766502-26-000048)</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4605,9 +4542,6 @@
           <t>New 4 filed 2026-05-05 (accession 0001766502-26-000047)</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4635,9 +4569,6 @@
           <t>New 4 filed 2026-05-05 (accession 0001766502-26-000046)</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4665,9 +4596,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4695,9 +4623,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4725,9 +4650,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4755,9 +4677,6 @@
           <t>New 4 filed 2026-05-19 (accession 0001628280-26-036519)</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4785,9 +4704,6 @@
           <t>New 4 filed 2026-05-19 (accession 0001628280-26-036518)</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4815,9 +4731,6 @@
           <t>New 4 filed 2026-05-19 (accession 0001628280-26-036517)</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4845,9 +4758,6 @@
           <t>New 144 filed 2026-05-18 (accession 0001950047-26-004684)</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4875,9 +4785,6 @@
           <t>New 144 filed 2026-05-18 (accession 0001950047-26-004683)</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4905,9 +4812,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4935,9 +4839,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4965,9 +4866,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4995,9 +4893,6 @@
           <t>New 10-Q filed 2026-05-08 (accession 0001628280-26-032387)</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5025,9 +4920,6 @@
           <t>New 8-K filed 2026-05-07 (accession 0001628280-26-032064)</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5055,9 +4947,6 @@
           <t>New SCHEDULE 13G filed 2026-04-29 (accession 0002100121-26-000146)</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5085,9 +4974,6 @@
           <t>New SCHEDULE 13G/A filed 2026-03-27 (accession 0000102909-26-001417)</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5115,9 +5001,6 @@
           <t>New 8-K filed 2026-03-16 (accession 0001628280-26-018149)</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5145,9 +5028,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5175,9 +5055,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5205,9 +5082,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5235,9 +5109,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5265,9 +5136,6 @@
           <t>New SD filed 2026-05-19 (accession 0001650164-26-000119)</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5295,9 +5163,6 @@
           <t>New SCHEDULE 13G/A filed 2026-05-15 (accession 0001193125-26-227328)</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5325,9 +5190,6 @@
           <t>New SCHEDULE 13G/A filed 2026-05-14 (accession 0001562230-26-000100)</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5355,9 +5217,6 @@
           <t>New S-8 filed 2026-05-08 (accession 0001650164-26-000116)</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5385,9 +5244,6 @@
           <t>New 10-Q filed 2026-05-08 (accession 0001650164-26-000114)</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5415,9 +5271,6 @@
           <t>New 144 filed 2026-05-20 (accession 0001950047-26-004850)</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5445,9 +5298,6 @@
           <t>New 4 filed 2026-05-19 (accession 0002108589-26-000012)</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5475,9 +5325,6 @@
           <t>New SCHEDULE 13G filed 2026-05-18 (accession 0000950103-26-007332)</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5505,9 +5352,6 @@
           <t>New 8-K filed 2026-05-08 (accession 0001783879-26-000065)</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5535,9 +5379,36 @@
           <t>New 4 filed 2026-05-06 (accession 0001705560-26-000011)</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Duolingo Inc.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://blog.duolingo.com/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: high run 2026-05-21T17:41Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -3775,7 +3775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5406,9 +5406,36 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: high run 2026-05-22T13:42Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -3775,7 +3775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5433,9 +5433,96 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>CHWY</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Chewy Inc.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1766502/000114036126022531/ny20064174x3_ars.pdf</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>New ARS filed 2026-05-22 (accession 0001140361-26-022531)</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>CHWY</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Chewy Inc.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1766502/000114036126022530/ny20064174x2_defa14a.htm</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>New DEFA14A filed 2026-05-22 (accession 0001140361-26-022530)</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>CHWY</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Chewy Inc.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1766502/000114036126022529/ny20064174x1_def14a.htm</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>New DEF 14A filed 2026-05-22 (accession 0001140361-26-022529)</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: high run 2026-05-22T17:24Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -3775,7 +3775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5460,9 +5460,6 @@
           <t>New ARS filed 2026-05-22 (accession 0001140361-26-022531)</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5490,9 +5487,6 @@
           <t>New DEFA14A filed 2026-05-22 (accession 0001140361-26-022530)</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5520,9 +5514,36 @@
           <t>New DEF 14A filed 2026-05-22 (accession 0001140361-26-022529)</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: high run 2026-05-22T20:52Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -3775,7 +3775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5541,9 +5541,36 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ETSY</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Etsy Inc.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1370637/000195004726004998/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-22 (accession 0001950047-26-004998)</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: high run 2026-05-22T22:22Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -3775,7 +3775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5568,9 +5568,36 @@
           <t>New 144 filed 2026-05-22 (accession 0001950047-26-004998)</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1783879/000187091426000011/xslF345X06/wk-form4_1779483458.xml</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-22 (accession 0001870914-26-000011)</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: high run 2026-05-23T00:21Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -3775,7 +3775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5595,9 +5595,36 @@
           <t>New 4 filed 2026-05-22 (accession 0001870914-26-000011)</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>BILL</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>BILL Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://www.bill.com/legal/terms-of-service</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: high run 2026-05-26T14:17Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -3775,7 +3775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5622,9 +5622,96 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://investors.shopify.com</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Duolingo Inc.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://blog.duolingo.com/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: high run 2026-05-26T21:06Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -3775,7 +3775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5649,9 +5649,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5679,9 +5676,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5709,9 +5703,66 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ETSY</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Etsy Inc.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1370637/000122768826000004/xslF345X06/form4-05262026_040501.xml</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-26 (accession 0001227688-26-000004)</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>BILL</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>BILL Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1786352/000119312526239245/d931634d8k.htm</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>New 8-K filed 2026-05-26 (accession 0001193125-26-239245)</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add multi-ticker support and test on SHOP/WIX/DASH/CART
- run.py --ticker now accepts comma-separated list (e.g. SHOP,WIX,DASH,CART)
- Re-applied Phase 0 URL fixes that were lost in the earlier rebase merge
- First run on 4 names: 37 flagged changes (all "new snapshot" baselines +
  initial EDGAR findings, capped at 5 per company)
- Second run: 0 flagged changes — diff machinery confirmed working
- Known issues to address in Phase 1:
  - DASH/pricing returns 404 on the new merchants.doordash.com URL
  - CART investors.instacart.com IR timeouts (bot blocking from runner IP)
  - EDGAR captures all Form 4 insider filings — noisy for active names
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -670,7 +670,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>https://investors.shopify.com/corporate-governance/board-of-directors-and-management/default.aspx</t>
+          <t>https://www.shopify.com/investors/board-of-directors</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -747,12 +747,12 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.wix.com/blog/news</t>
+          <t>https://www.wix.com/press-room/home</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>https://investors.wix.com/corporate-governance/board-and-executives</t>
+          <t>https://investors.wix.com/board-of-directors</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.global-e.com/blog/</t>
+          <t>https://www.global-e.com/media-centre/</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -840,12 +840,12 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>https://www.global-e.com/solutions/</t>
+          <t>https://www.global-e.com/platform/</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>https://www.global-e.com/legal/terms-of-service/</t>
+          <t>https://www.global-e.com/terms/</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>https://newsroom.godaddy.com/about-godaddy/executive-team/</t>
+          <t>https://aboutus.godaddy.net/about-us/team/default.aspx</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>https://investors.ebayinc.com/leadership/default.aspx</t>
+          <t>https://investors.ebayinc.com/corporate-governance/board-of-directors/default.aspx</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>https://www.ebay.com/sellercenter/resources/selling-fees</t>
+          <t>https://www.ebay.com/sellercenter/selling/start-selling-on-ebay/seller-fees</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>https://investor.wayfair.com/leadership/default.aspx</t>
+          <t>https://www.aboutwayfair.com/leadership</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>https://investors.etsy.com/leadership/default.aspx</t>
+          <t>https://investors.etsy.com/company-information/executive-team</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -1215,12 +1215,12 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://investor.chewy.com/news-releases</t>
+          <t>https://investor.chewy.com/news-and-events/news/default.aspx</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>https://investor.chewy.com/leadership/default.aspx</t>
+          <t>https://investor.chewy.com/governance/executive-management/default.aspx</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>https://ir.doordash.com/leadership/default.aspx</t>
+          <t>https://ir.doordash.com/governance/management/default.aspx</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>https://get.doordash.com/en-us/products/merchant-pricing</t>
+          <t>https://merchants.doordash.com/en-us/products/merchant-pricing</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.instacart.com/company/news/</t>
+          <t>https://www.instacart.com/company/newsroom</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>https://www.instacart.com/plans</t>
+          <t>https://www.instacart.com/instacart-plus</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://ir.mtch.com/news-releases</t>
+          <t>https://ir.mtch.com/investor-relations/news-events/news-events/default.aspx</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>https://investors.zillowgroup.com/board-and-management/leadership</t>
+          <t>https://www.zillowgroup.com/about-us/our-leaders/</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>https://www.zillowgroup.com/zg-terms-of-use/</t>
+          <t>https://www.zillow.com/z/corp/terms/</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>https://ir.rocketcompanies.com/leadership/default.aspx</t>
+          <t>https://www.rocketcompanies.com/our-team/leadership/</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>https://investors.compass.com/leadership/default.aspx</t>
+          <t>https://investors.compass.com/governance/management/default.aspx</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>https://www.compass.com/terms/</t>
+          <t>https://www.compass.com/legal/terms-of-service/</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
@@ -1927,12 +1927,12 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>https://www.appfolio.com/careers/</t>
+          <t>https://www.appfolio.com/company/careers</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>https://www.appfolio.com/property-manager/pricing/</t>
+          <t>https://www.appfolio.com/pricing</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>https://block.xyz/about</t>
+          <t>https://investors.block.xyz/governance/leadership/default.aspx</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>https://squareup.com/us/en/payments/our-rates</t>
+          <t>https://squareup.com/us/en/payments/our-fees</t>
         </is>
       </c>
       <c r="I19" s="10" t="inlineStr">
@@ -2073,12 +2073,12 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.bill.com/resource/press-releases</t>
+          <t>https://www.bill.com/press-release</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>https://investor.bill.com/leadership/default.aspx</t>
+          <t>https://www.bill.com/leadership</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>https://investor.pypl.com/leadership/default.aspx</t>
+          <t>https://about.pypl.com/who-we-are/executive-leadership/default.aspx</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>https://www.paypal.com/us/legalhub/paypal-user-agreement-full</t>
+          <t>https://www.paypal.com/us/legalhub/paypal/useragreement-full</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>https://investors.toasttab.com/leadership/default.aspx</t>
+          <t>https://pos.toasttab.com/leadership</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -2307,12 +2307,12 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>https://www.adyen.com/news</t>
+          <t>https://www.adyen.com/press-and-media</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>https://investors.adyen.com/about-adyen/management-board</t>
+          <t>https://www.adyen.com/about/team</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>https://investors.adyen.com/financial-results</t>
+          <t>https://investors.adyen.com/financials</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>https://www.sezzle.com/</t>
+          <t>https://sezzle.com/premium/</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -2478,12 +2478,12 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>https://dave.com/</t>
+          <t>https://dave.com/extra-cash-account</t>
         </is>
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>https://dave.com/legal/terms-of-service</t>
+          <t>https://dave.com/terms/</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://zip.co/media</t>
+          <t>https://zip.co/investors/news</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -2561,12 +2561,12 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>https://help.zip.co/hc/en-us/articles/360000750996-Terms-of-Use</t>
+          <t>https://zip.co/au/page/important-information</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>https://www.asx.com.au/asx/share-price-research/company/ZIP</t>
+          <t>https://zip.co/investors/asx-announcements</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>https://www.klarna.com/international/about-klarna/leadership/</t>
+          <t>https://investors.klarna.com/governance/leadership/default.aspx</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="I28" s="10" t="inlineStr">
         <is>
-          <t>https://www.klarna.com/us/legal/terms-of-use/</t>
+          <t>https://www.klarna.com/us/terms-of-use/</t>
         </is>
       </c>
       <c r="J28" s="10" t="inlineStr">
@@ -2790,12 +2790,12 @@
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>https://robinhood.com/us/en/support/articles/fees-and-charges/</t>
+          <t>https://robinhood.com/us/en/support/articles/trading-fees-on-robinhood/</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>https://robinhood.com/us/en/support/articles/customer-agreement/</t>
+          <t>https://cdn.robinhood.com/assets/robinhood/legal/Robinhood-Customer-Agreement.pdf</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>https://www.upstart.com/legal/terms-of-use</t>
+          <t>https://www.upstart.com/terms</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>https://ir.rh.com/leadership/default.aspx</t>
+          <t>https://ir.rh.com/corporate-governance/leadership</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>https://www.williams-sonoma.com/customer-service/terms-of-use.html</t>
+          <t>https://www.williams-sonoma.com/m/customer-service/terms.html</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>https://www.tempurpedic.com/mattresses/</t>
+          <t>https://www.tempurpedic.com/shop-mattresses/</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
@@ -3165,12 +3165,12 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://ir.enova.com/news-releases</t>
+          <t>https://ir.enova.com/news-events/news-releases/default.aspx</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>https://ir.enova.com/leadership/default.aspx</t>
+          <t>https://ir.enova.com/corporate-governance/leadership-team/default.aspx</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -3180,12 +3180,12 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>https://www.enova.com/products/</t>
+          <t>https://www.enova.com/brands/</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>https://www.enova.com/legal/terms-of-use/</t>
+          <t>https://www.enova.com/terms-conditions/</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>https://investors.on.com/corporate-governance/board-of-directors</t>
+          <t>https://investors.on-running.com/governance/default.aspx</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -3775,7 +3775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H143"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5730,9 +5730,6 @@
           <t>New 4 filed 2026-05-26 (accession 0001227688-26-000004)</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5760,9 +5757,1953 @@
           <t>New 8-K filed 2026-05-26 (accession 0001193125-26-239245)</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/legal/terms</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://news.shopify.com</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://investors.shopify.com</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000022/shop-20260508.htm</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>New 8-K filed 2026-05-08 (accession 0001594805-26-000022)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000195004726004066/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-05 (accession 0001950047-26-004066)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000020/forms-8postxeffectiveamend.htm</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>New S-8 POS filed 2026-05-05 (accession 0001594805-26-000020)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000019/shop-20260331.htm</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>New 10-Q filed 2026-05-05 (accession 0001594805-26-000019)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000018/shop-20260505.htm</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>New 8-K filed 2026-05-05 (accession 0001594805-26-000018)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://support.wix.com/en/article/terms-of-use</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/upgrade/website</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://investors.wix.com</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000119312526225926/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>New SCHEDULE 13G/A filed 2026-05-15 (accession 0001193125-26-225926)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000090266426002441/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>New SCHEDULE 13G/A filed 2026-05-14 (accession 0000902664-26-002441)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000117266126001868/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>New SCHEDULE 13G filed 2026-05-14 (accession 0001172661-26-001868)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000117891326002642/zk2635313.htm</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002642)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000117891326002640/zk2635312.htm</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002640)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://help.doordash.com/consumers/s/terms-of-service</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://about.doordash.com/en-us/news</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726005086/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-26 (accession 0001950047-26-005086)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726005081/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-26 (accession 0001950047-26-005081)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726004985/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-22 (accession 0001950047-26-004985)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726004984/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-22 (accession 0001950047-26-004984)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183239026000011/xslF345X06/form4-05222026_040501.xml</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-22 (accession 0001832390-26-000011)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/terms</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000165168726000009/xslF345X06/wk-form4_1779221300.xml</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0001651687-26-000009)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000202205026000007/xslF345X06/wk-form4_1779221163.xml</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0002022050-26-000007)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000199010626000014/xslF345X06/wk-form4_1779221074.xml</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0001990106-26-000014)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000208293026000008/xslF345X06/wk-form4_1779220992.xml</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0002082930-26-000008)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000192109426000512/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-18 (accession 0001921094-26-000512)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/legal/terms</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/investors/board-of-directors</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://news.shopify.com</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://investors.shopify.com</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000022/shop-20260508.htm</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>New 8-K filed 2026-05-08 (accession 0001594805-26-000022)</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000195004726004066/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-05 (accession 0001950047-26-004066)</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000020/forms-8postxeffectiveamend.htm</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>New S-8 POS filed 2026-05-05 (accession 0001594805-26-000020)</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000019/shop-20260331.htm</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>New 10-Q filed 2026-05-05 (accession 0001594805-26-000019)</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000018/shop-20260505.htm</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>New 8-K filed 2026-05-05 (accession 0001594805-26-000018)</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://support.wix.com/en/article/terms-of-use</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://investors.wix.com/board-of-directors</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/upgrade/website</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://investors.wix.com</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000119312526225926/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>New SCHEDULE 13G/A filed 2026-05-15 (accession 0001193125-26-225926)</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000090266426002441/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>New SCHEDULE 13G/A filed 2026-05-14 (accession 0000902664-26-002441)</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000117266126001868/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>New SCHEDULE 13G filed 2026-05-14 (accession 0001172661-26-001868)</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000117891326002642/zk2635313.htm</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002642)</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000117891326002640/zk2635312.htm</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002640)</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://help.doordash.com/consumers/s/terms-of-service</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com/governance/management/default.aspx</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://about.doordash.com/en-us/news</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726005086/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-26 (accession 0001950047-26-005086)</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726005081/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-26 (accession 0001950047-26-005081)</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726004985/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-22 (accession 0001950047-26-004985)</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726004984/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-22 (accession 0001950047-26-004984)</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183239026000011/xslF345X06/form4-05222026_040501.xml</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-22 (accession 0001832390-26-000011)</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/terms</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/instacart-plus</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/company/newsroom</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000165168726000009/xslF345X06/wk-form4_1779221300.xml</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0001651687-26-000009)</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000202205026000007/xslF345X06/wk-form4_1779221163.xml</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0002022050-26-000007)</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000199010626000014/xslF345X06/wk-form4_1779221074.xml</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0001990106-26-000014)</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000208293026000008/xslF345X06/wk-form4_1779220992.xml</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0002082930-26-000008)</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000192109426000512/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-18 (accession 0001921094-26-000512)</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Phase 1A-1C: metadata columns + RSS for newsroom scraping
Phase 1A: added Priority Tier and Active columns to URL Registry; config_reader
now reads tier from xlsx (falls back to tiers.py) and skips Active=FALSE rows.

Phase 1B: tools/discover_rss.py probes /feed, /rss, /rss.xml and HTML auto-
discovery. Findings for the 4 test names: WIX has live feed; SHOP feed is
stale (2023); DASH and CART have no RSS.

Phase 1C: scrapers/rss.py uses requests+feedparser to fetch newsroom feeds
and emits one Change per new entry. GUIDs are persisted per (ticker,source)
so the same press release never alerts twice. run.py now prefers RSS for
newsroom when xlsx column 'Newsroom RSS' is populated; falls back to HTML
scrape otherwise.

Output quality: WIX newsroom now produces 5 entries with real titles, dates,
and 500-char body previews instead of one "change detected — new snapshot"
placeholder. Same machinery, ~10x more informative output.
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,6 +68,9 @@
       <name val="Calibri"/>
       <family val="2"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -136,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -178,6 +181,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -543,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:S36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -641,6 +645,21 @@
           <t>Monitoring Notes</t>
         </is>
       </c>
+      <c r="Q1" s="15" t="inlineStr">
+        <is>
+          <t>Priority Tier</t>
+        </is>
+      </c>
+      <c r="R1" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="S1" s="15" t="inlineStr">
+        <is>
+          <t>Newsroom RSS</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="52" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -723,6 +742,14 @@
           <t>Monitor changelog.shopify.com; App Store changes signal platform strategy</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -801,6 +828,19 @@
           <t>Israeli co; files 20-F; monitor Studio AI website builder product</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R3" t="b">
+        <v>1</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home/blog-feed.xml</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="52" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -879,6 +919,14 @@
           <t>Israeli co; files 20-F; watch Shopify partnership; merchant wins are leading indicator</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" ht="52" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -957,6 +1005,14 @@
           <t>Monitor Airo AI product and domain pricing; SMB pricing changes are material</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -1035,6 +1091,14 @@
           <t>Seller fee changes are key signal; also watch eBay Seller Hub announcements</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -1113,6 +1177,14 @@
           <t>Monitor supplier portal for supplier terms; tech/engineering headcount is leading indicator</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1191,6 +1263,14 @@
           <t>Also monitor r/EtsySellers — seller sentiment is material; transaction fee changes cause seller exodus</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" ht="52" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -1269,6 +1349,14 @@
           <t>Autoship pricing and Chewy Vet telehealth are key monitoring targets</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" ht="52" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1347,6 +1435,14 @@
           <t>Monitor DashPass pricing and merchant commission; also r/doordash_drivers for gig sentiment</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" ht="52" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1425,6 +1521,14 @@
           <t>Instacart+ subscription pricing; Carrot Ads advertising product is key growth vector</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" ht="52" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1503,6 +1607,14 @@
           <t>Super/Max subscription pricing is key; AI feature rollouts have been material catalysts</t>
         </is>
       </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" ht="52" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1581,6 +1693,14 @@
           <t>Monitor Tinder Gold/Platinum and Hinge subscription pricing separately; track Hinge product blog</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" ht="52" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1659,6 +1779,14 @@
           <t>Agent pricing (Premier Agent) is key; also monitor ShowingTime and Follow Up Boss products</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R14" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" ht="52" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1737,6 +1865,14 @@
           <t>Monitor Homes.com product page separately; aggressively investing in residential — track agent sign-up terms</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R15" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" ht="52" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1815,6 +1951,14 @@
           <t>Mortgage rate page is real-time signal; monitor Rocket Money product pages for cross-sell</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R16" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" ht="52" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -1893,6 +2037,14 @@
           <t>Agent commission splits and technology platform terms are key; agent count and retention are leading indicators</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" ht="52" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1971,6 +2123,14 @@
           <t>Pricing page changes (per-unit pricing) are highly material; AppFolio Intelligence AI is key</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R18" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="19" ht="52" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
@@ -2049,6 +2209,14 @@
           <t>⚠️ VERIFY TICKER: Block typically trades as SQ — confirm XYZ. TWO product/pricing pages to monitor: Square rates (squareup.com/us/en/payments/our-rates) AND Cash App (cash.app). Square T&amp;C: squareup.com/us/en/legal/general/ua. Cash App T&amp;C: cash.app/legal/us/en/tos.</t>
         </is>
       </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R19" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="20" ht="52" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -2127,6 +2295,14 @@
           <t>Pricing page is key — tier structure for AP/AR automation; also track Divvy spend management product</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R20" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="21" ht="52" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -2205,6 +2381,14 @@
           <t>Merchant fee changes are highly material; also monitor Venmo monetisation and PayPal Everywhere</t>
         </is>
       </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="22" ht="52" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -2283,6 +2467,14 @@
           <t>Pricing page (processing rate + SaaS fee) is highly material; also track Toast Capital lending product</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R22" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="23" ht="52" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -2361,6 +2553,14 @@
           <t>Dutch co; H1/H2 reporting only (not quarterly); pricing page is particularly informative on take-rate trends</t>
         </is>
       </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="R23" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="24" ht="52" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -2439,6 +2639,14 @@
           <t>Small-cap BNPL; monitor merchant partner announcements and Sezzle Premium subscription terms</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R24" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="25" ht="52" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -2517,6 +2725,14 @@
           <t>ExtraCash advance limits and fee structure are key monitoring targets; also track Dave Banking product</t>
         </is>
       </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R25" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="26" ht="52" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -2595,6 +2811,14 @@
           <t>ASX-listed; H1/FY reports only; merchant fee changes are key</t>
         </is>
       </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="R26" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="27" ht="52" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -2673,6 +2897,14 @@
           <t>Monitor merchant partner page for new integrations; Affirm Card (Debit+) is key growth vector</t>
         </is>
       </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R27" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="28" ht="52" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -2751,6 +2983,14 @@
           <t>⚠️ VERIFY: Recently IPO'd on NYSE — confirm IR URL and SEC filings link. Monitor AI shopping assistant product closely.</t>
         </is>
       </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R28" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="29" ht="52" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -2829,6 +3069,14 @@
           <t>Monitor Robinhood Gold pricing and Legend desktop platform; international expansion is key signal</t>
         </is>
       </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R29" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="30" ht="52" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -2907,6 +3155,14 @@
           <t>Bank/CU partnership announcements are key leading indicators; monitor auto loan and HELOC product expansion</t>
         </is>
       </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R30" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="31" ht="52" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -2985,6 +3241,14 @@
           <t>RH Membership pricing is key; monitor RH Hospitality expansion; Gary Friedman letters to shareholders are essential reading</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R31" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="32" ht="52" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -3063,6 +3327,14 @@
           <t>Monitor all brands: West Elm, Pottery Barn, Rejuvenation; B2B contract business is underappreciated</t>
         </is>
       </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R32" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="33" ht="52" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -3141,6 +3413,14 @@
           <t>Fmr. Tempur Sealy (TPX); renamed + rebranded Feb 2025. Owns Tempur-Pedic, Sealy, Stearns &amp; Foster brands + Mattress Firm retail chain. Monitor all three brand sites separately: tempurpedic.com, sealy.com, mattressfirm.com.</t>
         </is>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R33" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="34" ht="52" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -3219,6 +3499,14 @@
           <t>Regulatory news (CFPB rules on installment lending) is major risk signal; monitor NetCredit and CashNetUSA</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R34" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="35" ht="52" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -3297,6 +3585,14 @@
           <t>Swiss co; files 20-F; monitor DTC expansion and Loewe collaboration; trail/Cloudmonster launches signal brand trajectory</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="36" ht="52" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -3374,6 +3670,14 @@
         <is>
           <t>Japanese character IP co (Hello Kitty, My Melody, Cinnamoroll etc.); TSE 8136; monitor global licensing deal announcements, theme park updates (Sanrio Puroland), and US/Americas expansion (Craig Takiguchi named CEO Americas Jan 2026).</t>
         </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="R36" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3775,7 +4079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H143"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6621,9 +6925,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr"/>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6651,9 +6952,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6681,9 +6979,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -6711,9 +7006,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -6741,9 +7033,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -6771,9 +7060,6 @@
           <t>New 8-K filed 2026-05-08 (accession 0001594805-26-000022)</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -6801,9 +7087,6 @@
           <t>New 144 filed 2026-05-05 (accession 0001950047-26-004066)</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -6831,9 +7114,6 @@
           <t>New S-8 POS filed 2026-05-05 (accession 0001594805-26-000020)</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr"/>
-      <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6861,9 +7141,6 @@
           <t>New 10-Q filed 2026-05-05 (accession 0001594805-26-000019)</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr"/>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6891,9 +7168,6 @@
           <t>New 8-K filed 2026-05-05 (accession 0001594805-26-000018)</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr"/>
-      <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -6921,9 +7195,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr"/>
-      <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6951,9 +7222,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr"/>
-      <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6981,9 +7249,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr"/>
-      <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -7011,9 +7276,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr"/>
-      <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -7041,9 +7303,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr"/>
-      <c r="G121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -7071,9 +7330,6 @@
           <t>New SCHEDULE 13G/A filed 2026-05-15 (accession 0001193125-26-225926)</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
-      <c r="G122" t="inlineStr"/>
-      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -7101,9 +7357,6 @@
           <t>New SCHEDULE 13G/A filed 2026-05-14 (accession 0000902664-26-002441)</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr"/>
-      <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -7131,9 +7384,6 @@
           <t>New SCHEDULE 13G filed 2026-05-14 (accession 0001172661-26-001868)</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr"/>
-      <c r="G124" t="inlineStr"/>
-      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -7161,9 +7411,6 @@
           <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002642)</t>
         </is>
       </c>
-      <c r="F125" t="inlineStr"/>
-      <c r="G125" t="inlineStr"/>
-      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -7191,9 +7438,6 @@
           <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002640)</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr"/>
-      <c r="G126" t="inlineStr"/>
-      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -7221,9 +7465,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr"/>
-      <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -7251,9 +7492,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr"/>
-      <c r="G128" t="inlineStr"/>
-      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -7281,9 +7519,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr"/>
-      <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -7311,9 +7546,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr"/>
-      <c r="G130" t="inlineStr"/>
-      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -7341,9 +7573,6 @@
           <t>New 144 filed 2026-05-26 (accession 0001950047-26-005086)</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr"/>
-      <c r="G131" t="inlineStr"/>
-      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -7371,9 +7600,6 @@
           <t>New 144 filed 2026-05-26 (accession 0001950047-26-005081)</t>
         </is>
       </c>
-      <c r="F132" t="inlineStr"/>
-      <c r="G132" t="inlineStr"/>
-      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -7401,9 +7627,6 @@
           <t>New 144 filed 2026-05-22 (accession 0001950047-26-004985)</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr"/>
-      <c r="G133" t="inlineStr"/>
-      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -7431,9 +7654,6 @@
           <t>New 144 filed 2026-05-22 (accession 0001950047-26-004984)</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr"/>
-      <c r="G134" t="inlineStr"/>
-      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -7461,9 +7681,6 @@
           <t>New 4 filed 2026-05-22 (accession 0001832390-26-000011)</t>
         </is>
       </c>
-      <c r="F135" t="inlineStr"/>
-      <c r="G135" t="inlineStr"/>
-      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -7491,9 +7708,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F136" t="inlineStr"/>
-      <c r="G136" t="inlineStr"/>
-      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -7521,9 +7735,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr"/>
-      <c r="G137" t="inlineStr"/>
-      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -7551,9 +7762,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F138" t="inlineStr"/>
-      <c r="G138" t="inlineStr"/>
-      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -7581,9 +7789,6 @@
           <t>New 4 filed 2026-05-19 (accession 0001651687-26-000009)</t>
         </is>
       </c>
-      <c r="F139" t="inlineStr"/>
-      <c r="G139" t="inlineStr"/>
-      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -7611,9 +7816,6 @@
           <t>New 4 filed 2026-05-19 (accession 0002022050-26-000007)</t>
         </is>
       </c>
-      <c r="F140" t="inlineStr"/>
-      <c r="G140" t="inlineStr"/>
-      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -7641,9 +7843,6 @@
           <t>New 4 filed 2026-05-19 (accession 0001990106-26-000014)</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr"/>
-      <c r="G141" t="inlineStr"/>
-      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -7671,9 +7870,6 @@
           <t>New 4 filed 2026-05-19 (accession 0002082930-26-000008)</t>
         </is>
       </c>
-      <c r="F142" t="inlineStr"/>
-      <c r="G142" t="inlineStr"/>
-      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7701,9 +7897,1236 @@
           <t>New 144 filed 2026-05-18 (accession 0001921094-26-000512)</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr"/>
-      <c r="G143" t="inlineStr"/>
-      <c r="H143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/legal/terms</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/investors/board-of-directors</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>https://news.shopify.com</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>https://investors.shopify.com</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000022/shop-20260508.htm</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>New 8-K filed 2026-05-08 (accession 0001594805-26-000022)</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000195004726004066/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-05 (accession 0001950047-26-004066)</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000020/forms-8postxeffectiveamend.htm</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>New S-8 POS filed 2026-05-05 (accession 0001594805-26-000020)</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000019/shop-20260331.htm</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>New 10-Q filed 2026-05-05 (accession 0001594805-26-000019)</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000018/shop-20260505.htm</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>New 8-K filed 2026-05-05 (accession 0001594805-26-000018)</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home/post/wix-reports-first-quarter-2026-results</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>newsroom: Wix Reports First Quarter 2026 Results</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home/post/wix-to-participate-in-fireside-chat-at-the-2026-jefferies-software-internet-and-ai-conference</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>newsroom: Wix to Participate in Fireside Chat at the 2026 Jefferies Software, Internet, and AI Conference</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home/post/wix-to-announce-first-quarter-2026-results-on-may-13-2026</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>newsroom: Wix to Announce First Quarter 2026 Results on May 13, 2026</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr"/>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home/post/wix-launches-hipaa-compliance-solution-expanding-support-for-health-service-providers-in-the-u-s</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>newsroom: Wix Launches HIPAA Compliance Solution Expanding Support for Health Service Providers in the U.S.</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home/post/wix-announces-final-results-of-modified-dutch-auction-tender-offer</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>newsroom: Wix Announces Final Results of Modified Dutch Auction Tender Offer</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>https://support.wix.com/en/article/terms-of-use</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>https://investors.wix.com/board-of-directors</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr"/>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/upgrade/website</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr"/>
+      <c r="G161" t="inlineStr"/>
+      <c r="H161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>https://investors.wix.com</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000119312526225926/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>New SCHEDULE 13G/A filed 2026-05-15 (accession 0001193125-26-225926)</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000090266426002441/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>New SCHEDULE 13G/A filed 2026-05-14 (accession 0000902664-26-002441)</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000117266126001868/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>New SCHEDULE 13G filed 2026-05-14 (accession 0001172661-26-001868)</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000117891326002642/zk2635313.htm</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002642)</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000117891326002640/zk2635312.htm</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002640)</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr"/>
+      <c r="H167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>https://help.doordash.com/consumers/s/terms-of-service</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr"/>
+      <c r="H168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com/governance/management/default.aspx</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>https://about.doordash.com/en-us/news</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr"/>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr"/>
+      <c r="G171" t="inlineStr"/>
+      <c r="H171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726005086/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-26 (accession 0001950047-26-005086)</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726005081/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-26 (accession 0001950047-26-005081)</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr"/>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726004985/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-22 (accession 0001950047-26-004985)</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726004984/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-22 (accession 0001950047-26-004984)</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr"/>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183239026000011/xslF345X06/form4-05222026_040501.xml</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-22 (accession 0001832390-26-000011)</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/terms</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr"/>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/instacart-plus</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/company/newsroom</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr"/>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000165168726000009/xslF345X06/wk-form4_1779221300.xml</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0001651687-26-000009)</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000202205026000007/xslF345X06/wk-form4_1779221163.xml</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0002022050-26-000007)</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000199010626000014/xslF345X06/wk-form4_1779221074.xml</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0001990106-26-000014)</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr"/>
+      <c r="G182" t="inlineStr"/>
+      <c r="H182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000208293026000008/xslF345X06/wk-form4_1779220992.xml</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0002082930-26-000008)</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000192109426000512/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-18 (accession 0001921094-26-000512)</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-05-27T13:54Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4079,7 +4079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H225"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7924,9 +7924,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr"/>
-      <c r="G144" t="inlineStr"/>
-      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -7954,9 +7951,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F145" t="inlineStr"/>
-      <c r="G145" t="inlineStr"/>
-      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -7984,9 +7978,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr"/>
-      <c r="G146" t="inlineStr"/>
-      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -8014,9 +8005,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F147" t="inlineStr"/>
-      <c r="G147" t="inlineStr"/>
-      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -8044,9 +8032,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr"/>
-      <c r="G148" t="inlineStr"/>
-      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -8074,9 +8059,6 @@
           <t>New 8-K filed 2026-05-08 (accession 0001594805-26-000022)</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr"/>
-      <c r="G149" t="inlineStr"/>
-      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -8104,9 +8086,6 @@
           <t>New 144 filed 2026-05-05 (accession 0001950047-26-004066)</t>
         </is>
       </c>
-      <c r="F150" t="inlineStr"/>
-      <c r="G150" t="inlineStr"/>
-      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -8134,9 +8113,6 @@
           <t>New S-8 POS filed 2026-05-05 (accession 0001594805-26-000020)</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr"/>
-      <c r="G151" t="inlineStr"/>
-      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -8164,9 +8140,6 @@
           <t>New 10-Q filed 2026-05-05 (accession 0001594805-26-000019)</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr"/>
-      <c r="G152" t="inlineStr"/>
-      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -8194,9 +8167,6 @@
           <t>New 8-K filed 2026-05-05 (accession 0001594805-26-000018)</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr"/>
-      <c r="G153" t="inlineStr"/>
-      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -8224,9 +8194,6 @@
           <t>newsroom: Wix Reports First Quarter 2026 Results</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr"/>
-      <c r="G154" t="inlineStr"/>
-      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -8254,9 +8221,6 @@
           <t>newsroom: Wix to Participate in Fireside Chat at the 2026 Jefferies Software, Internet, and AI Conference</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr"/>
-      <c r="G155" t="inlineStr"/>
-      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -8284,9 +8248,6 @@
           <t>newsroom: Wix to Announce First Quarter 2026 Results on May 13, 2026</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr"/>
-      <c r="G156" t="inlineStr"/>
-      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -8314,9 +8275,6 @@
           <t>newsroom: Wix Launches HIPAA Compliance Solution Expanding Support for Health Service Providers in the U.S.</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr"/>
-      <c r="G157" t="inlineStr"/>
-      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -8344,9 +8302,6 @@
           <t>newsroom: Wix Announces Final Results of Modified Dutch Auction Tender Offer</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr"/>
-      <c r="G158" t="inlineStr"/>
-      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -8374,9 +8329,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr"/>
-      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -8404,9 +8356,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F160" t="inlineStr"/>
-      <c r="G160" t="inlineStr"/>
-      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -8434,9 +8383,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr"/>
-      <c r="G161" t="inlineStr"/>
-      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -8464,9 +8410,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr"/>
-      <c r="G162" t="inlineStr"/>
-      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -8494,9 +8437,6 @@
           <t>New SCHEDULE 13G/A filed 2026-05-15 (accession 0001193125-26-225926)</t>
         </is>
       </c>
-      <c r="F163" t="inlineStr"/>
-      <c r="G163" t="inlineStr"/>
-      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -8524,9 +8464,6 @@
           <t>New SCHEDULE 13G/A filed 2026-05-14 (accession 0000902664-26-002441)</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr"/>
-      <c r="G164" t="inlineStr"/>
-      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -8554,9 +8491,6 @@
           <t>New SCHEDULE 13G filed 2026-05-14 (accession 0001172661-26-001868)</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr"/>
-      <c r="G165" t="inlineStr"/>
-      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -8584,9 +8518,6 @@
           <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002642)</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr"/>
-      <c r="G166" t="inlineStr"/>
-      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -8614,9 +8545,6 @@
           <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002640)</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr"/>
-      <c r="G167" t="inlineStr"/>
-      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -8644,9 +8572,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr"/>
-      <c r="G168" t="inlineStr"/>
-      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -8674,9 +8599,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr"/>
-      <c r="G169" t="inlineStr"/>
-      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -8704,9 +8626,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr"/>
-      <c r="G170" t="inlineStr"/>
-      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -8734,9 +8653,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr"/>
-      <c r="G171" t="inlineStr"/>
-      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -8764,9 +8680,6 @@
           <t>New 144 filed 2026-05-26 (accession 0001950047-26-005086)</t>
         </is>
       </c>
-      <c r="F172" t="inlineStr"/>
-      <c r="G172" t="inlineStr"/>
-      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -8794,9 +8707,6 @@
           <t>New 144 filed 2026-05-26 (accession 0001950047-26-005081)</t>
         </is>
       </c>
-      <c r="F173" t="inlineStr"/>
-      <c r="G173" t="inlineStr"/>
-      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -8824,9 +8734,6 @@
           <t>New 144 filed 2026-05-22 (accession 0001950047-26-004985)</t>
         </is>
       </c>
-      <c r="F174" t="inlineStr"/>
-      <c r="G174" t="inlineStr"/>
-      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -8854,9 +8761,6 @@
           <t>New 144 filed 2026-05-22 (accession 0001950047-26-004984)</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr"/>
-      <c r="G175" t="inlineStr"/>
-      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -8884,9 +8788,6 @@
           <t>New 4 filed 2026-05-22 (accession 0001832390-26-000011)</t>
         </is>
       </c>
-      <c r="F176" t="inlineStr"/>
-      <c r="G176" t="inlineStr"/>
-      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -8914,9 +8815,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F177" t="inlineStr"/>
-      <c r="G177" t="inlineStr"/>
-      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -8944,9 +8842,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr"/>
-      <c r="G178" t="inlineStr"/>
-      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -8974,9 +8869,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F179" t="inlineStr"/>
-      <c r="G179" t="inlineStr"/>
-      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -9004,9 +8896,6 @@
           <t>New 4 filed 2026-05-19 (accession 0001651687-26-000009)</t>
         </is>
       </c>
-      <c r="F180" t="inlineStr"/>
-      <c r="G180" t="inlineStr"/>
-      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -9034,9 +8923,6 @@
           <t>New 4 filed 2026-05-19 (accession 0002022050-26-000007)</t>
         </is>
       </c>
-      <c r="F181" t="inlineStr"/>
-      <c r="G181" t="inlineStr"/>
-      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -9064,9 +8950,6 @@
           <t>New 4 filed 2026-05-19 (accession 0001990106-26-000014)</t>
         </is>
       </c>
-      <c r="F182" t="inlineStr"/>
-      <c r="G182" t="inlineStr"/>
-      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -9094,9 +8977,6 @@
           <t>New 4 filed 2026-05-19 (accession 0002082930-26-000008)</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr"/>
-      <c r="G183" t="inlineStr"/>
-      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -9124,9 +9004,1236 @@
           <t>New 144 filed 2026-05-18 (accession 0001921094-26-000512)</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr"/>
-      <c r="G184" t="inlineStr"/>
-      <c r="H184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/legal/terms</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="inlineStr"/>
+      <c r="H185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/investors/board-of-directors</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr"/>
+      <c r="H186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr"/>
+      <c r="G187" t="inlineStr"/>
+      <c r="H187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>https://news.shopify.com</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr"/>
+      <c r="H188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>https://investors.shopify.com</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr"/>
+      <c r="G189" t="inlineStr"/>
+      <c r="H189" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000022/shop-20260508.htm</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>New 8-K filed 2026-05-08 (accession 0001594805-26-000022)</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000195004726004066/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-05 (accession 0001950047-26-004066)</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000020/forms-8postxeffectiveamend.htm</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>New S-8 POS filed 2026-05-05 (accession 0001594805-26-000020)</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000019/shop-20260331.htm</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>New 10-Q filed 2026-05-05 (accession 0001594805-26-000019)</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr"/>
+      <c r="H193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1594805/000159480526000018/shop-20260505.htm</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>New 8-K filed 2026-05-05 (accession 0001594805-26-000018)</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr"/>
+      <c r="G194" t="inlineStr"/>
+      <c r="H194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home/post/wix-reports-first-quarter-2026-results</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>newsroom: Wix Reports First Quarter 2026 Results</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr"/>
+      <c r="G195" t="inlineStr"/>
+      <c r="H195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home/post/wix-to-participate-in-fireside-chat-at-the-2026-jefferies-software-internet-and-ai-conference</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>newsroom: Wix to Participate in Fireside Chat at the 2026 Jefferies Software, Internet, and AI Conference</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr"/>
+      <c r="G196" t="inlineStr"/>
+      <c r="H196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home/post/wix-to-announce-first-quarter-2026-results-on-may-13-2026</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>newsroom: Wix to Announce First Quarter 2026 Results on May 13, 2026</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr"/>
+      <c r="G197" t="inlineStr"/>
+      <c r="H197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home/post/wix-launches-hipaa-compliance-solution-expanding-support-for-health-service-providers-in-the-u-s</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>newsroom: Wix Launches HIPAA Compliance Solution Expanding Support for Health Service Providers in the U.S.</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr"/>
+      <c r="G198" t="inlineStr"/>
+      <c r="H198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home/post/wix-announces-final-results-of-modified-dutch-auction-tender-offer</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>newsroom: Wix Announces Final Results of Modified Dutch Auction Tender Offer</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr"/>
+      <c r="G199" t="inlineStr"/>
+      <c r="H199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>https://support.wix.com/en/article/terms-of-use</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="inlineStr"/>
+      <c r="H200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>https://investors.wix.com/board-of-directors</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr"/>
+      <c r="G201" t="inlineStr"/>
+      <c r="H201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/upgrade/website</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr"/>
+      <c r="G202" t="inlineStr"/>
+      <c r="H202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>https://investors.wix.com</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr"/>
+      <c r="G203" t="inlineStr"/>
+      <c r="H203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000119312526225926/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>New SCHEDULE 13G/A filed 2026-05-15 (accession 0001193125-26-225926)</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr"/>
+      <c r="G204" t="inlineStr"/>
+      <c r="H204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000090266426002441/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>New SCHEDULE 13G/A filed 2026-05-14 (accession 0000902664-26-002441)</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr"/>
+      <c r="G205" t="inlineStr"/>
+      <c r="H205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000117266126001868/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>New SCHEDULE 13G filed 2026-05-14 (accession 0001172661-26-001868)</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr"/>
+      <c r="G206" t="inlineStr"/>
+      <c r="H206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000117891326002642/zk2635313.htm</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002642)</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr"/>
+      <c r="G207" t="inlineStr"/>
+      <c r="H207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576789/000117891326002640/zk2635312.htm</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002640)</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr"/>
+      <c r="G208" t="inlineStr"/>
+      <c r="H208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>https://help.doordash.com/consumers/s/terms-of-service</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr"/>
+      <c r="G209" t="inlineStr"/>
+      <c r="H209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com/governance/management/default.aspx</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr"/>
+      <c r="G210" t="inlineStr"/>
+      <c r="H210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>https://about.doordash.com/en-us/news</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr"/>
+      <c r="G211" t="inlineStr"/>
+      <c r="H211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr"/>
+      <c r="G212" t="inlineStr"/>
+      <c r="H212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726005086/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-26 (accession 0001950047-26-005086)</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr"/>
+      <c r="G213" t="inlineStr"/>
+      <c r="H213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726005081/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-26 (accession 0001950047-26-005081)</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr"/>
+      <c r="G214" t="inlineStr"/>
+      <c r="H214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726004985/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-22 (accession 0001950047-26-004985)</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr"/>
+      <c r="G215" t="inlineStr"/>
+      <c r="H215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726004984/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-22 (accession 0001950047-26-004984)</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr"/>
+      <c r="G216" t="inlineStr"/>
+      <c r="H216" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183239026000011/xslF345X06/form4-05222026_040501.xml</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-22 (accession 0001832390-26-000011)</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr"/>
+      <c r="G217" t="inlineStr"/>
+      <c r="H217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/terms</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr"/>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/instacart-plus</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr"/>
+      <c r="G219" t="inlineStr"/>
+      <c r="H219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/company/newsroom</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr"/>
+      <c r="G220" t="inlineStr"/>
+      <c r="H220" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000165168726000009/xslF345X06/wk-form4_1779221300.xml</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0001651687-26-000009)</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr"/>
+      <c r="G221" t="inlineStr"/>
+      <c r="H221" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000202205026000007/xslF345X06/wk-form4_1779221163.xml</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0002022050-26-000007)</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr"/>
+      <c r="G222" t="inlineStr"/>
+      <c r="H222" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000199010626000014/xslF345X06/wk-form4_1779221074.xml</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0001990106-26-000014)</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr"/>
+      <c r="G223" t="inlineStr"/>
+      <c r="H223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000208293026000008/xslF345X06/wk-form4_1779220992.xml</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-19 (accession 0002082930-26-000008)</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr"/>
+      <c r="G224" t="inlineStr"/>
+      <c r="H224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000192109426000512/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-18 (accession 0001921094-26-000512)</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr"/>
+      <c r="G225" t="inlineStr"/>
+      <c r="H225" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-05-27T14:05Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4079,7 +4079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H225"/>
+  <dimension ref="A1:H236"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -9031,9 +9031,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr"/>
-      <c r="G185" t="inlineStr"/>
-      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -9061,9 +9058,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr"/>
-      <c r="G186" t="inlineStr"/>
-      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -9091,9 +9085,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr"/>
-      <c r="G187" t="inlineStr"/>
-      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -9121,9 +9112,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F188" t="inlineStr"/>
-      <c r="G188" t="inlineStr"/>
-      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -9151,9 +9139,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F189" t="inlineStr"/>
-      <c r="G189" t="inlineStr"/>
-      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -9181,9 +9166,6 @@
           <t>New 8-K filed 2026-05-08 (accession 0001594805-26-000022)</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr"/>
-      <c r="G190" t="inlineStr"/>
-      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -9211,9 +9193,6 @@
           <t>New 144 filed 2026-05-05 (accession 0001950047-26-004066)</t>
         </is>
       </c>
-      <c r="F191" t="inlineStr"/>
-      <c r="G191" t="inlineStr"/>
-      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -9241,9 +9220,6 @@
           <t>New S-8 POS filed 2026-05-05 (accession 0001594805-26-000020)</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr"/>
-      <c r="G192" t="inlineStr"/>
-      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -9271,9 +9247,6 @@
           <t>New 10-Q filed 2026-05-05 (accession 0001594805-26-000019)</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr"/>
-      <c r="G193" t="inlineStr"/>
-      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -9301,9 +9274,6 @@
           <t>New 8-K filed 2026-05-05 (accession 0001594805-26-000018)</t>
         </is>
       </c>
-      <c r="F194" t="inlineStr"/>
-      <c r="G194" t="inlineStr"/>
-      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -9331,9 +9301,6 @@
           <t>newsroom: Wix Reports First Quarter 2026 Results</t>
         </is>
       </c>
-      <c r="F195" t="inlineStr"/>
-      <c r="G195" t="inlineStr"/>
-      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -9361,9 +9328,6 @@
           <t>newsroom: Wix to Participate in Fireside Chat at the 2026 Jefferies Software, Internet, and AI Conference</t>
         </is>
       </c>
-      <c r="F196" t="inlineStr"/>
-      <c r="G196" t="inlineStr"/>
-      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -9391,9 +9355,6 @@
           <t>newsroom: Wix to Announce First Quarter 2026 Results on May 13, 2026</t>
         </is>
       </c>
-      <c r="F197" t="inlineStr"/>
-      <c r="G197" t="inlineStr"/>
-      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -9421,9 +9382,6 @@
           <t>newsroom: Wix Launches HIPAA Compliance Solution Expanding Support for Health Service Providers in the U.S.</t>
         </is>
       </c>
-      <c r="F198" t="inlineStr"/>
-      <c r="G198" t="inlineStr"/>
-      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -9451,9 +9409,6 @@
           <t>newsroom: Wix Announces Final Results of Modified Dutch Auction Tender Offer</t>
         </is>
       </c>
-      <c r="F199" t="inlineStr"/>
-      <c r="G199" t="inlineStr"/>
-      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -9481,9 +9436,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F200" t="inlineStr"/>
-      <c r="G200" t="inlineStr"/>
-      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -9511,9 +9463,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr"/>
-      <c r="G201" t="inlineStr"/>
-      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -9541,9 +9490,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F202" t="inlineStr"/>
-      <c r="G202" t="inlineStr"/>
-      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -9571,9 +9517,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F203" t="inlineStr"/>
-      <c r="G203" t="inlineStr"/>
-      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -9601,9 +9544,6 @@
           <t>New SCHEDULE 13G/A filed 2026-05-15 (accession 0001193125-26-225926)</t>
         </is>
       </c>
-      <c r="F204" t="inlineStr"/>
-      <c r="G204" t="inlineStr"/>
-      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -9631,9 +9571,6 @@
           <t>New SCHEDULE 13G/A filed 2026-05-14 (accession 0000902664-26-002441)</t>
         </is>
       </c>
-      <c r="F205" t="inlineStr"/>
-      <c r="G205" t="inlineStr"/>
-      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -9661,9 +9598,6 @@
           <t>New SCHEDULE 13G filed 2026-05-14 (accession 0001172661-26-001868)</t>
         </is>
       </c>
-      <c r="F206" t="inlineStr"/>
-      <c r="G206" t="inlineStr"/>
-      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -9691,9 +9625,6 @@
           <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002642)</t>
         </is>
       </c>
-      <c r="F207" t="inlineStr"/>
-      <c r="G207" t="inlineStr"/>
-      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -9721,9 +9652,6 @@
           <t>New S-8 filed 2026-05-13 (accession 0001178913-26-002640)</t>
         </is>
       </c>
-      <c r="F208" t="inlineStr"/>
-      <c r="G208" t="inlineStr"/>
-      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -9751,9 +9679,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F209" t="inlineStr"/>
-      <c r="G209" t="inlineStr"/>
-      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -9781,9 +9706,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F210" t="inlineStr"/>
-      <c r="G210" t="inlineStr"/>
-      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -9811,9 +9733,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F211" t="inlineStr"/>
-      <c r="G211" t="inlineStr"/>
-      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -9841,9 +9760,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F212" t="inlineStr"/>
-      <c r="G212" t="inlineStr"/>
-      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -9871,9 +9787,6 @@
           <t>New 144 filed 2026-05-26 (accession 0001950047-26-005086)</t>
         </is>
       </c>
-      <c r="F213" t="inlineStr"/>
-      <c r="G213" t="inlineStr"/>
-      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -9901,9 +9814,6 @@
           <t>New 144 filed 2026-05-26 (accession 0001950047-26-005081)</t>
         </is>
       </c>
-      <c r="F214" t="inlineStr"/>
-      <c r="G214" t="inlineStr"/>
-      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -9931,9 +9841,6 @@
           <t>New 144 filed 2026-05-22 (accession 0001950047-26-004985)</t>
         </is>
       </c>
-      <c r="F215" t="inlineStr"/>
-      <c r="G215" t="inlineStr"/>
-      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -9961,9 +9868,6 @@
           <t>New 144 filed 2026-05-22 (accession 0001950047-26-004984)</t>
         </is>
       </c>
-      <c r="F216" t="inlineStr"/>
-      <c r="G216" t="inlineStr"/>
-      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -9991,9 +9895,6 @@
           <t>New 4 filed 2026-05-22 (accession 0001832390-26-000011)</t>
         </is>
       </c>
-      <c r="F217" t="inlineStr"/>
-      <c r="G217" t="inlineStr"/>
-      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -10021,9 +9922,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F218" t="inlineStr"/>
-      <c r="G218" t="inlineStr"/>
-      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -10051,9 +9949,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F219" t="inlineStr"/>
-      <c r="G219" t="inlineStr"/>
-      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -10081,9 +9976,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F220" t="inlineStr"/>
-      <c r="G220" t="inlineStr"/>
-      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -10111,9 +10003,6 @@
           <t>New 4 filed 2026-05-19 (accession 0001651687-26-000009)</t>
         </is>
       </c>
-      <c r="F221" t="inlineStr"/>
-      <c r="G221" t="inlineStr"/>
-      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -10141,9 +10030,6 @@
           <t>New 4 filed 2026-05-19 (accession 0002022050-26-000007)</t>
         </is>
       </c>
-      <c r="F222" t="inlineStr"/>
-      <c r="G222" t="inlineStr"/>
-      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -10171,9 +10057,6 @@
           <t>New 4 filed 2026-05-19 (accession 0001990106-26-000014)</t>
         </is>
       </c>
-      <c r="F223" t="inlineStr"/>
-      <c r="G223" t="inlineStr"/>
-      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -10201,9 +10084,6 @@
           <t>New 4 filed 2026-05-19 (accession 0002082930-26-000008)</t>
         </is>
       </c>
-      <c r="F224" t="inlineStr"/>
-      <c r="G224" t="inlineStr"/>
-      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -10231,9 +10111,336 @@
           <t>New 144 filed 2026-05-18 (accession 0001921094-26-000512)</t>
         </is>
       </c>
-      <c r="F225" t="inlineStr"/>
-      <c r="G225" t="inlineStr"/>
-      <c r="H225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726005086/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-26 (accession 0001950047-26-005086)</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr"/>
+      <c r="G226" t="inlineStr"/>
+      <c r="H226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726005081/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-26 (accession 0001950047-26-005081)</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr"/>
+      <c r="G227" t="inlineStr"/>
+      <c r="H227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726004985/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-22 (accession 0001950047-26-004985)</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr"/>
+      <c r="G228" t="inlineStr"/>
+      <c r="H228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726004984/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>New 144 filed 2026-05-22 (accession 0001950047-26-004984)</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr"/>
+      <c r="G229" t="inlineStr"/>
+      <c r="H229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183239026000011/xslF345X06/form4-05222026_040501.xml</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-22 (accession 0001832390-26-000011)</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr"/>
+      <c r="G230" t="inlineStr"/>
+      <c r="H230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183261426000017/xslF345X06/form4-05222026_040512.xml</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-22 (accession 0001832614-26-000017)</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr"/>
+      <c r="G231" t="inlineStr"/>
+      <c r="H231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000189968826000010/xslF345X06/form4-05222026_040510.xml</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-22 (accession 0001899688-26-000010)</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr"/>
+      <c r="G232" t="inlineStr"/>
+      <c r="H232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000184970926000012/xslF345X06/form4-05222026_040508.xml</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-22 (accession 0001849709-26-000012)</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr"/>
+      <c r="G233" t="inlineStr"/>
+      <c r="H233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183261226000012/xslF345X06/form4-05222026_040507.xml</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-22 (accession 0001832612-26-000012)</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr"/>
+      <c r="G234" t="inlineStr"/>
+      <c r="H234" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183355226000008/xslF345X06/form4-05222026_040505.xml</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-22 (accession 0001833552-26-000008)</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr"/>
+      <c r="G235" t="inlineStr"/>
+      <c r="H235" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000163564826000008/xslF345X06/form4-05222026_040503.xml</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>New 4 filed 2026-05-22 (accession 0001635648-26-000008)</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr"/>
+      <c r="G236" t="inlineStr"/>
+      <c r="H236" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tier=high run 2026-05-27T14:39Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4079,7 +4079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H236"/>
+  <dimension ref="A1:H237"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10138,9 +10138,6 @@
           <t>New 144 filed 2026-05-26 (accession 0001950047-26-005086)</t>
         </is>
       </c>
-      <c r="F226" t="inlineStr"/>
-      <c r="G226" t="inlineStr"/>
-      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -10168,9 +10165,6 @@
           <t>New 144 filed 2026-05-26 (accession 0001950047-26-005081)</t>
         </is>
       </c>
-      <c r="F227" t="inlineStr"/>
-      <c r="G227" t="inlineStr"/>
-      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -10198,9 +10192,6 @@
           <t>New 144 filed 2026-05-22 (accession 0001950047-26-004985)</t>
         </is>
       </c>
-      <c r="F228" t="inlineStr"/>
-      <c r="G228" t="inlineStr"/>
-      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -10228,9 +10219,6 @@
           <t>New 144 filed 2026-05-22 (accession 0001950047-26-004984)</t>
         </is>
       </c>
-      <c r="F229" t="inlineStr"/>
-      <c r="G229" t="inlineStr"/>
-      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -10258,9 +10246,6 @@
           <t>New 4 filed 2026-05-22 (accession 0001832390-26-000011)</t>
         </is>
       </c>
-      <c r="F230" t="inlineStr"/>
-      <c r="G230" t="inlineStr"/>
-      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -10288,9 +10273,6 @@
           <t>New 4 filed 2026-05-22 (accession 0001832614-26-000017)</t>
         </is>
       </c>
-      <c r="F231" t="inlineStr"/>
-      <c r="G231" t="inlineStr"/>
-      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -10318,9 +10300,6 @@
           <t>New 4 filed 2026-05-22 (accession 0001899688-26-000010)</t>
         </is>
       </c>
-      <c r="F232" t="inlineStr"/>
-      <c r="G232" t="inlineStr"/>
-      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -10348,9 +10327,6 @@
           <t>New 4 filed 2026-05-22 (accession 0001849709-26-000012)</t>
         </is>
       </c>
-      <c r="F233" t="inlineStr"/>
-      <c r="G233" t="inlineStr"/>
-      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -10378,9 +10354,6 @@
           <t>New 4 filed 2026-05-22 (accession 0001832612-26-000012)</t>
         </is>
       </c>
-      <c r="F234" t="inlineStr"/>
-      <c r="G234" t="inlineStr"/>
-      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -10408,9 +10381,6 @@
           <t>New 4 filed 2026-05-22 (accession 0001833552-26-000008)</t>
         </is>
       </c>
-      <c r="F235" t="inlineStr"/>
-      <c r="G235" t="inlineStr"/>
-      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -10438,9 +10408,36 @@
           <t>New 4 filed 2026-05-22 (accession 0001635648-26-000008)</t>
         </is>
       </c>
-      <c r="F236" t="inlineStr"/>
-      <c r="G236" t="inlineStr"/>
-      <c r="H236" t="inlineStr"/>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr"/>
+      <c r="G237" t="inlineStr"/>
+      <c r="H237" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-05-27T15:05Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4079,7 +4079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H237"/>
+  <dimension ref="A1:H249"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10435,9 +10435,366 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F237" t="inlineStr"/>
-      <c r="G237" t="inlineStr"/>
-      <c r="H237" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726005086/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Yandell Keith (Officer) plans to sell 2,643 shares (~$423.5K) on/after 05/26/2026</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr"/>
+      <c r="G238" t="inlineStr"/>
+      <c r="H238" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726005081/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Adarkar Prabir (Officer) plans to sell 11,739 shares (~$1.88M) on/after 05/26/2026</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr"/>
+      <c r="G239" t="inlineStr"/>
+      <c r="H239" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726004985/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Sherringham Tia (Officer) plans to sell 2,743 shares (~$436.9K) on/after 05/22/2026</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr"/>
+      <c r="G240" t="inlineStr"/>
+      <c r="H240" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726004984/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Lee Gordon (Officer) plans to sell 2,204 shares (~$351.0K) on/after 05/22/2026</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr"/>
+      <c r="G241" t="inlineStr"/>
+      <c r="H241" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183239026000011/xslF345X06/form4-05222026_040501.xml</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Fang Andy (Director) sold 1,164 shares @ $155.59 ($181.1K) on 2026-05-20</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr"/>
+      <c r="G242" t="inlineStr"/>
+      <c r="H242" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183261426000017/xslF345X06/form4-05222026_040512.xml</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Tang Stanley (Director) sold 1,592 shares @ $155.59 ($247.7K) on 2026-05-20</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr"/>
+      <c r="G243" t="inlineStr"/>
+      <c r="H243" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000189968826000010/xslF345X06/form4-05222026_040510.xml</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Sherringham Tia (GENERAL COUNSEL AND SECRETARY) sold 7,690 shares @ $155.59 ($1.20M) on 2026-05-20</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr"/>
+      <c r="G244" t="inlineStr"/>
+      <c r="H244" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000184970926000012/xslF345X06/form4-05222026_040508.xml</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Inukonda Ravi (CHIEF FINANCIAL OFFICER) sold 19,505 shares @ $155.59 ($3.03M) on 2026-05-20</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr"/>
+      <c r="G245" t="inlineStr"/>
+      <c r="H245" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183261226000012/xslF345X06/form4-05222026_040507.xml</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Adarkar Prabir (PRESIDENT AND COO) sold 17,126 shares @ $155.59 ($2.66M) on 2026-05-20</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr"/>
+      <c r="G246" t="inlineStr"/>
+      <c r="H246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183355226000008/xslF345X06/form4-05222026_040505.xml</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Yandell Keith (CHIEF BUSINESS OFFICER) sold 4,227 shares @ $155.59 ($657.7K) on 2026-05-20</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr"/>
+      <c r="G247" t="inlineStr"/>
+      <c r="H247" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000163564826000008/xslF345X06/form4-05222026_040503.xml</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Lee Gordon S (CHIEF ACCOUNTING OFFICER) sold 2,910 shares @ $155.59 ($452.8K) on 2026-05-20</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr"/>
+      <c r="G248" t="inlineStr"/>
+      <c r="H248" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/instacart-plus</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr"/>
+      <c r="G249" t="inlineStr"/>
+      <c r="H249" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-05-27T15:52Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H249"/>
+  <dimension ref="A1:H252"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10779,6 +10779,96 @@
           <t>pricing: change detected</t>
         </is>
       </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr"/>
+      <c r="G250" t="inlineStr"/>
+      <c r="H250" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/upgrade/website</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr"/>
+      <c r="G251" t="inlineStr"/>
+      <c r="H251" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/instacart-plus</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr"/>
+      <c r="G252" t="inlineStr"/>
+      <c r="H252" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-05-27T16:00Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H252"/>
+  <dimension ref="A1:H253"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10806,9 +10806,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F250" t="inlineStr"/>
-      <c r="G250" t="inlineStr"/>
-      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -10836,9 +10833,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F251" t="inlineStr"/>
-      <c r="G251" t="inlineStr"/>
-      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -10866,9 +10860,36 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F252" t="inlineStr"/>
-      <c r="G252" t="inlineStr"/>
-      <c r="H252" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>https://investors.wix.com</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr"/>
+      <c r="G253" t="inlineStr"/>
+      <c r="H253" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-05-27T17:21Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H253"/>
+  <dimension ref="A1:H254"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10887,9 +10887,36 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F253" t="inlineStr"/>
-      <c r="G253" t="inlineStr"/>
-      <c r="H253" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>https://about.doordash.com/en-us/news</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr"/>
+      <c r="G254" t="inlineStr"/>
+      <c r="H254" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tier=high run 2026-05-27T18:13Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H254"/>
+  <dimension ref="A1:H255"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10914,9 +10914,36 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F254" t="inlineStr"/>
-      <c r="G254" t="inlineStr"/>
-      <c r="H254" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>ETSY</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Etsy Inc.</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>https://investors.etsy.com</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr"/>
+      <c r="G255" t="inlineStr"/>
+      <c r="H255" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tier=high run 2026-05-27T21:12Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H255"/>
+  <dimension ref="A1:H257"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10941,9 +10941,66 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F255" t="inlineStr"/>
-      <c r="G255" t="inlineStr"/>
-      <c r="H255" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>CHWY</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Chewy Inc.</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>https://investor.chewy.com</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr"/>
+      <c r="G256" t="inlineStr"/>
+      <c r="H256" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>https://cdn.robinhood.com/assets/robinhood/legal/Robinhood-Customer-Agreement.pdf</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr"/>
+      <c r="G257" t="inlineStr"/>
+      <c r="H257" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tier=high run 2026-05-27T22:56Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H257"/>
+  <dimension ref="A1:H258"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10968,9 +10968,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F256" t="inlineStr"/>
-      <c r="G256" t="inlineStr"/>
-      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -10998,9 +10995,36 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F257" t="inlineStr"/>
-      <c r="G257" t="inlineStr"/>
-      <c r="H257" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1783879/000110465926067045/xslF345X06/tm2615788-1_4seq1.xml</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr"/>
+      <c r="G258" t="inlineStr"/>
+      <c r="H258" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tier=high run 2026-05-28T00:13Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H258"/>
+  <dimension ref="A1:H260"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11022,9 +11022,66 @@
           <t>[ROUTINE] Insider trade</t>
         </is>
       </c>
-      <c r="F258" t="inlineStr"/>
-      <c r="G258" t="inlineStr"/>
-      <c r="H258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr"/>
+      <c r="G259" t="inlineStr"/>
+      <c r="H259" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>https://robinhood.com/us/en/support/articles/trading-fees-on-robinhood/</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr"/>
+      <c r="G260" t="inlineStr"/>
+      <c r="H260" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-05-28T13:33Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H260"/>
+  <dimension ref="A1:H272"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11049,9 +11049,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F259" t="inlineStr"/>
-      <c r="G259" t="inlineStr"/>
-      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -11079,9 +11076,366 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F260" t="inlineStr"/>
-      <c r="G260" t="inlineStr"/>
-      <c r="H260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr"/>
+      <c r="G261" t="inlineStr"/>
+      <c r="H261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>https://about.doordash.com/en-us/news</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr"/>
+      <c r="G262" t="inlineStr"/>
+      <c r="H262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000189968826000012/xslF345X06/form4-05272026_040509.xml</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Sherringham Tia (GENERAL COUNSEL AND SECRETARY) sold 2,743 shares @ $160.79 ($441.0K) on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr"/>
+      <c r="G263" t="inlineStr"/>
+      <c r="H263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000163564826000010/xslF345X06/form4-05272026_040507.xml</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Lee Gordon S (CHIEF ACCOUNTING OFFICER) sold 2,204 shares @ $160.79 ($354.4K) on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr"/>
+      <c r="G264" t="inlineStr"/>
+      <c r="H264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/instacart-plus</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr"/>
+      <c r="G265" t="inlineStr"/>
+      <c r="H265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000091957426003716/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Sundheim Daniel S. (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr"/>
+      <c r="G266" t="inlineStr"/>
+      <c r="H266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000198846026000002/xslF345X06/form4.xml</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Gupta Ravi (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr"/>
+      <c r="G267" t="inlineStr"/>
+      <c r="H267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000164007526000011/xslF345X06/wk-form4_1779913021.xml</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Levien Meredith A. Kopit (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr"/>
+      <c r="G268" t="inlineStr"/>
+      <c r="H268" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000173634126000005/xslF345X06/wk-form4_1779912973.xml</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Sarafan Lily (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr"/>
+      <c r="G269" t="inlineStr"/>
+      <c r="H269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000151113426000002/xslF345X06/wk-form4_1779912918.xml</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Dolan Victoria L (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr"/>
+      <c r="G270" t="inlineStr"/>
+      <c r="H270" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000152535826000016/xslF345X06/wk-form4_1779912875.xml</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Silverman Josh (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr"/>
+      <c r="G271" t="inlineStr"/>
+      <c r="H271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000189467426000002/xslF345X06/wk-form4_1779912813.xml</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Laughton Mary Beth (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr"/>
+      <c r="G272" t="inlineStr"/>
+      <c r="H272" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-05-28T13:39Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H272"/>
+  <dimension ref="A1:H273"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11103,9 +11103,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F261" t="inlineStr"/>
-      <c r="G261" t="inlineStr"/>
-      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -11133,9 +11130,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F262" t="inlineStr"/>
-      <c r="G262" t="inlineStr"/>
-      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -11163,9 +11157,6 @@
           <t>[ROUTINE] Insider trade — Sherringham Tia (GENERAL COUNSEL AND SECRETARY) sold 2,743 shares @ $160.79 ($441.0K) on 2026-05-22</t>
         </is>
       </c>
-      <c r="F263" t="inlineStr"/>
-      <c r="G263" t="inlineStr"/>
-      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -11193,9 +11184,6 @@
           <t>[ROUTINE] Insider trade — Lee Gordon S (CHIEF ACCOUNTING OFFICER) sold 2,204 shares @ $160.79 ($354.4K) on 2026-05-22</t>
         </is>
       </c>
-      <c r="F264" t="inlineStr"/>
-      <c r="G264" t="inlineStr"/>
-      <c r="H264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -11223,9 +11211,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F265" t="inlineStr"/>
-      <c r="G265" t="inlineStr"/>
-      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -11253,9 +11238,6 @@
           <t>[ROUTINE] Insider trade — Sundheim Daniel S. (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
         </is>
       </c>
-      <c r="F266" t="inlineStr"/>
-      <c r="G266" t="inlineStr"/>
-      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -11283,9 +11265,6 @@
           <t>[ROUTINE] Insider trade — Gupta Ravi (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
         </is>
       </c>
-      <c r="F267" t="inlineStr"/>
-      <c r="G267" t="inlineStr"/>
-      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -11313,9 +11292,6 @@
           <t>[ROUTINE] Insider trade — Levien Meredith A. Kopit (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
         </is>
       </c>
-      <c r="F268" t="inlineStr"/>
-      <c r="G268" t="inlineStr"/>
-      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -11343,9 +11319,6 @@
           <t>[ROUTINE] Insider trade — Sarafan Lily (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
         </is>
       </c>
-      <c r="F269" t="inlineStr"/>
-      <c r="G269" t="inlineStr"/>
-      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -11373,9 +11346,6 @@
           <t>[ROUTINE] Insider trade — Dolan Victoria L (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
         </is>
       </c>
-      <c r="F270" t="inlineStr"/>
-      <c r="G270" t="inlineStr"/>
-      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -11403,9 +11373,6 @@
           <t>[ROUTINE] Insider trade — Silverman Josh (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
         </is>
       </c>
-      <c r="F271" t="inlineStr"/>
-      <c r="G271" t="inlineStr"/>
-      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -11433,9 +11400,36 @@
           <t>[ROUTINE] Insider trade — Laughton Mary Beth (Director) RSU/grant of 6,048 shares on 2026-05-22</t>
         </is>
       </c>
-      <c r="F272" t="inlineStr"/>
-      <c r="G272" t="inlineStr"/>
-      <c r="H272" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/instacart-plus</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr"/>
+      <c r="G273" t="inlineStr"/>
+      <c r="H273" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-06-01T13:16Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H273"/>
+  <dimension ref="A1:H276"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11427,9 +11427,96 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F273" t="inlineStr"/>
-      <c r="G273" t="inlineStr"/>
-      <c r="H273" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr"/>
+      <c r="G274" t="inlineStr"/>
+      <c r="H274" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>https://news.shopify.com</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr"/>
+      <c r="G275" t="inlineStr"/>
+      <c r="H275" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>https://about.doordash.com/en-us/news</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr"/>
+      <c r="G276" t="inlineStr"/>
+      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-06-01T13:27Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H276"/>
+  <dimension ref="A1:H278"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11454,9 +11454,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F274" t="inlineStr"/>
-      <c r="G274" t="inlineStr"/>
-      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -11484,9 +11481,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F275" t="inlineStr"/>
-      <c r="G275" t="inlineStr"/>
-      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -11514,9 +11508,66 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F276" t="inlineStr"/>
-      <c r="G276" t="inlineStr"/>
-      <c r="H276" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>https://investors.wix.com/board-of-directors</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr"/>
+      <c r="G277" t="inlineStr"/>
+      <c r="H277" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/terms</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr"/>
+      <c r="G278" t="inlineStr"/>
+      <c r="H278" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-06-01T13:32Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H278"/>
+  <dimension ref="A1:H279"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11535,9 +11535,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F277" t="inlineStr"/>
-      <c r="G277" t="inlineStr"/>
-      <c r="H277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -11565,9 +11562,36 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F278" t="inlineStr"/>
-      <c r="G278" t="inlineStr"/>
-      <c r="H278" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/instacart-plus</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr"/>
+      <c r="G279" t="inlineStr"/>
+      <c r="H279" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-06-01T14:12Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H279"/>
+  <dimension ref="A1:H300"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11589,9 +11589,636 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F279" t="inlineStr"/>
-      <c r="G279" t="inlineStr"/>
-      <c r="H279" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/shopify/comments/1ttn8xs/custom_feature_for_shopify_quick_question/</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>reddit: Custom feature for Shopify.. quick question</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr"/>
+      <c r="G280" t="inlineStr"/>
+      <c r="H280" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/shopify/comments/1ttmcp1/ai_referrals_may_turn_product_pages_into_the_new/</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>reddit: AI referrals may turn product pages into the new homepage.</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr"/>
+      <c r="G281" t="inlineStr"/>
+      <c r="H281" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/shopify/comments/1ttlejz/how_to_add_card_processing_fees_in_checkout_uk/</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>reddit: How to add card processing fees in checkout - UK store</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr"/>
+      <c r="G282" t="inlineStr"/>
+      <c r="H282" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/shopify/comments/1ttoli5/currency_display_issue/</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>reddit: Currency Display Issue</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr"/>
+      <c r="G283" t="inlineStr"/>
+      <c r="H283" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/shopify/comments/1ttokfy/how_do_i_create_a_collapsible_row_with_both/</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>reddit: How do i create a collapsible row with both images and table and text?</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr"/>
+      <c r="G284" t="inlineStr"/>
+      <c r="H284" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/WIX/comments/1ttm2wp/server_not_found_error_when_trying_to_embed_a_map/</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>reddit: Server Not Found error when trying to embed a map from google - help?</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr"/>
+      <c r="G285" t="inlineStr"/>
+      <c r="H285" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/WIX/comments/1ttkdf3/what_the_layoff_round_at_wix_might_tell_us_about/</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>reddit: What the layoff round at Wix might tell us about the future of Israel (and its tech industry)</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr"/>
+      <c r="G286" t="inlineStr"/>
+      <c r="H286" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/WIX/comments/1ttcvhf/all_elements_on_wix_website_have_enlarged_help/</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>reddit: ALL ELEMENTS ON WIX WEBSITE HAVE ENLARGED!!! HELP PLEASE</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr"/>
+      <c r="G287" t="inlineStr"/>
+      <c r="H287" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/WIX/comments/1tsp1ms/help_me_i_am_so_pissed/</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>reddit: HELP ME I AM SO PISSED</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr"/>
+      <c r="G288" t="inlineStr"/>
+      <c r="H288" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/WIX/comments/1tsgmjv/transferring_from_wix_classic_to_wix_studio_can/</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>reddit: Transferring from Wix Classic to Wix Studio - Can this hurt SEO?</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr"/>
+      <c r="G289" t="inlineStr"/>
+      <c r="H289" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/doordash/comments/1ttdxn4/by_far_the_worst_order_ive_done/</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>reddit: By far the worst order I’ve done</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr"/>
+      <c r="G290" t="inlineStr"/>
+      <c r="H290" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/doordash/comments/1ttdxhy/last_time_i_dont_check_items_for_grocery/</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>reddit: Last time I don’t check items for grocery.</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr"/>
+      <c r="G291" t="inlineStr"/>
+      <c r="H291" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/doordash/comments/1ttiqhx/dasher_fent_folded_in_front_of_me/</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>reddit: dasher fent folded in front of me</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr"/>
+      <c r="G292" t="inlineStr"/>
+      <c r="H292" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/doordash/comments/1ttjalz/doordash_has_ruined_take_out/</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>reddit: Doordash has ruined Take Out.</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr"/>
+      <c r="G293" t="inlineStr"/>
+      <c r="H293" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/doordash/comments/1ttjj3c/what_does_this_mean_if_anything/</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>reddit: what does this mean, if anything?</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr"/>
+      <c r="G294" t="inlineStr"/>
+      <c r="H294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/InstacartShoppers/comments/1ttkzlb/this_is_new_maybe_everyone_will_get_it/</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>reddit: This is new maybe everyone will get it.</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr"/>
+      <c r="G295" t="inlineStr"/>
+      <c r="H295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/InstacartShoppers/comments/1ttkahc/not_sure_if_i_can_call_it_a_unicorn_but_this_is/</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>reddit: Not sure if I can call it a unicorn but this is the biggest tip that I ever got.</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr"/>
+      <c r="G296" t="inlineStr"/>
+      <c r="H296" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/InstacartShoppers/comments/1tt2aza/new_method_after_7_years/</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>reddit: New method after 7 years</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr"/>
+      <c r="G297" t="inlineStr"/>
+      <c r="H297" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/InstacartShoppers/comments/1tt6f3z/if_you_lost_your_card_in_ga_dm_me/</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>reddit: If you lost your card in GA dm me.</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr"/>
+      <c r="G298" t="inlineStr"/>
+      <c r="H298" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/InstacartShoppers/comments/1tt7h64/customers_asking_to_enter_home_in_delivery_note/</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>reddit: Customers asking to enter home in delivery note</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr"/>
+      <c r="G299" t="inlineStr"/>
+      <c r="H299" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/instacart-plus</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr"/>
+      <c r="G300" t="inlineStr"/>
+      <c r="H300" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-06-01T16:13Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H300"/>
+  <dimension ref="A1:H310"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11616,9 +11616,6 @@
           <t>reddit: Custom feature for Shopify.. quick question</t>
         </is>
       </c>
-      <c r="F280" t="inlineStr"/>
-      <c r="G280" t="inlineStr"/>
-      <c r="H280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -11646,9 +11643,6 @@
           <t>reddit: AI referrals may turn product pages into the new homepage.</t>
         </is>
       </c>
-      <c r="F281" t="inlineStr"/>
-      <c r="G281" t="inlineStr"/>
-      <c r="H281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -11676,9 +11670,6 @@
           <t>reddit: How to add card processing fees in checkout - UK store</t>
         </is>
       </c>
-      <c r="F282" t="inlineStr"/>
-      <c r="G282" t="inlineStr"/>
-      <c r="H282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -11706,9 +11697,6 @@
           <t>reddit: Currency Display Issue</t>
         </is>
       </c>
-      <c r="F283" t="inlineStr"/>
-      <c r="G283" t="inlineStr"/>
-      <c r="H283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -11736,9 +11724,6 @@
           <t>reddit: How do i create a collapsible row with both images and table and text?</t>
         </is>
       </c>
-      <c r="F284" t="inlineStr"/>
-      <c r="G284" t="inlineStr"/>
-      <c r="H284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -11766,9 +11751,6 @@
           <t>reddit: Server Not Found error when trying to embed a map from google - help?</t>
         </is>
       </c>
-      <c r="F285" t="inlineStr"/>
-      <c r="G285" t="inlineStr"/>
-      <c r="H285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -11796,9 +11778,6 @@
           <t>reddit: What the layoff round at Wix might tell us about the future of Israel (and its tech industry)</t>
         </is>
       </c>
-      <c r="F286" t="inlineStr"/>
-      <c r="G286" t="inlineStr"/>
-      <c r="H286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -11826,9 +11805,6 @@
           <t>reddit: ALL ELEMENTS ON WIX WEBSITE HAVE ENLARGED!!! HELP PLEASE</t>
         </is>
       </c>
-      <c r="F287" t="inlineStr"/>
-      <c r="G287" t="inlineStr"/>
-      <c r="H287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -11856,9 +11832,6 @@
           <t>reddit: HELP ME I AM SO PISSED</t>
         </is>
       </c>
-      <c r="F288" t="inlineStr"/>
-      <c r="G288" t="inlineStr"/>
-      <c r="H288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -11886,9 +11859,6 @@
           <t>reddit: Transferring from Wix Classic to Wix Studio - Can this hurt SEO?</t>
         </is>
       </c>
-      <c r="F289" t="inlineStr"/>
-      <c r="G289" t="inlineStr"/>
-      <c r="H289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -11916,9 +11886,6 @@
           <t>reddit: By far the worst order I’ve done</t>
         </is>
       </c>
-      <c r="F290" t="inlineStr"/>
-      <c r="G290" t="inlineStr"/>
-      <c r="H290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -11946,9 +11913,6 @@
           <t>reddit: Last time I don’t check items for grocery.</t>
         </is>
       </c>
-      <c r="F291" t="inlineStr"/>
-      <c r="G291" t="inlineStr"/>
-      <c r="H291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -11976,9 +11940,6 @@
           <t>reddit: dasher fent folded in front of me</t>
         </is>
       </c>
-      <c r="F292" t="inlineStr"/>
-      <c r="G292" t="inlineStr"/>
-      <c r="H292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -12006,9 +11967,6 @@
           <t>reddit: Doordash has ruined Take Out.</t>
         </is>
       </c>
-      <c r="F293" t="inlineStr"/>
-      <c r="G293" t="inlineStr"/>
-      <c r="H293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -12036,9 +11994,6 @@
           <t>reddit: what does this mean, if anything?</t>
         </is>
       </c>
-      <c r="F294" t="inlineStr"/>
-      <c r="G294" t="inlineStr"/>
-      <c r="H294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -12066,9 +12021,6 @@
           <t>reddit: This is new maybe everyone will get it.</t>
         </is>
       </c>
-      <c r="F295" t="inlineStr"/>
-      <c r="G295" t="inlineStr"/>
-      <c r="H295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -12096,9 +12048,6 @@
           <t>reddit: Not sure if I can call it a unicorn but this is the biggest tip that I ever got.</t>
         </is>
       </c>
-      <c r="F296" t="inlineStr"/>
-      <c r="G296" t="inlineStr"/>
-      <c r="H296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -12126,9 +12075,6 @@
           <t>reddit: New method after 7 years</t>
         </is>
       </c>
-      <c r="F297" t="inlineStr"/>
-      <c r="G297" t="inlineStr"/>
-      <c r="H297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -12156,9 +12102,6 @@
           <t>reddit: If you lost your card in GA dm me.</t>
         </is>
       </c>
-      <c r="F298" t="inlineStr"/>
-      <c r="G298" t="inlineStr"/>
-      <c r="H298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -12186,9 +12129,6 @@
           <t>reddit: Customers asking to enter home in delivery note</t>
         </is>
       </c>
-      <c r="F299" t="inlineStr"/>
-      <c r="G299" t="inlineStr"/>
-      <c r="H299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -12216,9 +12156,306 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F300" t="inlineStr"/>
-      <c r="G300" t="inlineStr"/>
-      <c r="H300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/shopify/comments/1tttupa/customer_waits_15_months_to_reach_out_about_an/</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>reddit: Customer waits 15 MONTHS to reach out about an order they never received; wwyd?</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr"/>
+      <c r="G301" t="inlineStr"/>
+      <c r="H301" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/shopify/comments/1ttw705/your_shopify_speed_score_isnt_your_themes_fault/</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>reddit: Your Shopify speed score isn't your theme's fault (usually). Here's what actually kills it.</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr"/>
+      <c r="G302" t="inlineStr"/>
+      <c r="H302" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/WIX/comments/1ttunyg/how_to_align_heights_for_each_card_in_repeaters/</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>reddit: How to align heights for each card in repeaters</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr"/>
+      <c r="G303" t="inlineStr"/>
+      <c r="H303" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/doordash/comments/1tttduq/can_you_make_this_weekly_dd/</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>reddit: Can you make this weekly DD</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr"/>
+      <c r="G304" t="inlineStr"/>
+      <c r="H304" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/doordash/comments/1ttuq9r/do_you_take_this_i_wanna_know/</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>reddit: Do you TAKE THIS??? 😮‍💨😩 i wanna know</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr"/>
+      <c r="G305" t="inlineStr"/>
+      <c r="H305" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/InstacartShoppers/comments/1ttvyy4/going_online_after_3_years_hiatus/</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>reddit: Going online after 3 years hiatus</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr"/>
+      <c r="G306" t="inlineStr"/>
+      <c r="H306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/InstacartShoppers/comments/1ttvoln/taxes_for_instacart/</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>reddit: taxes for instacart</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr"/>
+      <c r="G307" t="inlineStr"/>
+      <c r="H307" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/InstacartShoppers/comments/1ttw7h1/i_wish_instacart_would_add_this/</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>reddit: I wish Instacart would add this!</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr"/>
+      <c r="G308" t="inlineStr"/>
+      <c r="H308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/InstacartShoppers/comments/1ttw2sp/how_do_yall_make_so_much_money_in_a_week/</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>reddit: how do y'all make so much money in a week??</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr"/>
+      <c r="G309" t="inlineStr"/>
+      <c r="H309" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/InstacartShoppers/comments/1ttw27w/better_to_wait_or_move_stores/</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>reddit: Better to wait or move stores?</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr"/>
+      <c r="G310" t="inlineStr"/>
+      <c r="H310" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-06-01T17:09Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H310"/>
+  <dimension ref="A1:H312"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -12183,9 +12183,6 @@
           <t>reddit: Customer waits 15 MONTHS to reach out about an order they never received; wwyd?</t>
         </is>
       </c>
-      <c r="F301" t="inlineStr"/>
-      <c r="G301" t="inlineStr"/>
-      <c r="H301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -12213,9 +12210,6 @@
           <t>reddit: Your Shopify speed score isn't your theme's fault (usually). Here's what actually kills it.</t>
         </is>
       </c>
-      <c r="F302" t="inlineStr"/>
-      <c r="G302" t="inlineStr"/>
-      <c r="H302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -12243,9 +12237,6 @@
           <t>reddit: How to align heights for each card in repeaters</t>
         </is>
       </c>
-      <c r="F303" t="inlineStr"/>
-      <c r="G303" t="inlineStr"/>
-      <c r="H303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -12273,9 +12264,6 @@
           <t>reddit: Can you make this weekly DD</t>
         </is>
       </c>
-      <c r="F304" t="inlineStr"/>
-      <c r="G304" t="inlineStr"/>
-      <c r="H304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -12303,9 +12291,6 @@
           <t>reddit: Do you TAKE THIS??? 😮‍💨😩 i wanna know</t>
         </is>
       </c>
-      <c r="F305" t="inlineStr"/>
-      <c r="G305" t="inlineStr"/>
-      <c r="H305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -12333,9 +12318,6 @@
           <t>reddit: Going online after 3 years hiatus</t>
         </is>
       </c>
-      <c r="F306" t="inlineStr"/>
-      <c r="G306" t="inlineStr"/>
-      <c r="H306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -12363,9 +12345,6 @@
           <t>reddit: taxes for instacart</t>
         </is>
       </c>
-      <c r="F307" t="inlineStr"/>
-      <c r="G307" t="inlineStr"/>
-      <c r="H307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -12393,9 +12372,6 @@
           <t>reddit: I wish Instacart would add this!</t>
         </is>
       </c>
-      <c r="F308" t="inlineStr"/>
-      <c r="G308" t="inlineStr"/>
-      <c r="H308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -12423,9 +12399,6 @@
           <t>reddit: how do y'all make so much money in a week??</t>
         </is>
       </c>
-      <c r="F309" t="inlineStr"/>
-      <c r="G309" t="inlineStr"/>
-      <c r="H309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -12453,9 +12426,66 @@
           <t>reddit: Better to wait or move stores?</t>
         </is>
       </c>
-      <c r="F310" t="inlineStr"/>
-      <c r="G310" t="inlineStr"/>
-      <c r="H310" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/careers</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr"/>
+      <c r="G311" t="inlineStr"/>
+      <c r="H311" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/instacart-plus</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr"/>
+      <c r="G312" t="inlineStr"/>
+      <c r="H312" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tier=high run 2026-06-01T17:48Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H312"/>
+  <dimension ref="A1:H318"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -12453,9 +12453,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F311" t="inlineStr"/>
-      <c r="G311" t="inlineStr"/>
-      <c r="H311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -12483,9 +12480,186 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F312" t="inlineStr"/>
-      <c r="G312" t="inlineStr"/>
-      <c r="H312" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/careers</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr"/>
+      <c r="G313" t="inlineStr"/>
+      <c r="H313" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>CHWY</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Chewy Inc.</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>https://www.chewy.com/app/content/terms</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr"/>
+      <c r="G314" t="inlineStr"/>
+      <c r="H314" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Duolingo Inc.</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>https://blog.duolingo.com/</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr"/>
+      <c r="G315" t="inlineStr"/>
+      <c r="H315" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>BILL</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>BILL Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>https://www.bill.com/product/pricing</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr"/>
+      <c r="G316" t="inlineStr"/>
+      <c r="H316" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>https://pos.toasttab.com/terms-of-service</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr"/>
+      <c r="G317" t="inlineStr"/>
+      <c r="H317" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>https://pos.toasttab.com/pricing</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr"/>
+      <c r="G318" t="inlineStr"/>
+      <c r="H318" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tier=high run 2026-06-01T18:49Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H318"/>
+  <dimension ref="A1:H319"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -12642,6 +12642,36 @@
           <t>pricing: change detected</t>
         </is>
       </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/careers</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr"/>
+      <c r="G319" t="inlineStr"/>
+      <c r="H319" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tier=high run 2026-06-02T13:14Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4099,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H319"/>
+  <dimension ref="A1:H332"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -12669,9 +12669,396 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F319" t="inlineStr"/>
-      <c r="G319" t="inlineStr"/>
-      <c r="H319" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>https://news.shopify.com</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr"/>
+      <c r="G320" t="inlineStr"/>
+      <c r="H320" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/careers</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr"/>
+      <c r="G321" t="inlineStr"/>
+      <c r="H321" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>ETSY</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Etsy Inc.</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1370637/000196922326000610/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Silverman Josh (Officer) plans to sell 134,730 shares (~$9.28M) on/after 06/01/2026</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr"/>
+      <c r="G322" t="inlineStr"/>
+      <c r="H322" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Duolingo Inc.</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>https://blog.duolingo.com/</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr"/>
+      <c r="G323" t="inlineStr"/>
+      <c r="H323" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>BILL</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>BILL Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1786352/000206742526000001/xslF345X06/form4-06012026_040616.xml</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Cieri Michael (Chief Product Officer) sold 32,875 shares @ $36.64 ($1.20M) on 2026-05-29</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr"/>
+      <c r="G324" t="inlineStr"/>
+      <c r="H324" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>BILL</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>BILL Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1786352/000179549726000002/xslF345X06/form4-06012026_040610.xml</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Lacerte Rene A. (CEO) 15,922 shares withheld for taxes (vest event) on 2026-05-28</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr"/>
+      <c r="G325" t="inlineStr"/>
+      <c r="H325" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>BILL</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>BILL Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1786352/000161395526000002/xslF345X06/form4-06012026_040614.xml</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Moss Kenneth A (Chief Technology Officer) 13,031 shares withheld for taxes (vest event) on 2026-05-28</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr"/>
+      <c r="G326" t="inlineStr"/>
+      <c r="H326" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>BILL</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>BILL Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1786352/000203968326000002/xslF345X06/form4-06012026_040612.xml</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Bowman Mary Kay (See Remarks) 6,976 shares withheld for taxes (vest event) on 2026-05-28</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr"/>
+      <c r="G327" t="inlineStr"/>
+      <c r="H327" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/toast</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>3 new non-senior roles posted</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr"/>
+      <c r="G328" t="inlineStr"/>
+      <c r="H328" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>https://pos.toasttab.com/pricing</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr"/>
+      <c r="G329" t="inlineStr"/>
+      <c r="H329" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/robinhood</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>2 new non-senior roles posted</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr"/>
+      <c r="G330" t="inlineStr"/>
+      <c r="H330" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>https://newsroom.aboutrobinhood.com</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr"/>
+      <c r="G331" t="inlineStr"/>
+      <c r="H331" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1783879/000110465926068980/xslF345X06/tm2616557-1_4seq1.xml</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Malka Meyer (Director) BOUGHT 249,000 shares @ $80.39 ($20.02M) on 2026-05-28</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr"/>
+      <c r="G332" t="inlineStr"/>
+      <c r="H332" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add v2 coverage set: LOGI GRMN TSLA LYFT UBER EXPE BKNG ABNB SPHR
Nine names spanning consumer hardware, ride-share, online travel,
and experiential venues. Tagged with Priority Tier = 'v2' so they
don't enter --tier high/medium/all filters by default — scraped only
when explicitly requested via --ticker.

URL guesses use common patterns (ir.{co}.com, newsroom.{co}.com,
etc.). Some may 404 on first run; we'll fix in a follow-up pass
based on what surfaces. EDGAR coverage works immediately via SEC's
ticker→CIK index for all 9 (all US-listed).

Monitoring Notes populated per company with thesis-relevant context
that flows into the LLM prompt (e.g. TSLA: "Watch FSD pricing,
vehicle MSRP changes, energy storage deployments"; ABNB: "Watch
host fee changes, Experiences relaunch, regulatory pressure").
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -547,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T36"/>
+  <dimension ref="A1:T45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3697,6 +3697,604 @@
         </is>
       </c>
       <c r="R36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>LOGI</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Logitech International S.A.</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://ir.logitech.com</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://www.logitech.com/en-us/about/newsroom.html</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://ir.logitech.com/corporate-governance/leadership-team</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://jobs.logitech.com</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://www.logitech.com/en-us/legal/terms-of-use.html</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=LOGI</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Consumer hardware (mice, keyboards, webcams); watch G PRO gaming and Streamlabs ecosystem</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="R37" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>GRMN</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Garmin Ltd.</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.garmin.com/en-US/company/investors/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://newsroom.garmin.com</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://www.garmin.com/en-US/company/leadership/</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://careers.garmin.com</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://www.garmin.com/en-US/legal/terms-of-use/</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=GRMN</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Garmin/</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>GPS, wearables, marine, aviation; watch fitness wearable segment vs Apple Watch</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="R38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://ir.tesla.com</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://www.tesla.com/blog</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://ir.tesla.com/corporate/leadership</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://www.tesla.com/careers</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://www.tesla.com/inventory/new/m3</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://www.tesla.com/about/legal</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=TSLA</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/teslamotors/</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Watch FSD pricing, vehicle MSRP changes, energy storage deployments, Cybertruck/Semi shipments</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="R39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://investor.lyft.com</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/blog</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://investor.lyft.com/corporate-governance/leadership</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/careers</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/pricing</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/terms</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=LYFT</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/lyftdrivers/</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Watch Lyft Pink subscription, driver pay, ride pricing; r/lyftdrivers leads on policy changes</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="R40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>UBER</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Uber Technologies, Inc.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://investor.uber.com</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://www.uber.com/newsroom/</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://investor.uber.com/governance/leadership</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.uber.com/global/en/careers/</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://www.uber.com/us/en/ride/uberone/</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://www.uber.com/legal/terms/</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=UBER</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/uberdrivers/</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Watch Uber One subscription, freight segment, autonomous vehicle partnerships, delivery commission</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="R41" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>EXPE</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Expedia Group, Inc.</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.expediagroup.com/investors/</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://newsroom.expediagroup.com</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://www.expediagroup.com/about/leadership/default.aspx</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://careers.expediagroup.com</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://www.expedia.com/legal</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=EXPE</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/expedia/</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Owns Vrbo, Hotels.com; watch ADR, room nights, take-rate changes, AI search rollout</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="R42" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BKNG</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Booking Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.bookingholdings.com/investors/</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://www.bookingholdings.com/news/</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://www.bookingholdings.com/about/leadership/</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://careers.bookingholdings.com</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/content/terms.html</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=BKNG</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Booking.com, Priceline, Agoda, Kayak; watch room-night growth, alternative-accommodations mix, Genius loyalty tier expansion</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="R43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://investors.airbnb.com</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://news.airbnb.com</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://investors.airbnb.com/leadership/</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://careers.airbnb.com</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://www.airbnb.com/terms</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=ABNB</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/airbnb_hosts/</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Watch host fee changes, Experiences relaunch, regulatory pressure (EU/NYC), Co-Host marketplace</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="R44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SPHR</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Sphere Entertainment Co.</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.sphereentertainmentco.com/investors/</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://www.sphereentertainmentco.com/newsroom/</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://www.sphereentertainmentco.com/governance/leadership/</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.sphereentertainmentco.com/careers/</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>https://www.thesphere.com/upcoming-events</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>https://www.sphereentertainmentco.com/legal/</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=SPHR</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Sphere Las Vegas venue + MSG Networks; watch event bookings, sponsor deals, Abu Dhabi sphere progress</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="R45" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4088,6 +4686,70 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId384"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId385"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId450"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12696,9 +13358,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F320" t="inlineStr"/>
-      <c r="G320" t="inlineStr"/>
-      <c r="H320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -12726,9 +13385,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F321" t="inlineStr"/>
-      <c r="G321" t="inlineStr"/>
-      <c r="H321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -12756,9 +13412,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Silverman Josh (Officer) plans to sell 134,730 shares (~$9.28M) on/after 06/01/2026</t>
         </is>
       </c>
-      <c r="F322" t="inlineStr"/>
-      <c r="G322" t="inlineStr"/>
-      <c r="H322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -12786,9 +13439,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F323" t="inlineStr"/>
-      <c r="G323" t="inlineStr"/>
-      <c r="H323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -12816,9 +13466,6 @@
           <t>[ROUTINE] Insider trade — Cieri Michael (Chief Product Officer) sold 32,875 shares @ $36.64 ($1.20M) on 2026-05-29</t>
         </is>
       </c>
-      <c r="F324" t="inlineStr"/>
-      <c r="G324" t="inlineStr"/>
-      <c r="H324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -12846,9 +13493,6 @@
           <t>[ROUTINE] Insider trade — Lacerte Rene A. (CEO) 15,922 shares withheld for taxes (vest event) on 2026-05-28</t>
         </is>
       </c>
-      <c r="F325" t="inlineStr"/>
-      <c r="G325" t="inlineStr"/>
-      <c r="H325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -12876,9 +13520,6 @@
           <t>[ROUTINE] Insider trade — Moss Kenneth A (Chief Technology Officer) 13,031 shares withheld for taxes (vest event) on 2026-05-28</t>
         </is>
       </c>
-      <c r="F326" t="inlineStr"/>
-      <c r="G326" t="inlineStr"/>
-      <c r="H326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -12906,9 +13547,6 @@
           <t>[ROUTINE] Insider trade — Bowman Mary Kay (See Remarks) 6,976 shares withheld for taxes (vest event) on 2026-05-28</t>
         </is>
       </c>
-      <c r="F327" t="inlineStr"/>
-      <c r="G327" t="inlineStr"/>
-      <c r="H327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -12936,9 +13574,6 @@
           <t>3 new non-senior roles posted</t>
         </is>
       </c>
-      <c r="F328" t="inlineStr"/>
-      <c r="G328" t="inlineStr"/>
-      <c r="H328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -12966,9 +13601,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F329" t="inlineStr"/>
-      <c r="G329" t="inlineStr"/>
-      <c r="H329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -12996,9 +13628,6 @@
           <t>2 new non-senior roles posted</t>
         </is>
       </c>
-      <c r="F330" t="inlineStr"/>
-      <c r="G330" t="inlineStr"/>
-      <c r="H330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -13026,9 +13655,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F331" t="inlineStr"/>
-      <c r="G331" t="inlineStr"/>
-      <c r="H331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -13056,9 +13682,6 @@
           <t>[ROUTINE] Insider trade — Malka Meyer (Director) BOUGHT 249,000 shares @ $80.39 ($20.02M) on 2026-05-28</t>
         </is>
       </c>
-      <c r="F332" t="inlineStr"/>
-      <c r="G332" t="inlineStr"/>
-      <c r="H332" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=LOGI,GRMN,TSLA,LYFT,UBER,EXPE,BKNG,ABNB,SPHR run 2026-06-02T13:26Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -3736,7 +3736,6 @@
           <t>https://jobs.logitech.com</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>https://www.logitech.com/en-us/legal/terms-of-use.html</t>
@@ -3747,7 +3746,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=LOGI</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
           <t>Consumer hardware (mice, keyboards, webcams); watch G PRO gaming and Streamlabs ecosystem</t>
@@ -3798,7 +3796,6 @@
           <t>https://careers.garmin.com</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>https://www.garmin.com/en-US/legal/terms-of-use/</t>
@@ -4074,7 +4071,6 @@
           <t>https://careers.expediagroup.com</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>https://www.expedia.com/legal</t>
@@ -4140,7 +4136,6 @@
           <t>https://careers.bookingholdings.com</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
           <t>https://www.booking.com/content/terms.html</t>
@@ -4151,7 +4146,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=BKNG</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
           <t>Booking.com, Priceline, Agoda, Kayak; watch room-night growth, alternative-accommodations mix, Genius loyalty tier expansion</t>
@@ -4202,7 +4196,6 @@
           <t>https://careers.airbnb.com</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
           <t>https://www.airbnb.com/terms</t>
@@ -4283,7 +4276,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=SPHR</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
           <t>Sphere Las Vegas venue + MSG Networks; watch event bookings, sponsor deals, Abu Dhabi sphere progress</t>
@@ -4761,7 +4753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H332"/>
+  <dimension ref="A1:H336"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -13682,6 +13674,126 @@
           <t>[ROUTINE] Insider trade — Malka Meyer (Director) BOUGHT 249,000 shares @ $80.39 ($20.02M) on 2026-05-28</t>
         </is>
       </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1759509/000162828026039513/lyft-formsd2026.htm</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>[UNKNOWN] Form SD</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr"/>
+      <c r="G333" t="inlineStr"/>
+      <c r="H333" t="inlineStr"/>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1759509/000192109426000578/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Llewellyn Lindsay Catherine (Officer) plans to sell 11,491 shares (~$172.4K) on/after 06/01/2026</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr"/>
+      <c r="G334" t="inlineStr"/>
+      <c r="H334" t="inlineStr"/>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1559720/000196858226000514/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Joseph Gebbia (Director) plans to sell 1,855,000 shares (~$247.29M) on/after 06/01/2026</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr"/>
+      <c r="G335" t="inlineStr"/>
+      <c r="H335" t="inlineStr"/>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1559720/000195917326004228/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Chesky Brian (Officer) plans to sell 257,273 shares (~$35.00M) on/after 06/01/2026</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr"/>
+      <c r="G336" t="inlineStr"/>
+      <c r="H336" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=LOGI,GRMN,TSLA,LYFT,UBER,EXPE,BKNG,ABNB,SPHR run 2026-06-24T02:05Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4753,7 +4753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H336"/>
+  <dimension ref="A1:H347"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -13701,9 +13701,6 @@
           <t>[UNKNOWN] Form SD</t>
         </is>
       </c>
-      <c r="F333" t="inlineStr"/>
-      <c r="G333" t="inlineStr"/>
-      <c r="H333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -13731,9 +13728,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Llewellyn Lindsay Catherine (Officer) plans to sell 11,491 shares (~$172.4K) on/after 06/01/2026</t>
         </is>
       </c>
-      <c r="F334" t="inlineStr"/>
-      <c r="G334" t="inlineStr"/>
-      <c r="H334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -13761,9 +13755,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Joseph Gebbia (Director) plans to sell 1,855,000 shares (~$247.29M) on/after 06/01/2026</t>
         </is>
       </c>
-      <c r="F335" t="inlineStr"/>
-      <c r="G335" t="inlineStr"/>
-      <c r="H335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -13791,9 +13782,336 @@
           <t>[ROUTINE] Notice of proposed insider sale — Chesky Brian (Officer) plans to sell 257,273 shares (~$35.00M) on/after 06/01/2026</t>
         </is>
       </c>
-      <c r="F336" t="inlineStr"/>
-      <c r="G336" t="inlineStr"/>
-      <c r="H336" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>LOGI</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Logitech International S.A.</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>https://ir.logitech.com</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr"/>
+      <c r="G337" t="inlineStr"/>
+      <c r="H337" t="inlineStr"/>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>GRMN</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Garmin Ltd.</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>https://newsroom.garmin.com</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr"/>
+      <c r="G338" t="inlineStr"/>
+      <c r="H338" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/blog</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr"/>
+      <c r="G339" t="inlineStr"/>
+      <c r="H339" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>https://investor.lyft.com</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr"/>
+      <c r="G340" t="inlineStr"/>
+      <c r="H340" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>EXPE</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Expedia Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>https://careers.expediagroup.com</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr"/>
+      <c r="G341" t="inlineStr"/>
+      <c r="H341" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>EXPE</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Expedia Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1324424/000132442426000042/expe-20260617.htm</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Material event disclosure</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr"/>
+      <c r="G342" t="inlineStr"/>
+      <c r="H342" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>BKNG</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Booking Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>https://www.bookingholdings.com/about/leadership/</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr"/>
+      <c r="G343" t="inlineStr"/>
+      <c r="H343" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>https://www.airbnb.com/terms</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr"/>
+      <c r="G344" t="inlineStr"/>
+      <c r="H344" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>https://news.airbnb.com</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr"/>
+      <c r="G345" t="inlineStr"/>
+      <c r="H345" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>https://careers.airbnb.com</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr"/>
+      <c r="G346" t="inlineStr"/>
+      <c r="H346" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>SPHR</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Sphere Entertainment Co.</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>https://www.sphereentertainmentco.com/careers/</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr"/>
+      <c r="G347" t="inlineStr"/>
+      <c r="H347" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=LOGI,GRMN,TSLA,LYFT,UBER,EXPE,BKNG,ABNB,SPHR run 2026-06-25T16:07Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4753,7 +4753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H347"/>
+  <dimension ref="A1:H353"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -13809,9 +13809,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr"/>
-      <c r="G337" t="inlineStr"/>
-      <c r="H337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -13839,9 +13836,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F338" t="inlineStr"/>
-      <c r="G338" t="inlineStr"/>
-      <c r="H338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -13869,9 +13863,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F339" t="inlineStr"/>
-      <c r="G339" t="inlineStr"/>
-      <c r="H339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -13899,9 +13890,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F340" t="inlineStr"/>
-      <c r="G340" t="inlineStr"/>
-      <c r="H340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -13929,9 +13917,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F341" t="inlineStr"/>
-      <c r="G341" t="inlineStr"/>
-      <c r="H341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -13959,9 +13944,6 @@
           <t>[MATERIAL] Material event disclosure</t>
         </is>
       </c>
-      <c r="F342" t="inlineStr"/>
-      <c r="G342" t="inlineStr"/>
-      <c r="H342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -13989,9 +13971,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F343" t="inlineStr"/>
-      <c r="G343" t="inlineStr"/>
-      <c r="H343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -14019,9 +13998,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F344" t="inlineStr"/>
-      <c r="G344" t="inlineStr"/>
-      <c r="H344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -14049,9 +14025,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F345" t="inlineStr"/>
-      <c r="G345" t="inlineStr"/>
-      <c r="H345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -14079,9 +14052,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F346" t="inlineStr"/>
-      <c r="G346" t="inlineStr"/>
-      <c r="H346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -14109,9 +14079,186 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F347" t="inlineStr"/>
-      <c r="G347" t="inlineStr"/>
-      <c r="H347" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>GRMN</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Garmin Ltd.</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>https://newsroom.garmin.com</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr"/>
+      <c r="G348" t="inlineStr"/>
+      <c r="H348" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>EXPE</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Expedia Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>https://careers.expediagroup.com</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr"/>
+      <c r="G349" t="inlineStr"/>
+      <c r="H349" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>BKNG</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Booking Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/content/terms.html</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr"/>
+      <c r="G350" t="inlineStr"/>
+      <c r="H350" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>https://careers.airbnb.com</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr"/>
+      <c r="G351" t="inlineStr"/>
+      <c r="H351" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1559720/000195917326004865/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Blecharczyk Nathan (Officer) plans to sell 88,366 shares (~$12.88M) on/after 06/24/2026</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr"/>
+      <c r="G352" t="inlineStr"/>
+      <c r="H352" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1559720/000195917326004851/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Blecharczyk Nathan (Officer) plans to sell 34,614 shares (~$5.02M) on/after 06/24/2026</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr"/>
+      <c r="G353" t="inlineStr"/>
+      <c r="H353" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=LOGI,GRMN,TSLA,LYFT,UBER,EXPE,BKNG,ABNB,SPHR run 2026-07-09T15:37Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4753,7 +4753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H353"/>
+  <dimension ref="A1:H366"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -14106,9 +14106,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F348" t="inlineStr"/>
-      <c r="G348" t="inlineStr"/>
-      <c r="H348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -14136,9 +14133,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F349" t="inlineStr"/>
-      <c r="G349" t="inlineStr"/>
-      <c r="H349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -14166,9 +14160,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F350" t="inlineStr"/>
-      <c r="G350" t="inlineStr"/>
-      <c r="H350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -14196,9 +14187,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F351" t="inlineStr"/>
-      <c r="G351" t="inlineStr"/>
-      <c r="H351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -14226,9 +14214,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Blecharczyk Nathan (Officer) plans to sell 88,366 shares (~$12.88M) on/after 06/24/2026</t>
         </is>
       </c>
-      <c r="F352" t="inlineStr"/>
-      <c r="G352" t="inlineStr"/>
-      <c r="H352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -14256,9 +14241,396 @@
           <t>[ROUTINE] Notice of proposed insider sale — Blecharczyk Nathan (Officer) plans to sell 34,614 shares (~$5.02M) on/after 06/24/2026</t>
         </is>
       </c>
-      <c r="F353" t="inlineStr"/>
-      <c r="G353" t="inlineStr"/>
-      <c r="H353" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>LOGI</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Logitech International S.A.</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>https://ir.logitech.com</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr"/>
+      <c r="G354" t="inlineStr"/>
+      <c r="H354" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>GRMN</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Garmin Ltd.</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>https://newsroom.garmin.com</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr"/>
+      <c r="G355" t="inlineStr"/>
+      <c r="H355" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>GRMN</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Garmin Ltd.</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1121788/000101410826000038/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Update to 5%+ passive owner disclosure</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr"/>
+      <c r="G356" t="inlineStr"/>
+      <c r="H356" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/terms</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr"/>
+      <c r="G357" t="inlineStr"/>
+      <c r="H357" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/blog</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr"/>
+      <c r="G358" t="inlineStr"/>
+      <c r="H358" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>https://investor.lyft.com</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr"/>
+      <c r="G359" t="inlineStr"/>
+      <c r="H359" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1759509/000119312526298108/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Update to 5%+ passive owner disclosure</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr"/>
+      <c r="G360" t="inlineStr"/>
+      <c r="H360" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>UBER</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Uber Technologies, Inc.</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1543151/000155278126000379/xslSCHEDULE_13D_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Update to 5%+ active owner disclosure</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr"/>
+      <c r="G361" t="inlineStr"/>
+      <c r="H361" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>EXPE</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Expedia Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>https://careers.expediagroup.com</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr"/>
+      <c r="G362" t="inlineStr"/>
+      <c r="H362" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>https://careers.airbnb.com</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr"/>
+      <c r="G363" t="inlineStr"/>
+      <c r="H363" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1559720/000119312526298928/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Blecharczyk Nathan (Chief Strategy Officer) sold 13,615 shares @ $148.37 ($2.02M) on 2026-07-06</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr"/>
+      <c r="G364" t="inlineStr"/>
+      <c r="H364" t="inlineStr"/>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1559720/000119312526297868/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Gebbia Joseph (Director) sold 27,733 shares @ $150.01 ($4.16M) on 2026-07-02</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr"/>
+      <c r="G365" t="inlineStr"/>
+      <c r="H365" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1559720/000119312526297867/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Mertz Elinor (Chief Financial Officer) sold 3,750 shares @ $148.01 ($555.0K) on 2026-07-02</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr"/>
+      <c r="G366" t="inlineStr"/>
+      <c r="H366" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=CART,DASH,CHWY run 2026-07-09T15:54Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4753,7 +4753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H366"/>
+  <dimension ref="A1:H374"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -14268,9 +14268,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F354" t="inlineStr"/>
-      <c r="G354" t="inlineStr"/>
-      <c r="H354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -14298,9 +14295,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F355" t="inlineStr"/>
-      <c r="G355" t="inlineStr"/>
-      <c r="H355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -14328,9 +14322,6 @@
           <t>[MATERIAL] Update to 5%+ passive owner disclosure</t>
         </is>
       </c>
-      <c r="F356" t="inlineStr"/>
-      <c r="G356" t="inlineStr"/>
-      <c r="H356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -14358,9 +14349,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F357" t="inlineStr"/>
-      <c r="G357" t="inlineStr"/>
-      <c r="H357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -14388,9 +14376,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F358" t="inlineStr"/>
-      <c r="G358" t="inlineStr"/>
-      <c r="H358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -14418,9 +14403,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F359" t="inlineStr"/>
-      <c r="G359" t="inlineStr"/>
-      <c r="H359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -14448,9 +14430,6 @@
           <t>[MATERIAL] Update to 5%+ passive owner disclosure</t>
         </is>
       </c>
-      <c r="F360" t="inlineStr"/>
-      <c r="G360" t="inlineStr"/>
-      <c r="H360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -14478,9 +14457,6 @@
           <t>[MATERIAL] Update to 5%+ active owner disclosure</t>
         </is>
       </c>
-      <c r="F361" t="inlineStr"/>
-      <c r="G361" t="inlineStr"/>
-      <c r="H361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -14508,9 +14484,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F362" t="inlineStr"/>
-      <c r="G362" t="inlineStr"/>
-      <c r="H362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -14538,9 +14511,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F363" t="inlineStr"/>
-      <c r="G363" t="inlineStr"/>
-      <c r="H363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -14568,9 +14538,6 @@
           <t>[ROUTINE] Insider trade — Blecharczyk Nathan (Chief Strategy Officer) sold 13,615 shares @ $148.37 ($2.02M) on 2026-07-06</t>
         </is>
       </c>
-      <c r="F364" t="inlineStr"/>
-      <c r="G364" t="inlineStr"/>
-      <c r="H364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -14598,9 +14565,6 @@
           <t>[ROUTINE] Insider trade — Gebbia Joseph (Director) sold 27,733 shares @ $150.01 ($4.16M) on 2026-07-02</t>
         </is>
       </c>
-      <c r="F365" t="inlineStr"/>
-      <c r="G365" t="inlineStr"/>
-      <c r="H365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -14628,9 +14592,246 @@
           <t>[ROUTINE] Insider trade — Mertz Elinor (Chief Financial Officer) sold 3,750 shares @ $148.01 ($555.0K) on 2026-07-02</t>
         </is>
       </c>
-      <c r="F366" t="inlineStr"/>
-      <c r="G366" t="inlineStr"/>
-      <c r="H366" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>CHWY</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Chewy Inc.</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>https://www.chewy.com/app/content/terms</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr"/>
+      <c r="G367" t="inlineStr"/>
+      <c r="H367" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com/governance/management/default.aspx</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr"/>
+      <c r="G368" t="inlineStr"/>
+      <c r="H368" t="inlineStr"/>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>https://about.doordash.com/en-us/news</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr"/>
+      <c r="G369" t="inlineStr"/>
+      <c r="H369" t="inlineStr"/>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr"/>
+      <c r="G370" t="inlineStr"/>
+      <c r="H370" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000195004726006964/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Ravi Inukonda (Officer) plans to sell 21,129 shares (~$4.14M) on/after 07/08/2026</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr"/>
+      <c r="G371" t="inlineStr"/>
+      <c r="H371" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183261426000021/xslF345X06/form4-07072026_040701.xml</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Tang Stanley (Director) sold 23,125 shares @ $191.19 ($4.42M) on 2026-07-02</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr"/>
+      <c r="G372" t="inlineStr"/>
+      <c r="H372" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/instacart-plus</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr"/>
+      <c r="G373" t="inlineStr"/>
+      <c r="H373" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/company/newsroom</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr"/>
+      <c r="G374" t="inlineStr"/>
+      <c r="H374" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=SHOP,WIX,DASH,CART run 2026-07-09T15:59Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4753,7 +4753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H374"/>
+  <dimension ref="A1:H380"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -14619,9 +14619,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F367" t="inlineStr"/>
-      <c r="G367" t="inlineStr"/>
-      <c r="H367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -14649,9 +14646,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F368" t="inlineStr"/>
-      <c r="G368" t="inlineStr"/>
-      <c r="H368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -14679,9 +14673,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F369" t="inlineStr"/>
-      <c r="G369" t="inlineStr"/>
-      <c r="H369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -14709,9 +14700,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F370" t="inlineStr"/>
-      <c r="G370" t="inlineStr"/>
-      <c r="H370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -14739,9 +14727,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Ravi Inukonda (Officer) plans to sell 21,129 shares (~$4.14M) on/after 07/08/2026</t>
         </is>
       </c>
-      <c r="F371" t="inlineStr"/>
-      <c r="G371" t="inlineStr"/>
-      <c r="H371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -14769,9 +14754,6 @@
           <t>[ROUTINE] Insider trade — Tang Stanley (Director) sold 23,125 shares @ $191.19 ($4.42M) on 2026-07-02</t>
         </is>
       </c>
-      <c r="F372" t="inlineStr"/>
-      <c r="G372" t="inlineStr"/>
-      <c r="H372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -14799,9 +14781,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F373" t="inlineStr"/>
-      <c r="G373" t="inlineStr"/>
-      <c r="H373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -14829,9 +14808,186 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F374" t="inlineStr"/>
-      <c r="G374" t="inlineStr"/>
-      <c r="H374" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/investors/board-of-directors</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr"/>
+      <c r="G375" t="inlineStr"/>
+      <c r="H375" t="inlineStr"/>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr"/>
+      <c r="G376" t="inlineStr"/>
+      <c r="H376" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>https://news.shopify.com</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr"/>
+      <c r="G377" t="inlineStr"/>
+      <c r="H377" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>https://investors.shopify.com</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr"/>
+      <c r="G378" t="inlineStr"/>
+      <c r="H378" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/careers</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr"/>
+      <c r="G379" t="inlineStr"/>
+      <c r="H379" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/upgrade/website</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr"/>
+      <c r="G380" t="inlineStr"/>
+      <c r="H380" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add v3 coverage set: VRSK CVNA HQY ARMK
Four names spanning insurance-analytics, online auto retail, HSA
custodian, and food services / uniforms. Priority Tier = 'v3' so
they're excluded from high/medium/all tier filters — use --ticker.

URL guesses follow common patterns (investor.{co}.com, etc.). Some
will 404 first run; EDGAR coverage works immediately for all 4
(all US-listed).

Monitoring Notes populated per company (e.g. CVNA: 'watch GPU,
ADESA integration, retail unit growth vs guidance'; HQY: 'HSA
account growth, custodial yield spread, investment AUM balance').
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -547,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T45"/>
+  <dimension ref="A1:T49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4287,6 +4287,258 @@
         </is>
       </c>
       <c r="R45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>VRSK</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Verisk Analytics, Inc.</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://investor.verisk.com</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://www.verisk.com/newsroom/</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://investor.verisk.com/corporate-governance/leadership</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://careers.verisk.com</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://www.verisk.com/legal/terms-of-use/</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=VRSK</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Insurance analytics + data; watch subscription revenue growth, environmental/climate data expansion, insurance underwriting product launches</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="R46" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>CVNA</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Carvana Co.</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://investors.carvana.com</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://www.carvana.com/blog</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://investors.carvana.com/corporate-governance/management</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.carvana.com/careers</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>https://www.carvana.com/terms</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=CVNA</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/carvana/</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Online used-car retailer; watch GPU (gross profit per unit), ADESA integration, retail unit growth vs guidance, auto finance spread</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="R47" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>HQY</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>HealthEquity, Inc.</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://ir.healthequity.com</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://ir.healthequity.com/news-events/press-releases</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://ir.healthequity.com/corporate-governance/leadership</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://careers.healthequity.com</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://www.healthequity.com/terms/</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=HQY</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>HSA custodian; watch HSA account growth, custodial yield spread, investment AUM balance, HSA-related legislation</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="R48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ARMK</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Aramark</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.aramark.com/about-us/investors</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://www.aramark.com/about-us/news</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://www.aramark.com/about-us/leadership</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://careers.aramark.com</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://www.aramark.com/legal/terms-of-use</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=ARMK</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Food services + uniforms; watch food inflation pass-through, uniform rental growth, education/business/healthcare segment mix</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="R49" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4742,6 +4994,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId448"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId449"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId475"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14835,9 +15112,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F375" t="inlineStr"/>
-      <c r="G375" t="inlineStr"/>
-      <c r="H375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -14865,9 +15139,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F376" t="inlineStr"/>
-      <c r="G376" t="inlineStr"/>
-      <c r="H376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -14895,9 +15166,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F377" t="inlineStr"/>
-      <c r="G377" t="inlineStr"/>
-      <c r="H377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -14925,9 +15193,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F378" t="inlineStr"/>
-      <c r="G378" t="inlineStr"/>
-      <c r="H378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -14955,9 +15220,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F379" t="inlineStr"/>
-      <c r="G379" t="inlineStr"/>
-      <c r="H379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -14985,9 +15247,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F380" t="inlineStr"/>
-      <c r="G380" t="inlineStr"/>
-      <c r="H380" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=VRSK,CVNA,HQY,ARMK run 2026-07-09T16:18Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4326,7 +4326,6 @@
           <t>https://careers.verisk.com</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>https://www.verisk.com/legal/terms-of-use/</t>
@@ -4337,7 +4336,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=VRSK</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
           <t>Insurance analytics + data; watch subscription revenue growth, environmental/climate data expansion, insurance underwriting product launches</t>
@@ -4388,7 +4386,6 @@
           <t>https://www.carvana.com/careers</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
           <t>https://www.carvana.com/terms</t>
@@ -4454,7 +4451,6 @@
           <t>https://careers.healthequity.com</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
           <t>https://www.healthequity.com/terms/</t>
@@ -4465,7 +4461,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=HQY</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
           <t>HSA custodian; watch HSA account growth, custodial yield spread, investment AUM balance, HSA-related legislation</t>
@@ -4516,7 +4511,6 @@
           <t>https://careers.aramark.com</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
           <t>https://www.aramark.com/legal/terms-of-use</t>
@@ -4527,7 +4521,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=ARMK</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
           <t>Food services + uniforms; watch food inflation pass-through, uniform rental growth, education/business/healthcare segment mix</t>
@@ -5030,7 +5023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H380"/>
+  <dimension ref="A1:H386"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15247,6 +15240,186 @@
           <t>pricing: change detected</t>
         </is>
       </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>VRSK</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Verisk Analytics, Inc.</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1442145/000119312526298574/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Purtill Sabra R. (Director) RSU/grant of 163 shares on 2026-06-30</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr"/>
+      <c r="G381" t="inlineStr"/>
+      <c r="H381" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>VRSK</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Verisk Analytics, Inc.</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1442145/000119312526298568/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Christopher John Perry (Director) RSU/grant of 146 shares on 2026-06-30</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr"/>
+      <c r="G382" t="inlineStr"/>
+      <c r="H382" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>VRSK</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Verisk Analytics, Inc.</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1442145/000119312526298564/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Hendrick Gregory (Director) RSU/grant of 146 shares on 2026-06-30</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr"/>
+      <c r="G383" t="inlineStr"/>
+      <c r="H383" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>VRSK</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Verisk Analytics, Inc.</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1442145/000119312526298561/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Patiath Pradip (Director) RSU/grant of 69 shares on 2026-06-30</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr"/>
+      <c r="G384" t="inlineStr"/>
+      <c r="H384" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>VRSK</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Verisk Analytics, Inc.</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1442145/000119312526298556/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Samuel G Liss (Director) RSU/grant of 167 shares on 2026-06-30</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr"/>
+      <c r="G385" t="inlineStr"/>
+      <c r="H385" t="inlineStr"/>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>HQY</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>HealthEquity, Inc.</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1428336/000201611626000014/xslF345X06/form4-07072026_080705.xml</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Fiore Michael Henry (EVP, CHIEF COMMERCIAL OFFICER) sold 2,470 shares @ $95.00 ($234.7K) on 2026-07-02</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr"/>
+      <c r="G386" t="inlineStr"/>
+      <c r="H386" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=CART,DASH,SHOP,WIX run 2026-07-10T12:26Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -5023,7 +5023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H386"/>
+  <dimension ref="A1:H389"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15267,9 +15267,6 @@
           <t>[ROUTINE] Insider trade — Purtill Sabra R. (Director) RSU/grant of 163 shares on 2026-06-30</t>
         </is>
       </c>
-      <c r="F381" t="inlineStr"/>
-      <c r="G381" t="inlineStr"/>
-      <c r="H381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -15297,9 +15294,6 @@
           <t>[ROUTINE] Insider trade — Christopher John Perry (Director) RSU/grant of 146 shares on 2026-06-30</t>
         </is>
       </c>
-      <c r="F382" t="inlineStr"/>
-      <c r="G382" t="inlineStr"/>
-      <c r="H382" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -15327,9 +15321,6 @@
           <t>[ROUTINE] Insider trade — Hendrick Gregory (Director) RSU/grant of 146 shares on 2026-06-30</t>
         </is>
       </c>
-      <c r="F383" t="inlineStr"/>
-      <c r="G383" t="inlineStr"/>
-      <c r="H383" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -15357,9 +15348,6 @@
           <t>[ROUTINE] Insider trade — Patiath Pradip (Director) RSU/grant of 69 shares on 2026-06-30</t>
         </is>
       </c>
-      <c r="F384" t="inlineStr"/>
-      <c r="G384" t="inlineStr"/>
-      <c r="H384" t="inlineStr"/>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -15387,9 +15375,6 @@
           <t>[ROUTINE] Insider trade — Samuel G Liss (Director) RSU/grant of 167 shares on 2026-06-30</t>
         </is>
       </c>
-      <c r="F385" t="inlineStr"/>
-      <c r="G385" t="inlineStr"/>
-      <c r="H385" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -15417,9 +15402,96 @@
           <t>[ROUTINE] Insider trade — Fiore Michael Henry (EVP, CHIEF COMMERCIAL OFFICER) sold 2,470 shares @ $95.00 ($234.7K) on 2026-07-02</t>
         </is>
       </c>
-      <c r="F386" t="inlineStr"/>
-      <c r="G386" t="inlineStr"/>
-      <c r="H386" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/careers</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr"/>
+      <c r="G387" t="inlineStr"/>
+      <c r="H387" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com/governance/management/default.aspx</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr"/>
+      <c r="G388" t="inlineStr"/>
+      <c r="H388" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr"/>
+      <c r="G389" t="inlineStr"/>
+      <c r="H389" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=ABNB,BKNG,EXPE,GRMN,LOGI,LYFT,SPHR,TSLA,UBER run 2026-07-10T12:34Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -5023,7 +5023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H389"/>
+  <dimension ref="A1:H394"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15429,9 +15429,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F387" t="inlineStr"/>
-      <c r="G387" t="inlineStr"/>
-      <c r="H387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -15459,9 +15456,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F388" t="inlineStr"/>
-      <c r="G388" t="inlineStr"/>
-      <c r="H388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -15489,9 +15483,156 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F389" t="inlineStr"/>
-      <c r="G389" t="inlineStr"/>
-      <c r="H389" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>LOGI</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Logitech International S.A.</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>https://ir.logitech.com</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr"/>
+      <c r="G390" t="inlineStr"/>
+      <c r="H390" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/blog</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr"/>
+      <c r="G391" t="inlineStr"/>
+      <c r="H391" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>EXPE</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Expedia Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>https://careers.expediagroup.com</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr"/>
+      <c r="G392" t="inlineStr"/>
+      <c r="H392" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>https://careers.airbnb.com</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr"/>
+      <c r="G393" t="inlineStr"/>
+      <c r="H393" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1559720/000119312526299741/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Gebbia Joseph (Director) sold 2,460 shares @ $150.00 ($369.0K) on 2026-07-07</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr"/>
+      <c r="G394" t="inlineStr"/>
+      <c r="H394" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=ARMK,CVNA,HQY,VRSK run 2026-07-10T12:36Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -5023,7 +5023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H394"/>
+  <dimension ref="A1:H395"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15510,9 +15510,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F390" t="inlineStr"/>
-      <c r="G390" t="inlineStr"/>
-      <c r="H390" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -15540,9 +15537,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F391" t="inlineStr"/>
-      <c r="G391" t="inlineStr"/>
-      <c r="H391" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -15570,9 +15564,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F392" t="inlineStr"/>
-      <c r="G392" t="inlineStr"/>
-      <c r="H392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -15600,9 +15591,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F393" t="inlineStr"/>
-      <c r="G393" t="inlineStr"/>
-      <c r="H393" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -15630,9 +15618,36 @@
           <t>[ROUTINE] Insider trade — Gebbia Joseph (Director) sold 2,460 shares @ $150.00 ($369.0K) on 2026-07-07</t>
         </is>
       </c>
-      <c r="F394" t="inlineStr"/>
-      <c r="G394" t="inlineStr"/>
-      <c r="H394" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>ARMK</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Aramark</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>https://careers.aramark.com</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr"/>
+      <c r="G395" t="inlineStr"/>
+      <c r="H395" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add v4 coverage set (32 names: media, gaming, HR tech, travel, ads)
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -547,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T49"/>
+  <dimension ref="A1:T81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4532,6 +4532,1854 @@
         </is>
       </c>
       <c r="R49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>YOU</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Clear Secure, Inc.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://ir.clearme.com</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://ir.clearme.com/news-events</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.clearme.com/careers</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>https://www.clearme.com/legal</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=YOU</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Biometric identity verification; watch Clear Plus subscription growth, airport partnership expansions, TSA PreCheck competition</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CHH</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Choice Hotels International, Inc.</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://media.choicehotels.com/investors</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://media.choicehotels.com</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://careers.choicehotels.com</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>https://www.choicehotels.com/legal/terms-of-use</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=CHH</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Franchised hotels (Comfort, Quality, Radisson Americas); watch RevPAR, unit growth, Radisson integration</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://investor.atmeta.com</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://about.fb.com/news/</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://about.meta.com/company-info/</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.metacareers.com</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/legal/terms</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=META</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Watch Reels monetization, Threads growth, Reality Labs spend, AI capex, WhatsApp Business</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R52" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://abc.xyz/investor/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://blog.google</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://abc.xyz/investor/other/management/</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://careers.google.com</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://policies.google.com/terms</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=GOOG</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Watch Search AI overviews impact, Cloud growth vs AWS/Azure, YouTube ad revenue, Waymo scaling, DOJ antitrust remedies</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://investor.snap.com</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://newsroom.snap.com</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://investor.snap.com/corporate-governance/leadership/</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://careers.snap.com</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://snap.com/en-US/terms</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=SNAP</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr"/>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Watch DAU trend, Snapchat+ subscription, ad revenue vs guidance, AR partnerships</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R54" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>PINS</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Pinterest, Inc.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://investor.pinterestinc.com</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://newsroom.pinterest.com</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.pinterestcareers.com</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>https://policy.pinterest.com/en/terms-of-service</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=PINS</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Watch MAU trend, ARPU growth, shopping/commerce integrations, Amazon partnership scaling</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Reddit, Inc.</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://investor.redditinc.com</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://redditinc.com/press</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://redditinc.com/careers</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>https://www.redditinc.com/policies/user-agreement</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=RDDT</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/reddit/</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Watch data licensing deals (Google/OpenAI), ad revenue growth, DAUq trend, Reddit Answers rollout</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R56" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>AppLovin Corporation</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://investors.applovin.com</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://www.applovin.com/blog/</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.applovin.com/careers/</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>https://www.applovin.com/legal/</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=APP</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Ad tech / mobile gaming; watch AXON 2 ML model performance, e-commerce ad expansion, gaming vs non-gaming ad mix</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R57" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Unity Software Inc.</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://investors.unity.com</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://unity.com/company/press</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://careers.unity.com</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>https://unity.com/legal/terms-of-service</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=U</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Watch Runtime Fee resolution/aftermath, Create/Grow segment split, subscription renewals</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R58" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Netflix, Inc.</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://ir.netflix.net</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://about.netflix.com/en/news</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://jobs.netflix.com</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://help.netflix.com/en/node/24926</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>https://help.netflix.com/legal/termsofuse</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=NFLX</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Watch subscriber adds, ARM changes, ads-tier growth, content spend, live sports strategy, password-sharing crackdown effect</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R59" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://investors.spotify.com</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://newsroom.spotify.com</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.lifeatspotify.com</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://www.spotify.com/premium</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>https://www.spotify.com/legal/end-user-agreement/</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=SPOT</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Watch MAU/Premium sub growth, gross margin (audiobook/podcast), pricing power, Marketplace ad revenue</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R60" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>NYT</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>The New York Times Company</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://investors.nytco.com</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://www.nytco.com/press/</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.nytco.com/careers/</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>https://help.nytimes.com/hc/en-us/articles/115014893428</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=NYT</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Watch digital subs adds (news, cooking, games, Wirecutter, Athletic), ARPU, bundle attach rate</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R61" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>LIF</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>LIF (verify ticker)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=LIF</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr"/>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Ticker unclear — could be Life Insurance / other. Verify via SEC index.</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R62" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BBY</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Best Buy Co., Inc.</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://investors.bestbuy.com</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://corporate.bestbuy.com/newsroom/</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://jobs.bestbuy.com</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>https://www.bestbuy.com/site/help-topics/terms-and-conditions/pcmcat204400050067.c</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=BBY</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Watch comparable sales, membership (My Best Buy Total), TotalTech services attach, gaming/PC upgrade cycle</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R63" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://thewaltdisneycompany.com/investor-relations/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://thewaltdisneycompany.com/news/</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://jobs.disneycareers.com</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://www.disneyplus.com/welcome</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>https://disneytermsofuse.com</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=DIS</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Watch DTC (Disney+/Hulu/ESPN+) sub growth + profitability, ESPN direct-to-consumer 2025 launch, Parks OI, streaming ARPU</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R64" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://investor.foxcorporation.com</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://www.foxcorporation.com/news/</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://foxcareers.com</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>https://www.fox.com/terms-of-use</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=FOXA</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr"/>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Watch Tubi ad growth, Fox News ratings + political cycle, Sports rights renewals, retransmission fees</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R65" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>UMG</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Universal Music Group N.V.</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Euronext Amsterdam</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://www.universalmusic.com/investor-relations/</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://www.universalmusic.com/news/</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://www.universalmusic.com/careers/</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=UMG</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Non-US listed (Euronext); watch subscription streaming ARPU trends, TikTok deal, artist advance write-downs</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R66" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>WMG</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Warner Music Group Corp.</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://investors.wmg.com</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://www.wmg.com/news/</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://careers.wmg.com</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>https://www.wmg.com/terms-of-use</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=WMG</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Watch streaming revenue growth, mechanical royalty rates, artist advances, Live Nation vs. WMG dynamics</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R67" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>LYV</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Live Nation Entertainment, Inc.</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://investors.livenationentertainment.com</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://www.livenationentertainment.com/newsroom/</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://careers.livenationentertainment.com</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>https://help.ticketmaster.com/hc/en-us/articles/10736907984657</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=LYV</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Watch DOJ lawsuit outcomes, ticket AOV, concert attendance, Ticketmaster market share, VIP/premium seat mix</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R68" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>STUB</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>StubHub Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://investors.stubhub.com</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/press</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/careers/</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/legal/</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=STUB</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr"/>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Recent 2024/2025 IPO; watch GMV growth, take rate, marketing spend, international expansion</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R69" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>LION (verify ticker)</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=LION</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr"/>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Ticker unclear — could be Fidelity National Financial or Lions Gate. Verify via SEC index.</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R70" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>OUTFRONT Media Inc.</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://investor.outfrontmedia.com</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://www.outfrontmedia.com/newsroom/</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://www.outfrontmedia.com/careers</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>https://www.outfrontmedia.com/legal/</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=OUT</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr"/>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Out-of-home advertising (billboards, transit); watch same-store growth, digital conversion, MTA contract</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R71" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>LAMR</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Lamar Advertising Company</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://www.lamar.com/investor-relations</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://www.lamar.com/news</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://www.lamar.com/careers</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>https://www.lamar.com/terms-of-use</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=LAMR</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Out-of-home advertising REIT; watch same-store growth, digital board conversion, dividend policy</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R72" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Take-Two Interactive Software, Inc.</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://ir.take2games.com</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>https://ir.take2games.com/press-releases</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.take2games.com/careers</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=TTWO</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr"/>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Watch GTA VI launch timing/reception, NBA 2K + Zynga performance, deferred revenue accretion</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R73" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Electronic Arts Inc.</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://ir.ea.com</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>https://www.ea.com/news</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://ea.com/careers</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>https://tos.ea.com</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=EA</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr"/>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Watch EA SPORTS FC engagement, Battlefield launches, live services bookings, mobile gaming</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R74" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>RBLX</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Roblox Corporation</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://ir.roblox.com</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>https://ir.roblox.com/news-releases</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://careers.roblox.com</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>https://en.help.roblox.com/hc/en-us/articles/115004647846</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=RBLX</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr"/>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Watch DAU trend (esp older cohorts), bookings/DAU, developer earnings share, advertising rollout, Roblox Studio AI</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R75" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Intuit Inc.</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://investors.intuit.com</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>https://www.intuit.com/company/press-room/</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://www.intuit.com/careers/</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>https://quickbooks.intuit.com/pricing/</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>https://www.intuit.com/legal/terms-of-service/</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=INTU</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr"/>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Watch QuickBooks Online growth, TurboTax mix, Credit Karma monetization, Mailchimp cross-sell, AI features</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R76" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing, Inc.</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://investors.adp.com</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>https://mediacenter.adp.com</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://jobs.adp.com</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>https://www.adp.com/about-adp/privacy.aspx</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=ADP</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr"/>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Watch pays per control (employment proxy), client fund float, employer services growth, PEO segment</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R77" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>PAYX</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Paychex, Inc.</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://investor.paychex.com</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>https://www.paychex.com/newsroom</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://www.paychex.com/careers</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>https://www.paychex.com/terms-of-use</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=PAYX</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr"/>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Watch client count, HR services attach rates, retention, float income, PEO expansion</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R78" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>PAYC</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Paycom Software, Inc.</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://investors.paycom.com</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>https://www.paycom.com/resources/news/</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://paycom.com/careers</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>https://www.paycom.com/terms-of-use/</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=PAYC</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr"/>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>Watch Beti self-service adoption, revenue per client, sales productivity, competitive pressure vs Rippling/Gusto</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R79" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>PCTY</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Paylocity Holding Corporation</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://investors.paylocity.com</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>https://www.paylocity.com/resources/press-releases/</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://www.paylocity.com/careers</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>https://www.paylocity.com/terms/</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=PCTY</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr"/>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Watch mid-market win rate, revenue per client, community features / employee experience adoption</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R80" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>CDW Corporation</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://investor.cdw.com</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>https://www.cdw.com/content/cdw/en/about/newsroom.html</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://www.cdw.com/content/cdw/en/careers.html</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>https://www.cdw.com/content/cdw/en/terms-conditions.html</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=CDW</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr"/>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>IT reseller; watch corporate/public/small-biz mix, gross margin, hardware refresh cycle, cloud services growth</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="R81" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5012,6 +6860,164 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId473"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId474"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId633"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15645,9 +17651,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F395" t="inlineStr"/>
-      <c r="G395" t="inlineStr"/>
-      <c r="H395" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=BKNG,EXPE,ABNB,YOU,CHH,META,GOOG,SNAP,PINS,RDDT,APP,U,UBER,LYFT,TSLA,NFLX,SPOT,NYT,LIF,LOGI,GRMN,BBY,DIS,FOXA,UMG,WMG,LYV,SPHR,STUB,LION,OUT,LAMR,TTWO,EA,RBLX,INTU,ADP,PAYX,PAYC,PCTY,CDW run 2026-07-13T15:47Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -4561,13 +4561,11 @@
           <t>https://ir.clearme.com/news-events</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>https://www.clearme.com/careers</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
           <t>https://www.clearme.com/legal</t>
@@ -4578,7 +4576,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=YOU</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
         <is>
           <t>Biometric identity verification; watch Clear Plus subscription growth, airport partnership expansions, TSA PreCheck competition</t>
@@ -4619,13 +4616,11 @@
           <t>https://media.choicehotels.com</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>https://careers.choicehotels.com</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
           <t>https://www.choicehotels.com/legal/terms-of-use</t>
@@ -4636,7 +4631,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=CHH</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
         <is>
           <t>Franchised hotels (Comfort, Quality, Radisson Americas); watch RevPAR, unit growth, Radisson integration</t>
@@ -4687,7 +4681,6 @@
           <t>https://www.metacareers.com</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>https://www.facebook.com/legal/terms</t>
@@ -4698,7 +4691,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=META</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
           <t>Watch Reels monetization, Threads growth, Reality Labs spend, AI capex, WhatsApp Business</t>
@@ -4749,7 +4741,6 @@
           <t>https://careers.google.com</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
           <t>https://policies.google.com/terms</t>
@@ -4760,7 +4751,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=GOOG</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
       <c r="P53" t="inlineStr">
         <is>
           <t>Watch Search AI overviews impact, Cloud growth vs AWS/Azure, YouTube ad revenue, Waymo scaling, DOJ antitrust remedies</t>
@@ -4811,7 +4801,6 @@
           <t>https://careers.snap.com</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>https://snap.com/en-US/terms</t>
@@ -4822,7 +4811,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=SNAP</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
         <is>
           <t>Watch DAU trend, Snapchat+ subscription, ad revenue vs guidance, AR partnerships</t>
@@ -4863,13 +4851,11 @@
           <t>https://newsroom.pinterest.com</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>https://www.pinterestcareers.com</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>https://policy.pinterest.com/en/terms-of-service</t>
@@ -4880,7 +4866,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=PINS</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
         <is>
           <t>Watch MAU trend, ARPU growth, shopping/commerce integrations, Amazon partnership scaling</t>
@@ -4921,13 +4906,11 @@
           <t>https://redditinc.com/press</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
           <t>https://redditinc.com/careers</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
           <t>https://www.redditinc.com/policies/user-agreement</t>
@@ -4983,13 +4966,11 @@
           <t>https://www.applovin.com/blog/</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
           <t>https://www.applovin.com/careers/</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
           <t>https://www.applovin.com/legal/</t>
@@ -5000,7 +4981,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=APP</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
           <t>Ad tech / mobile gaming; watch AXON 2 ML model performance, e-commerce ad expansion, gaming vs non-gaming ad mix</t>
@@ -5041,13 +5021,11 @@
           <t>https://unity.com/company/press</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
           <t>https://careers.unity.com</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
           <t>https://unity.com/legal/terms-of-service</t>
@@ -5058,7 +5036,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=U</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
         <is>
           <t>Watch Runtime Fee resolution/aftermath, Create/Grow segment split, subscription renewals</t>
@@ -5099,7 +5076,6 @@
           <t>https://about.netflix.com/en/news</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
           <t>https://jobs.netflix.com</t>
@@ -5120,7 +5096,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=NFLX</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
           <t>Watch subscriber adds, ARM changes, ads-tier growth, content spend, live sports strategy, password-sharing crackdown effect</t>
@@ -5161,7 +5136,6 @@
           <t>https://newsroom.spotify.com</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>https://www.lifeatspotify.com</t>
@@ -5182,7 +5156,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=SPOT</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
           <t>Watch MAU/Premium sub growth, gross margin (audiobook/podcast), pricing power, Marketplace ad revenue</t>
@@ -5223,13 +5196,11 @@
           <t>https://www.nytco.com/press/</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
           <t>https://www.nytco.com/careers/</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
           <t>https://help.nytimes.com/hc/en-us/articles/115014893428</t>
@@ -5240,7 +5211,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=NYT</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
       <c r="P61" t="inlineStr">
         <is>
           <t>Watch digital subs adds (news, cooking, games, Wirecutter, Athletic), ARPU, bundle attach rate</t>
@@ -5271,18 +5241,11 @@
           <t>?</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr">
         <is>
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=LIF</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
         <is>
           <t>Ticker unclear — could be Life Insurance / other. Verify via SEC index.</t>
@@ -5323,13 +5286,11 @@
           <t>https://corporate.bestbuy.com/newsroom/</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
           <t>https://jobs.bestbuy.com</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
           <t>https://www.bestbuy.com/site/help-topics/terms-and-conditions/pcmcat204400050067.c</t>
@@ -5340,7 +5301,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=BBY</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
       <c r="P63" t="inlineStr">
         <is>
           <t>Watch comparable sales, membership (My Best Buy Total), TotalTech services attach, gaming/PC upgrade cycle</t>
@@ -5381,7 +5341,6 @@
           <t>https://thewaltdisneycompany.com/news/</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
           <t>https://jobs.disneycareers.com</t>
@@ -5402,7 +5361,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=DIS</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
         <is>
           <t>Watch DTC (Disney+/Hulu/ESPN+) sub growth + profitability, ESPN direct-to-consumer 2025 launch, Parks OI, streaming ARPU</t>
@@ -5443,13 +5401,11 @@
           <t>https://www.foxcorporation.com/news/</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
           <t>https://foxcareers.com</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
           <t>https://www.fox.com/terms-of-use</t>
@@ -5460,7 +5416,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=FOXA</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
       <c r="P65" t="inlineStr">
         <is>
           <t>Watch Tubi ad growth, Fox News ratings + political cycle, Sports rights renewals, retransmission fees</t>
@@ -5501,20 +5456,16 @@
           <t>https://www.universalmusic.com/news/</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>https://www.universalmusic.com/careers/</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr">
         <is>
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=UMG</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr"/>
       <c r="P66" t="inlineStr">
         <is>
           <t>Non-US listed (Euronext); watch subscription streaming ARPU trends, TikTok deal, artist advance write-downs</t>
@@ -5555,13 +5506,11 @@
           <t>https://www.wmg.com/news/</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
           <t>https://careers.wmg.com</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>https://www.wmg.com/terms-of-use</t>
@@ -5572,7 +5521,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=WMG</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
       <c r="P67" t="inlineStr">
         <is>
           <t>Watch streaming revenue growth, mechanical royalty rates, artist advances, Live Nation vs. WMG dynamics</t>
@@ -5613,13 +5561,11 @@
           <t>https://www.livenationentertainment.com/newsroom/</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
           <t>https://careers.livenationentertainment.com</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr">
         <is>
           <t>https://help.ticketmaster.com/hc/en-us/articles/10736907984657</t>
@@ -5630,7 +5576,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=LYV</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
       <c r="P68" t="inlineStr">
         <is>
           <t>Watch DOJ lawsuit outcomes, ticket AOV, concert attendance, Ticketmaster market share, VIP/premium seat mix</t>
@@ -5671,13 +5616,11 @@
           <t>https://www.stubhub.com/press</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
           <t>https://www.stubhub.com/careers/</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
         <is>
           <t>https://www.stubhub.com/legal/</t>
@@ -5688,7 +5631,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=STUB</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
       <c r="P69" t="inlineStr">
         <is>
           <t>Recent 2024/2025 IPO; watch GMV growth, take rate, marketing spend, international expansion</t>
@@ -5719,18 +5661,11 @@
           <t>?</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr">
         <is>
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=LION</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr"/>
       <c r="P70" t="inlineStr">
         <is>
           <t>Ticker unclear — could be Fidelity National Financial or Lions Gate. Verify via SEC index.</t>
@@ -5771,13 +5706,11 @@
           <t>https://www.outfrontmedia.com/newsroom/</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
           <t>https://www.outfrontmedia.com/careers</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr">
         <is>
           <t>https://www.outfrontmedia.com/legal/</t>
@@ -5788,7 +5721,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=OUT</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr"/>
       <c r="P71" t="inlineStr">
         <is>
           <t>Out-of-home advertising (billboards, transit); watch same-store growth, digital conversion, MTA contract</t>
@@ -5829,13 +5761,11 @@
           <t>https://www.lamar.com/news</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
           <t>https://www.lamar.com/careers</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr">
         <is>
           <t>https://www.lamar.com/terms-of-use</t>
@@ -5846,7 +5776,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=LAMR</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
       <c r="P72" t="inlineStr">
         <is>
           <t>Out-of-home advertising REIT; watch same-store growth, digital board conversion, dividend policy</t>
@@ -5887,20 +5816,16 @@
           <t>https://ir.take2games.com/press-releases</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>https://www.take2games.com/careers</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=TTWO</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr"/>
       <c r="P73" t="inlineStr">
         <is>
           <t>Watch GTA VI launch timing/reception, NBA 2K + Zynga performance, deferred revenue accretion</t>
@@ -5941,13 +5866,11 @@
           <t>https://www.ea.com/news</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
           <t>https://ea.com/careers</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr">
         <is>
           <t>https://tos.ea.com</t>
@@ -5958,7 +5881,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=EA</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr"/>
       <c r="P74" t="inlineStr">
         <is>
           <t>Watch EA SPORTS FC engagement, Battlefield launches, live services bookings, mobile gaming</t>
@@ -5999,13 +5921,11 @@
           <t>https://ir.roblox.com/news-releases</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
           <t>https://careers.roblox.com</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
           <t>https://en.help.roblox.com/hc/en-us/articles/115004647846</t>
@@ -6016,7 +5936,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=RBLX</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
       <c r="P75" t="inlineStr">
         <is>
           <t>Watch DAU trend (esp older cohorts), bookings/DAU, developer earnings share, advertising rollout, Roblox Studio AI</t>
@@ -6057,7 +5976,6 @@
           <t>https://www.intuit.com/company/press-room/</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
           <t>https://www.intuit.com/careers/</t>
@@ -6078,7 +5996,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=INTU</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr"/>
       <c r="P76" t="inlineStr">
         <is>
           <t>Watch QuickBooks Online growth, TurboTax mix, Credit Karma monetization, Mailchimp cross-sell, AI features</t>
@@ -6119,13 +6036,11 @@
           <t>https://mediacenter.adp.com</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>https://jobs.adp.com</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
           <t>https://www.adp.com/about-adp/privacy.aspx</t>
@@ -6136,7 +6051,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=ADP</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr"/>
       <c r="P77" t="inlineStr">
         <is>
           <t>Watch pays per control (employment proxy), client fund float, employer services growth, PEO segment</t>
@@ -6177,13 +6091,11 @@
           <t>https://www.paychex.com/newsroom</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>https://www.paychex.com/careers</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr">
         <is>
           <t>https://www.paychex.com/terms-of-use</t>
@@ -6194,7 +6106,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=PAYX</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr"/>
       <c r="P78" t="inlineStr">
         <is>
           <t>Watch client count, HR services attach rates, retention, float income, PEO expansion</t>
@@ -6235,13 +6146,11 @@
           <t>https://www.paycom.com/resources/news/</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
           <t>https://paycom.com/careers</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
           <t>https://www.paycom.com/terms-of-use/</t>
@@ -6252,7 +6161,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=PAYC</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr"/>
       <c r="P79" t="inlineStr">
         <is>
           <t>Watch Beti self-service adoption, revenue per client, sales productivity, competitive pressure vs Rippling/Gusto</t>
@@ -6293,13 +6201,11 @@
           <t>https://www.paylocity.com/resources/press-releases/</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
           <t>https://www.paylocity.com/careers</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
       <c r="I80" t="inlineStr">
         <is>
           <t>https://www.paylocity.com/terms/</t>
@@ -6310,7 +6216,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=PCTY</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr"/>
       <c r="P80" t="inlineStr">
         <is>
           <t>Watch mid-market win rate, revenue per client, community features / employee experience adoption</t>
@@ -6351,13 +6256,11 @@
           <t>https://www.cdw.com/content/cdw/en/about/newsroom.html</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>https://www.cdw.com/content/cdw/en/careers.html</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
           <t>https://www.cdw.com/content/cdw/en/terms-conditions.html</t>
@@ -6368,7 +6271,6 @@
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=CDW</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr"/>
       <c r="P81" t="inlineStr">
         <is>
           <t>IT reseller; watch corporate/public/small-biz mix, gross margin, hardware refresh cycle, cloud services growth</t>
@@ -7029,7 +6931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H395"/>
+  <dimension ref="A1:H398"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17651,6 +17553,96 @@
           <t>careers: change detected</t>
         </is>
       </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/blog</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr"/>
+      <c r="G396" t="inlineStr"/>
+      <c r="H396" t="inlineStr"/>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>EXPE</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Expedia Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>https://careers.expediagroup.com</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr"/>
+      <c r="G397" t="inlineStr"/>
+      <c r="H397" t="inlineStr"/>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>LIF</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>LIF (verify ticker)</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1581760/000195917326005204/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Prober Charles J. (Director) plans to sell 7,930 shares (~$420.7K) on/after 07/13/2026</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr"/>
+      <c r="G398" t="inlineStr"/>
+      <c r="H398" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix 24 v4 URL failures + clear 13 bot-blocked URLs
Mechanical HEAD-audit pass over the 78 URL failures from yesterday's
41-ticker run. tools/audit_and_fix_v4.py tries a small set of common
per-source URL patterns against each broken host and keeps the first
200 + real-content hit.

Fixed 24 URLs across 18 tickers (ADP, BBY, BKNG, EXPE, GOOG, LAMR,
LOGI, LYV, NFLX, OUT, PAYX, RBLX, SNAP, SPHR, U, WMG, YOU) and blanked
13 permanently bot-blocked URLs on TSLA/UBER/PAYC so the scraper stops
retrying and logs clean skips.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -3723,12 +3723,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.logitech.com/en-us/about/newsroom.html</t>
+          <t>https://www.logitech.com/press</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://ir.logitech.com/corporate-governance/leadership-team</t>
+          <t>https://ir.logitech.com/corporate-governance/leadership</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://www.logitech.com/en-us/legal/terms-of-use.html</t>
+          <t>https://www.logitech.com/terms</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -3841,36 +3841,6 @@
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>https://ir.tesla.com</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>https://www.tesla.com/blog</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>https://ir.tesla.com/corporate/leadership</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>https://www.tesla.com/careers</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>https://www.tesla.com/inventory/new/m3</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>https://www.tesla.com/about/legal</t>
-        </is>
-      </c>
       <c r="J39" t="inlineStr">
         <is>
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=TSLA</t>
@@ -3986,29 +3956,9 @@
           <t>https://investor.uber.com</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>https://www.uber.com/newsroom/</t>
-        </is>
-      </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>https://investor.uber.com/governance/leadership</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>https://www.uber.com/global/en/careers/</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>https://www.uber.com/us/en/ride/uberone/</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>https://www.uber.com/legal/terms/</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4058,7 +4008,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://newsroom.expediagroup.com</t>
+          <t>https://www.expediagroup.com/media</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4123,7 +4073,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://www.bookingholdings.com/news/</t>
+          <t>https://www.bookingholdings.com/press-releases</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -4133,7 +4083,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://careers.bookingholdings.com</t>
+          <t>https://www.bookingholdings.com/careers</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4253,7 +4203,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://www.sphereentertainmentco.com/governance/leadership/</t>
+          <t>https://www.sphereentertainmentco.com/leadership</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4268,7 +4218,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://www.sphereentertainmentco.com/legal/</t>
+          <t>https://www.sphereentertainmentco.com/terms</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4568,7 +4518,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>https://www.clearme.com/legal</t>
+          <t>https://www.clearme.com/terms</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -4733,7 +4683,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://abc.xyz/investor/other/management/</t>
+          <t>https://abc.xyz/governance/leadership</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -4793,7 +4743,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://investor.snap.com/corporate-governance/leadership/</t>
+          <t>https://investor.snap.com/governance/leadership</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -5018,7 +4968,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://unity.com/company/press</t>
+          <t>https://unity.com/news</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -5073,7 +5023,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://about.netflix.com/en/news</t>
+          <t>https://about.netflix.com/newsroom</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -5283,7 +5233,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>https://corporate.bestbuy.com/newsroom/</t>
+          <t>https://corporate.bestbuy.com/news</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -5508,7 +5458,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://careers.wmg.com</t>
+          <t>https://www.wmg.com/careers</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -5563,12 +5513,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://careers.livenationentertainment.com</t>
+          <t>https://www.livenationentertainment.com/careers</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>https://help.ticketmaster.com/hc/en-us/articles/10736907984657</t>
+          <t>https://www.livenationentertainment.com/terms</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -5703,7 +5653,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://www.outfrontmedia.com/newsroom/</t>
+          <t>https://www.outfrontmedia.com/media</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -5713,7 +5663,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>https://www.outfrontmedia.com/legal/</t>
+          <t>https://www.outfrontmedia.com/terms-of-use</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -5753,7 +5703,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://www.lamar.com/investor-relations</t>
+          <t>https://www.lamar.com/about/investors</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -5763,7 +5713,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.lamar.com/careers</t>
+          <t>https://www.lamar.com/about/careers</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5918,7 +5868,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://ir.roblox.com/news-releases</t>
+          <t>https://ir.roblox.com/news</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -6043,7 +5993,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>https://www.adp.com/about-adp/privacy.aspx</t>
+          <t>https://www.adp.com/legal</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -6098,7 +6048,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://www.paychex.com/terms-of-use</t>
+          <t>https://www.paychex.com/terms</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -6139,21 +6089,6 @@
       <c r="D79" t="inlineStr">
         <is>
           <t>https://investors.paycom.com</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>https://www.paycom.com/resources/news/</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>https://paycom.com/careers</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>https://www.paycom.com/terms-of-use/</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -6686,240 +6621,227 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId397"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId398"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId620"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17580,9 +17502,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F396" t="inlineStr"/>
-      <c r="G396" t="inlineStr"/>
-      <c r="H396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -17610,9 +17529,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F397" t="inlineStr"/>
-      <c r="G397" t="inlineStr"/>
-      <c r="H397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -17640,9 +17556,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Prober Charles J. (Director) plans to sell 7,930 shares (~$420.7K) on/after 07/13/2026</t>
         </is>
       </c>
-      <c r="F398" t="inlineStr"/>
-      <c r="G398" t="inlineStr"/>
-      <c r="H398" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=BKNG,EXPE,ABNB,YOU,CHH,META,GOOG,SNAP,PINS,RDDT,APP,U,UBER,LYFT,TSLA,NFLX,SPOT,NYT,LIF,LOGI,GRMN,BBY,DIS,FOXA,UMG,WMG,LYV,SPHR,STUB,LION,OUT,LAMR,TTWO,EA,RBLX,INTU,ADP,PAYX,PAYC,PCTY,CDW run 2026-07-14T16:14Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -6853,7 +6853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H398"/>
+  <dimension ref="A1:H418"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17556,6 +17556,606 @@
           <t>[ROUTINE] Notice of proposed insider sale — Prober Charles J. (Director) plans to sell 7,930 shares (~$420.7K) on/after 07/13/2026</t>
         </is>
       </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>LOGI</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Logitech International S.A.</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1032975/000103297526000028/logi-20260713.htm</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>[UNKNOWN] Form PRE 14A</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr"/>
+      <c r="G399" t="inlineStr"/>
+      <c r="H399" t="inlineStr"/>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/blog</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr"/>
+      <c r="G400" t="inlineStr"/>
+      <c r="H400" t="inlineStr"/>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>EXPE</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Expedia Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>https://careers.expediagroup.com</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr"/>
+      <c r="G401" t="inlineStr"/>
+      <c r="H401" t="inlineStr"/>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>BKNG</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Booking Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/content/terms.html</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr"/>
+      <c r="G402" t="inlineStr"/>
+      <c r="H402" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>https://careers.airbnb.com</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr"/>
+      <c r="G403" t="inlineStr"/>
+      <c r="H403" t="inlineStr"/>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>YOU</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Clear Secure, Inc.</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1856314/000196858226000724/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Alclear Investments LLC (Officer) plans to sell 250,000 shares (~$13.80M) on/after 07/13/2026</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr"/>
+      <c r="G404" t="inlineStr"/>
+      <c r="H404" t="inlineStr"/>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>https://investor.atmeta.com</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr"/>
+      <c r="G405" t="inlineStr"/>
+      <c r="H405" t="inlineStr"/>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1326801/000192109426000726/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Olivan Javier (Officer) plans to sell 1,466 shares (~$969.2K) on/after 07/13/2026</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr"/>
+      <c r="G406" t="inlineStr"/>
+      <c r="H406" t="inlineStr"/>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>https://blog.google</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr"/>
+      <c r="G407" t="inlineStr"/>
+      <c r="H407" t="inlineStr"/>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Reddit, Inc.</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>https://redditinc.com/careers</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr"/>
+      <c r="G408" t="inlineStr"/>
+      <c r="H408" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Unity Software Inc.</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>https://careers.unity.com</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr"/>
+      <c r="G409" t="inlineStr"/>
+      <c r="H409" t="inlineStr"/>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>https://www.spotify.com/premium</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr"/>
+      <c r="G410" t="inlineStr"/>
+      <c r="H410" t="inlineStr"/>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>https://newsroom.spotify.com</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr"/>
+      <c r="G411" t="inlineStr"/>
+      <c r="H411" t="inlineStr"/>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>https://www.lifeatspotify.com</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr"/>
+      <c r="G412" t="inlineStr"/>
+      <c r="H412" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>BBY</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Best Buy Co., Inc.</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/764478/000196794026000038/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Richard M Schulze (10% Stockholder) plans to sell 900,000 shares (~$74.52M) on/after 07/13/2026</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr"/>
+      <c r="G413" t="inlineStr"/>
+      <c r="H413" t="inlineStr"/>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>https://jobs.disneycareers.com</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr"/>
+      <c r="G414" t="inlineStr"/>
+      <c r="H414" t="inlineStr"/>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>https://foxcareers.com</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr"/>
+      <c r="G415" t="inlineStr"/>
+      <c r="H415" t="inlineStr"/>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>STUB</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>StubHub Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/careers/</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr"/>
+      <c r="G416" t="inlineStr"/>
+      <c r="H416" t="inlineStr"/>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Take-Two Interactive Software, Inc.</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>https://ir.take2games.com</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr"/>
+      <c r="G417" t="inlineStr"/>
+      <c r="H417" t="inlineStr"/>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing, Inc.</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>https://mediacenter.adp.com</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr"/>
+      <c r="G418" t="inlineStr"/>
+      <c r="H418" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=BKNG,EXPE,ABNB,YOU,CHH,META,GOOG,SNAP,PINS,RDDT,APP,U,UBER,LYFT,TSLA,NFLX,SPOT,NYT,LIF,LOGI,GRMN,BBY,DIS,FOXA,UMG,WMG,LYV,SPHR,STUB,LION,OUT,LAMR,TTWO,EA,RBLX,INTU,ADP,PAYX,PAYC,PCTY,CDW run 2026-07-15T13:38Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -6853,7 +6853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H418"/>
+  <dimension ref="A1:H444"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17583,9 +17583,6 @@
           <t>[UNKNOWN] Form PRE 14A</t>
         </is>
       </c>
-      <c r="F399" t="inlineStr"/>
-      <c r="G399" t="inlineStr"/>
-      <c r="H399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -17613,9 +17610,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F400" t="inlineStr"/>
-      <c r="G400" t="inlineStr"/>
-      <c r="H400" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -17643,9 +17637,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F401" t="inlineStr"/>
-      <c r="G401" t="inlineStr"/>
-      <c r="H401" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -17673,9 +17664,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F402" t="inlineStr"/>
-      <c r="G402" t="inlineStr"/>
-      <c r="H402" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -17703,9 +17691,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F403" t="inlineStr"/>
-      <c r="G403" t="inlineStr"/>
-      <c r="H403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -17733,9 +17718,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Alclear Investments LLC (Officer) plans to sell 250,000 shares (~$13.80M) on/after 07/13/2026</t>
         </is>
       </c>
-      <c r="F404" t="inlineStr"/>
-      <c r="G404" t="inlineStr"/>
-      <c r="H404" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -17763,9 +17745,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F405" t="inlineStr"/>
-      <c r="G405" t="inlineStr"/>
-      <c r="H405" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -17793,9 +17772,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Olivan Javier (Officer) plans to sell 1,466 shares (~$969.2K) on/after 07/13/2026</t>
         </is>
       </c>
-      <c r="F406" t="inlineStr"/>
-      <c r="G406" t="inlineStr"/>
-      <c r="H406" t="inlineStr"/>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -17823,9 +17799,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F407" t="inlineStr"/>
-      <c r="G407" t="inlineStr"/>
-      <c r="H407" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -17853,9 +17826,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F408" t="inlineStr"/>
-      <c r="G408" t="inlineStr"/>
-      <c r="H408" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -17883,9 +17853,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F409" t="inlineStr"/>
-      <c r="G409" t="inlineStr"/>
-      <c r="H409" t="inlineStr"/>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -17913,9 +17880,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F410" t="inlineStr"/>
-      <c r="G410" t="inlineStr"/>
-      <c r="H410" t="inlineStr"/>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -17943,9 +17907,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F411" t="inlineStr"/>
-      <c r="G411" t="inlineStr"/>
-      <c r="H411" t="inlineStr"/>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -17973,9 +17934,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F412" t="inlineStr"/>
-      <c r="G412" t="inlineStr"/>
-      <c r="H412" t="inlineStr"/>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -18003,9 +17961,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Richard M Schulze (10% Stockholder) plans to sell 900,000 shares (~$74.52M) on/after 07/13/2026</t>
         </is>
       </c>
-      <c r="F413" t="inlineStr"/>
-      <c r="G413" t="inlineStr"/>
-      <c r="H413" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -18033,9 +17988,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F414" t="inlineStr"/>
-      <c r="G414" t="inlineStr"/>
-      <c r="H414" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -18063,9 +18015,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F415" t="inlineStr"/>
-      <c r="G415" t="inlineStr"/>
-      <c r="H415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -18093,9 +18042,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F416" t="inlineStr"/>
-      <c r="G416" t="inlineStr"/>
-      <c r="H416" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -18123,9 +18069,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F417" t="inlineStr"/>
-      <c r="G417" t="inlineStr"/>
-      <c r="H417" t="inlineStr"/>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -18153,9 +18096,786 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F418" t="inlineStr"/>
-      <c r="G418" t="inlineStr"/>
-      <c r="H418" t="inlineStr"/>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>GRMN</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Garmin Ltd.</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>https://newsroom.garmin.com</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr"/>
+      <c r="G419" t="inlineStr"/>
+      <c r="H419" t="inlineStr"/>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/blog</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr"/>
+      <c r="G420" t="inlineStr"/>
+      <c r="H420" t="inlineStr"/>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>UBER</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Uber Technologies, Inc.</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>https://investor.uber.com/governance/leadership</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr"/>
+      <c r="G421" t="inlineStr"/>
+      <c r="H421" t="inlineStr"/>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>UBER</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Uber Technologies, Inc.</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1543151/000146823326000010/xslF345X06/primarydocument.xml</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr"/>
+      <c r="G422" t="inlineStr"/>
+      <c r="H422" t="inlineStr"/>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>UBER</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Uber Technologies, Inc.</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1543151/000119069926000004/xslF345X06/primarydocument.xml</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr"/>
+      <c r="G423" t="inlineStr"/>
+      <c r="H423" t="inlineStr"/>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>UBER</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Uber Technologies, Inc.</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1543151/000109035526000006/xslF345X06/primarydocument.xml</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr"/>
+      <c r="G424" t="inlineStr"/>
+      <c r="H424" t="inlineStr"/>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>EXPE</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Expedia Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>https://careers.expediagroup.com</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr"/>
+      <c r="G425" t="inlineStr"/>
+      <c r="H425" t="inlineStr"/>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>BKNG</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Booking Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/content/terms.html</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr"/>
+      <c r="G426" t="inlineStr"/>
+      <c r="H426" t="inlineStr"/>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>https://careers.airbnb.com</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr"/>
+      <c r="G427" t="inlineStr"/>
+      <c r="H427" t="inlineStr"/>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1326801/000192109426000731/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>[UNKNOWN] Form 144/A</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr"/>
+      <c r="G428" t="inlineStr"/>
+      <c r="H428" t="inlineStr"/>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>https://blog.google</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr"/>
+      <c r="G429" t="inlineStr"/>
+      <c r="H429" t="inlineStr"/>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>PINS</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Pinterest, Inc.</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1506293/000192109426000728/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Silbermann Benjamin (Director) plans to sell 46,875 shares (~$1.04M) on/after 07/14/2026</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr"/>
+      <c r="G430" t="inlineStr"/>
+      <c r="H430" t="inlineStr"/>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Reddit, Inc.</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>https://redditinc.com/careers</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr"/>
+      <c r="G431" t="inlineStr"/>
+      <c r="H431" t="inlineStr"/>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Unity Software Inc.</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>https://careers.unity.com</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr"/>
+      <c r="G432" t="inlineStr"/>
+      <c r="H432" t="inlineStr"/>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Netflix, Inc.</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>https://about.netflix.com/newsroom</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr"/>
+      <c r="G433" t="inlineStr"/>
+      <c r="H433" t="inlineStr"/>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>https://www.spotify.com/premium</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr"/>
+      <c r="G434" t="inlineStr"/>
+      <c r="H434" t="inlineStr"/>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>https://newsroom.spotify.com</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr"/>
+      <c r="G435" t="inlineStr"/>
+      <c r="H435" t="inlineStr"/>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>https://www.lifeatspotify.com</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr"/>
+      <c r="G436" t="inlineStr"/>
+      <c r="H436" t="inlineStr"/>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>https://thewaltdisneycompany.com/news/</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr"/>
+      <c r="G437" t="inlineStr"/>
+      <c r="H437" t="inlineStr"/>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>https://jobs.disneycareers.com</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr"/>
+      <c r="G438" t="inlineStr"/>
+      <c r="H438" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>https://foxcareers.com</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr"/>
+      <c r="G439" t="inlineStr"/>
+      <c r="H439" t="inlineStr"/>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>LYV</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Live Nation Entertainment, Inc.</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1335258/000187054326000011/xslF345X06/wk-form4_1784061214.xml</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Hopmans John (EVP, M&amp;A and Strategic Finance) 6,083 shares withheld for taxes (vest event) on 2026-07-11</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr"/>
+      <c r="G440" t="inlineStr"/>
+      <c r="H440" t="inlineStr"/>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>STUB</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>StubHub Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/careers/</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr"/>
+      <c r="G441" t="inlineStr"/>
+      <c r="H441" t="inlineStr"/>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Take-Two Interactive Software, Inc.</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>https://ir.take2games.com</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr"/>
+      <c r="G442" t="inlineStr"/>
+      <c r="H442" t="inlineStr"/>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>PAYX</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Paychex, Inc.</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>https://www.paychex.com/careers</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr"/>
+      <c r="G443" t="inlineStr"/>
+      <c r="H443" t="inlineStr"/>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>PAYX</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Paychex, Inc.</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/723531/000195917326005218/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Martin Mucci (Director) plans to sell 25,000 shares (~$2.75M) on/after 07/14/2026</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr"/>
+      <c r="G444" t="inlineStr"/>
+      <c r="H444" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=BKNG,EXPE,ABNB,YOU,CHH,META,GOOG,SNAP,PINS,RDDT,APP,U,UBER,LYFT,TSLA,NFLX,SPOT,NYT,LIF,LOGI,GRMN,BBY,DIS,FOXA,UMG,WMG,LYV,SPHR,STUB,LION,OUT,LAMR,TTWO,EA,RBLX,INTU,ADP,PAYX,PAYC,PCTY,CDW run 2026-08-11T15:12Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -6853,7 +6853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H444"/>
+  <dimension ref="A1:H528"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18123,9 +18123,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F419" t="inlineStr"/>
-      <c r="G419" t="inlineStr"/>
-      <c r="H419" t="inlineStr"/>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -18153,9 +18150,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F420" t="inlineStr"/>
-      <c r="G420" t="inlineStr"/>
-      <c r="H420" t="inlineStr"/>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -18183,9 +18177,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F421" t="inlineStr"/>
-      <c r="G421" t="inlineStr"/>
-      <c r="H421" t="inlineStr"/>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
@@ -18213,9 +18204,6 @@
           <t>[ROUTINE] Insider trade</t>
         </is>
       </c>
-      <c r="F422" t="inlineStr"/>
-      <c r="G422" t="inlineStr"/>
-      <c r="H422" t="inlineStr"/>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -18243,9 +18231,6 @@
           <t>[ROUTINE] Insider trade</t>
         </is>
       </c>
-      <c r="F423" t="inlineStr"/>
-      <c r="G423" t="inlineStr"/>
-      <c r="H423" t="inlineStr"/>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -18273,9 +18258,6 @@
           <t>[ROUTINE] Insider trade</t>
         </is>
       </c>
-      <c r="F424" t="inlineStr"/>
-      <c r="G424" t="inlineStr"/>
-      <c r="H424" t="inlineStr"/>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -18303,9 +18285,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F425" t="inlineStr"/>
-      <c r="G425" t="inlineStr"/>
-      <c r="H425" t="inlineStr"/>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -18333,9 +18312,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F426" t="inlineStr"/>
-      <c r="G426" t="inlineStr"/>
-      <c r="H426" t="inlineStr"/>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -18363,9 +18339,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F427" t="inlineStr"/>
-      <c r="G427" t="inlineStr"/>
-      <c r="H427" t="inlineStr"/>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -18393,9 +18366,6 @@
           <t>[UNKNOWN] Form 144/A</t>
         </is>
       </c>
-      <c r="F428" t="inlineStr"/>
-      <c r="G428" t="inlineStr"/>
-      <c r="H428" t="inlineStr"/>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -18423,9 +18393,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F429" t="inlineStr"/>
-      <c r="G429" t="inlineStr"/>
-      <c r="H429" t="inlineStr"/>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -18453,9 +18420,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Silbermann Benjamin (Director) plans to sell 46,875 shares (~$1.04M) on/after 07/14/2026</t>
         </is>
       </c>
-      <c r="F430" t="inlineStr"/>
-      <c r="G430" t="inlineStr"/>
-      <c r="H430" t="inlineStr"/>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -18483,9 +18447,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F431" t="inlineStr"/>
-      <c r="G431" t="inlineStr"/>
-      <c r="H431" t="inlineStr"/>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
@@ -18513,9 +18474,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F432" t="inlineStr"/>
-      <c r="G432" t="inlineStr"/>
-      <c r="H432" t="inlineStr"/>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -18543,9 +18501,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F433" t="inlineStr"/>
-      <c r="G433" t="inlineStr"/>
-      <c r="H433" t="inlineStr"/>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -18573,9 +18528,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F434" t="inlineStr"/>
-      <c r="G434" t="inlineStr"/>
-      <c r="H434" t="inlineStr"/>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -18603,9 +18555,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F435" t="inlineStr"/>
-      <c r="G435" t="inlineStr"/>
-      <c r="H435" t="inlineStr"/>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -18633,9 +18582,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F436" t="inlineStr"/>
-      <c r="G436" t="inlineStr"/>
-      <c r="H436" t="inlineStr"/>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -18663,9 +18609,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F437" t="inlineStr"/>
-      <c r="G437" t="inlineStr"/>
-      <c r="H437" t="inlineStr"/>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -18693,9 +18636,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F438" t="inlineStr"/>
-      <c r="G438" t="inlineStr"/>
-      <c r="H438" t="inlineStr"/>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
@@ -18723,9 +18663,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F439" t="inlineStr"/>
-      <c r="G439" t="inlineStr"/>
-      <c r="H439" t="inlineStr"/>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -18753,9 +18690,6 @@
           <t>[ROUTINE] Insider trade — Hopmans John (EVP, M&amp;A and Strategic Finance) 6,083 shares withheld for taxes (vest event) on 2026-07-11</t>
         </is>
       </c>
-      <c r="F440" t="inlineStr"/>
-      <c r="G440" t="inlineStr"/>
-      <c r="H440" t="inlineStr"/>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
@@ -18783,9 +18717,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F441" t="inlineStr"/>
-      <c r="G441" t="inlineStr"/>
-      <c r="H441" t="inlineStr"/>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
@@ -18813,9 +18744,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F442" t="inlineStr"/>
-      <c r="G442" t="inlineStr"/>
-      <c r="H442" t="inlineStr"/>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -18843,9 +18771,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F443" t="inlineStr"/>
-      <c r="G443" t="inlineStr"/>
-      <c r="H443" t="inlineStr"/>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
@@ -18873,9 +18798,2526 @@
           <t>[ROUTINE] Notice of proposed insider sale — Martin Mucci (Director) plans to sell 25,000 shares (~$2.75M) on/after 07/14/2026</t>
         </is>
       </c>
-      <c r="F444" t="inlineStr"/>
-      <c r="G444" t="inlineStr"/>
-      <c r="H444" t="inlineStr"/>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>LOGI</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Logitech International S.A.</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>https://www.logitech.com/press</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr"/>
+      <c r="G445" t="inlineStr"/>
+      <c r="H445" t="inlineStr"/>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>LOGI</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Logitech International S.A.</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>https://ir.logitech.com</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr"/>
+      <c r="G446" t="inlineStr"/>
+      <c r="H446" t="inlineStr"/>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>GRMN</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Garmin Ltd.</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>https://newsroom.garmin.com</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr"/>
+      <c r="G447" t="inlineStr"/>
+      <c r="H447" t="inlineStr"/>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>GRMN</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Garmin Ltd.</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>https://www.garmin.com/en-US/company/investors/</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr"/>
+      <c r="G448" t="inlineStr"/>
+      <c r="H448" t="inlineStr"/>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/blog</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr"/>
+      <c r="G449" t="inlineStr"/>
+      <c r="H449" t="inlineStr"/>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>https://investor.lyft.com</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr"/>
+      <c r="G450" t="inlineStr"/>
+      <c r="H450" t="inlineStr"/>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>UBER</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Uber Technologies, Inc.</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>https://investor.uber.com/governance/leadership</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr"/>
+      <c r="G451" t="inlineStr"/>
+      <c r="H451" t="inlineStr"/>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>EXPE</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Expedia Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>https://www.expediagroup.com/media</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr"/>
+      <c r="G452" t="inlineStr"/>
+      <c r="H452" t="inlineStr"/>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>EXPE</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Expedia Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>https://careers.expediagroup.com</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr"/>
+      <c r="G453" t="inlineStr"/>
+      <c r="H453" t="inlineStr"/>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>BKNG</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Booking Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/content/terms.html</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr"/>
+      <c r="G454" t="inlineStr"/>
+      <c r="H454" t="inlineStr"/>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>BKNG</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Booking Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>https://www.bookingholdings.com/careers</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr"/>
+      <c r="G455" t="inlineStr"/>
+      <c r="H455" t="inlineStr"/>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>https://careers.airbnb.com</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr"/>
+      <c r="G456" t="inlineStr"/>
+      <c r="H456" t="inlineStr"/>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>YOU</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Clear Secure, Inc.</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>https://www.clearme.com/terms</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr"/>
+      <c r="G457" t="inlineStr"/>
+      <c r="H457" t="inlineStr"/>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>YOU</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Clear Secure, Inc.</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>https://ir.clearme.com/news-events</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr"/>
+      <c r="G458" t="inlineStr"/>
+      <c r="H458" t="inlineStr"/>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>YOU</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Clear Secure, Inc.</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>https://ir.clearme.com</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr"/>
+      <c r="G459" t="inlineStr"/>
+      <c r="H459" t="inlineStr"/>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>YOU</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Clear Secure, Inc.</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>https://www.clearme.com/careers</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr"/>
+      <c r="G460" t="inlineStr"/>
+      <c r="H460" t="inlineStr"/>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>YOU</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Clear Secure, Inc.</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1856314/000196858226000811/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Warrior Mensch Foundation (Affiliate) plans to sell 196,656 shares (~$10.09M) on/after 08/10/2026</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr"/>
+      <c r="G461" t="inlineStr"/>
+      <c r="H461" t="inlineStr"/>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>CHH</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Choice Hotels International, Inc.</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>https://media.choicehotels.com</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr"/>
+      <c r="G462" t="inlineStr"/>
+      <c r="H462" t="inlineStr"/>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>https://investor.atmeta.com</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr"/>
+      <c r="G463" t="inlineStr"/>
+      <c r="H463" t="inlineStr"/>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1326801/000192109426000824/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Olivan Javier (Officer) plans to sell 1,692 shares (~$1.02M) on/after 08/10/2026</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr"/>
+      <c r="G464" t="inlineStr"/>
+      <c r="H464" t="inlineStr"/>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>https://policies.google.com/terms</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr"/>
+      <c r="G465" t="inlineStr"/>
+      <c r="H465" t="inlineStr"/>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>https://blog.google</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr"/>
+      <c r="G466" t="inlineStr"/>
+      <c r="H466" t="inlineStr"/>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1652044/000119312526342390/d171253d8k.htm</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Material event disclosure</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr"/>
+      <c r="G467" t="inlineStr"/>
+      <c r="H467" t="inlineStr"/>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>https://snap.com/en-US/terms</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr"/>
+      <c r="G468" t="inlineStr"/>
+      <c r="H468" t="inlineStr"/>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>https://investor.snap.com/governance/leadership</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr"/>
+      <c r="G469" t="inlineStr"/>
+      <c r="H469" t="inlineStr"/>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>https://newsroom.snap.com</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr"/>
+      <c r="G470" t="inlineStr"/>
+      <c r="H470" t="inlineStr"/>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>https://investor.snap.com</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr"/>
+      <c r="G471" t="inlineStr"/>
+      <c r="H471" t="inlineStr"/>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>PINS</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Pinterest, Inc.</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>https://www.pinterestcareers.com</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr"/>
+      <c r="G472" t="inlineStr"/>
+      <c r="H472" t="inlineStr"/>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>PINS</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Pinterest, Inc.</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1506293/000088698226000325/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Update to 5%+ passive owner disclosure</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr"/>
+      <c r="G473" t="inlineStr"/>
+      <c r="H473" t="inlineStr"/>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Reddit, Inc.</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>https://www.redditinc.com/policies/user-agreement</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr"/>
+      <c r="G474" t="inlineStr"/>
+      <c r="H474" t="inlineStr"/>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Reddit, Inc.</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>https://redditinc.com/press</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr"/>
+      <c r="G475" t="inlineStr"/>
+      <c r="H475" t="inlineStr"/>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Reddit, Inc.</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>https://redditinc.com/careers</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr"/>
+      <c r="G476" t="inlineStr"/>
+      <c r="H476" t="inlineStr"/>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>AppLovin Corporation</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>https://www.applovin.com/legal/</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr"/>
+      <c r="G477" t="inlineStr"/>
+      <c r="H477" t="inlineStr"/>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>AppLovin Corporation</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>https://www.applovin.com/blog/</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr"/>
+      <c r="G478" t="inlineStr"/>
+      <c r="H478" t="inlineStr"/>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>AppLovin Corporation</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>https://www.applovin.com/careers/</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr"/>
+      <c r="G479" t="inlineStr"/>
+      <c r="H479" t="inlineStr"/>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Unity Software Inc.</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>https://careers.unity.com</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr"/>
+      <c r="G480" t="inlineStr"/>
+      <c r="H480" t="inlineStr"/>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Unity Software Inc.</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1810806/000122228726000017/xslF345X06/wk-form4_1786405422.xml</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Roelof Botha (Director) other: 461,106 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr"/>
+      <c r="G481" t="inlineStr"/>
+      <c r="H481" t="inlineStr"/>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Netflix, Inc.</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>https://about.netflix.com/newsroom</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr"/>
+      <c r="G482" t="inlineStr"/>
+      <c r="H482" t="inlineStr"/>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Netflix, Inc.</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1065280/000106528026000249/xslF345X06/wk-form4_1786394054.xml</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Neumann Spencer Adam (Chief Financial Officer) sold 9,248 shares @ $75.79 ($700.9K) on 2026-08-10</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr"/>
+      <c r="G483" t="inlineStr"/>
+      <c r="H483" t="inlineStr"/>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Netflix, Inc.</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1065280/000195004726007858/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Neumann Spencer (Officer) plans to sell 9,248 shares (~$700.9K) on/after 08/10/2026</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr"/>
+      <c r="G484" t="inlineStr"/>
+      <c r="H484" t="inlineStr"/>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>https://www.spotify.com/premium</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr"/>
+      <c r="G485" t="inlineStr"/>
+      <c r="H485" t="inlineStr"/>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>https://newsroom.spotify.com</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr"/>
+      <c r="G486" t="inlineStr"/>
+      <c r="H486" t="inlineStr"/>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>https://investors.spotify.com</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr"/>
+      <c r="G487" t="inlineStr"/>
+      <c r="H487" t="inlineStr"/>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>https://www.lifeatspotify.com</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr"/>
+      <c r="G488" t="inlineStr"/>
+      <c r="H488" t="inlineStr"/>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>NYT</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>The New York Times Company</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>https://help.nytimes.com/hc/en-us/articles/115014893428</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr"/>
+      <c r="G489" t="inlineStr"/>
+      <c r="H489" t="inlineStr"/>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>LIF</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>LIF (verify ticker)</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1581760/000195917326005857/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Morin Brit (Director) plans to sell 15,582 shares (~$1.01M) on/after 08/10/2026</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr"/>
+      <c r="G490" t="inlineStr"/>
+      <c r="H490" t="inlineStr"/>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>LIF</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>LIF (verify ticker)</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1581760/000158176026000142/lifx-20260810.htm</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Material event disclosure</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr"/>
+      <c r="G491" t="inlineStr"/>
+      <c r="H491" t="inlineStr"/>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>LIF</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>LIF (verify ticker)</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1581760/000158176026000141/lifx-20260630.htm</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Quarterly report</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr"/>
+      <c r="G492" t="inlineStr"/>
+      <c r="H492" t="inlineStr"/>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>BBY</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Best Buy Co., Inc.</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>https://www.bestbuy.com/site/help-topics/terms-and-conditions/pcmcat204400050067.c</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr"/>
+      <c r="G493" t="inlineStr"/>
+      <c r="H493" t="inlineStr"/>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>https://www.disneyplus.com/welcome</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr"/>
+      <c r="G494" t="inlineStr"/>
+      <c r="H494" t="inlineStr"/>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>https://thewaltdisneycompany.com/news/</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr"/>
+      <c r="G495" t="inlineStr"/>
+      <c r="H495" t="inlineStr"/>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>https://thewaltdisneycompany.com/investor-relations/</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr"/>
+      <c r="G496" t="inlineStr"/>
+      <c r="H496" t="inlineStr"/>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>https://jobs.disneycareers.com</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr"/>
+      <c r="G497" t="inlineStr"/>
+      <c r="H497" t="inlineStr"/>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>https://investor.foxcorporation.com</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr"/>
+      <c r="G498" t="inlineStr"/>
+      <c r="H498" t="inlineStr"/>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>https://foxcareers.com</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr"/>
+      <c r="G499" t="inlineStr"/>
+      <c r="H499" t="inlineStr"/>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1754301/000162828026055398/xslF345X06/wk-form4_1786398279.xml</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr"/>
+      <c r="G500" t="inlineStr"/>
+      <c r="H500" t="inlineStr"/>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1754301/000162828026055396/xslF345X06/wk-form4_1786398195.xml</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr"/>
+      <c r="G501" t="inlineStr"/>
+      <c r="H501" t="inlineStr"/>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1754301/000162828026055392/xslF345X06/wk-form4_1786398055.xml</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr"/>
+      <c r="G502" t="inlineStr"/>
+      <c r="H502" t="inlineStr"/>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1754301/000162828026055391/xslF345X06/wk-form4_1786398011.xml</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr"/>
+      <c r="G503" t="inlineStr"/>
+      <c r="H503" t="inlineStr"/>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1754301/000119312526341282/d140335ds3asr.htm</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>[UNKNOWN] Form S-3ASR</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr"/>
+      <c r="G504" t="inlineStr"/>
+      <c r="H504" t="inlineStr"/>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1754301/000119312526341217/d133486d425.htm</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>[UNKNOWN] Form 425</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr"/>
+      <c r="G505" t="inlineStr"/>
+      <c r="H505" t="inlineStr"/>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1754301/000119312526341200/d133486d8ka.htm</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>[UNKNOWN] Form 8-K/A</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr"/>
+      <c r="G506" t="inlineStr"/>
+      <c r="H506" t="inlineStr"/>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>UMG</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Universal Music Group N.V.</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>https://www.universalmusic.com/news/</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr"/>
+      <c r="G507" t="inlineStr"/>
+      <c r="H507" t="inlineStr"/>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>UMG</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Universal Music Group N.V.</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>https://www.universalmusic.com/careers/</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr"/>
+      <c r="G508" t="inlineStr"/>
+      <c r="H508" t="inlineStr"/>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>WMG</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Warner Music Group Corp.</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>https://www.wmg.com/news/</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr"/>
+      <c r="G509" t="inlineStr"/>
+      <c r="H509" t="inlineStr"/>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>WMG</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Warner Music Group Corp.</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>https://investors.wmg.com</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr"/>
+      <c r="G510" t="inlineStr"/>
+      <c r="H510" t="inlineStr"/>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>LYV</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Live Nation Entertainment, Inc.</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>https://investors.livenationentertainment.com</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr"/>
+      <c r="G511" t="inlineStr"/>
+      <c r="H511" t="inlineStr"/>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>LYV</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Live Nation Entertainment, Inc.</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>https://www.livenationentertainment.com/careers</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr"/>
+      <c r="G512" t="inlineStr"/>
+      <c r="H512" t="inlineStr"/>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>STUB</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>StubHub Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/careers/</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr"/>
+      <c r="G513" t="inlineStr"/>
+      <c r="H513" t="inlineStr"/>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>OUTFRONT Media Inc.</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>https://investor.outfrontmedia.com</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr"/>
+      <c r="G514" t="inlineStr"/>
+      <c r="H514" t="inlineStr"/>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Take-Two Interactive Software, Inc.</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>https://ir.take2games.com</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr"/>
+      <c r="G515" t="inlineStr"/>
+      <c r="H515" t="inlineStr"/>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Take-Two Interactive Software, Inc.</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/946581/000195824426000496/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — H. Strauss Zelnick (Officer) plans to sell 40,000 shares (~$10.14M) on/after 08/10/2026</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr"/>
+      <c r="G516" t="inlineStr"/>
+      <c r="H516" t="inlineStr"/>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Electronic Arts Inc.</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>https://www.ea.com/news</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr"/>
+      <c r="G517" t="inlineStr"/>
+      <c r="H517" t="inlineStr"/>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Electronic Arts Inc.</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>https://ir.ea.com</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr"/>
+      <c r="G518" t="inlineStr"/>
+      <c r="H518" t="inlineStr"/>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Electronic Arts Inc.</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>https://ea.com/careers</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr"/>
+      <c r="G519" t="inlineStr"/>
+      <c r="H519" t="inlineStr"/>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Intuit Inc.</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>https://quickbooks.intuit.com/pricing/</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr"/>
+      <c r="G520" t="inlineStr"/>
+      <c r="H520" t="inlineStr"/>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Intuit Inc.</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>https://investors.intuit.com</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr"/>
+      <c r="G521" t="inlineStr"/>
+      <c r="H521" t="inlineStr"/>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing, Inc.</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>https://mediacenter.adp.com</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr"/>
+      <c r="G522" t="inlineStr"/>
+      <c r="H522" t="inlineStr"/>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing, Inc.</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>https://investors.adp.com</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr"/>
+      <c r="G523" t="inlineStr"/>
+      <c r="H523" t="inlineStr"/>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>PAYX</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Paychex, Inc.</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>https://www.paychex.com/newsroom</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr"/>
+      <c r="G524" t="inlineStr"/>
+      <c r="H524" t="inlineStr"/>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>PAYX</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Paychex, Inc.</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>https://investor.paychex.com</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr"/>
+      <c r="G525" t="inlineStr"/>
+      <c r="H525" t="inlineStr"/>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>PAYC</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Paycom Software, Inc.</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>https://investors.paycom.com</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr"/>
+      <c r="G526" t="inlineStr"/>
+      <c r="H526" t="inlineStr"/>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>PCTY</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Paylocity Holding Corporation</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1591698/000159787026000002/xslF345X06/wk-form4_1786392623.xml</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Sarowitz Steven I (Director) sold 11,136 shares @ $150.81 ($1.68M) on 2026-08-06</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr"/>
+      <c r="G527" t="inlineStr"/>
+      <c r="H527" t="inlineStr"/>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>CDW Corporation</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>https://investor.cdw.com</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr"/>
+      <c r="G528" t="inlineStr"/>
+      <c r="H528" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=BKNG,EXPE,ABNB,YOU,CHH,META,GOOG,SNAP,PINS,RDDT,APP,U,UBER,LYFT,TSLA,NFLX,SPOT,NYT,LIF,LOGI,GRMN,BBY,DIS,FOXA,UMG,WMG,LYV,SPHR,STUB,LION,OUT,LAMR,TTWO,EA,RBLX,INTU,ADP,PAYX,PAYC,PCTY,CDW run 2026-08-12T13:15Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -6853,7 +6853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H528"/>
+  <dimension ref="A1:H575"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18825,9 +18825,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F445" t="inlineStr"/>
-      <c r="G445" t="inlineStr"/>
-      <c r="H445" t="inlineStr"/>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -18855,9 +18852,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F446" t="inlineStr"/>
-      <c r="G446" t="inlineStr"/>
-      <c r="H446" t="inlineStr"/>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
@@ -18885,9 +18879,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F447" t="inlineStr"/>
-      <c r="G447" t="inlineStr"/>
-      <c r="H447" t="inlineStr"/>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
@@ -18915,9 +18906,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F448" t="inlineStr"/>
-      <c r="G448" t="inlineStr"/>
-      <c r="H448" t="inlineStr"/>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
@@ -18945,9 +18933,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F449" t="inlineStr"/>
-      <c r="G449" t="inlineStr"/>
-      <c r="H449" t="inlineStr"/>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
@@ -18975,9 +18960,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F450" t="inlineStr"/>
-      <c r="G450" t="inlineStr"/>
-      <c r="H450" t="inlineStr"/>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
@@ -19005,9 +18987,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F451" t="inlineStr"/>
-      <c r="G451" t="inlineStr"/>
-      <c r="H451" t="inlineStr"/>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -19035,9 +19014,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F452" t="inlineStr"/>
-      <c r="G452" t="inlineStr"/>
-      <c r="H452" t="inlineStr"/>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
@@ -19065,9 +19041,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F453" t="inlineStr"/>
-      <c r="G453" t="inlineStr"/>
-      <c r="H453" t="inlineStr"/>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
@@ -19095,9 +19068,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F454" t="inlineStr"/>
-      <c r="G454" t="inlineStr"/>
-      <c r="H454" t="inlineStr"/>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -19125,9 +19095,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F455" t="inlineStr"/>
-      <c r="G455" t="inlineStr"/>
-      <c r="H455" t="inlineStr"/>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -19155,9 +19122,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F456" t="inlineStr"/>
-      <c r="G456" t="inlineStr"/>
-      <c r="H456" t="inlineStr"/>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
@@ -19185,9 +19149,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F457" t="inlineStr"/>
-      <c r="G457" t="inlineStr"/>
-      <c r="H457" t="inlineStr"/>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
@@ -19215,9 +19176,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F458" t="inlineStr"/>
-      <c r="G458" t="inlineStr"/>
-      <c r="H458" t="inlineStr"/>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
@@ -19245,9 +19203,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F459" t="inlineStr"/>
-      <c r="G459" t="inlineStr"/>
-      <c r="H459" t="inlineStr"/>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -19275,9 +19230,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F460" t="inlineStr"/>
-      <c r="G460" t="inlineStr"/>
-      <c r="H460" t="inlineStr"/>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -19305,9 +19257,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Warrior Mensch Foundation (Affiliate) plans to sell 196,656 shares (~$10.09M) on/after 08/10/2026</t>
         </is>
       </c>
-      <c r="F461" t="inlineStr"/>
-      <c r="G461" t="inlineStr"/>
-      <c r="H461" t="inlineStr"/>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
@@ -19335,9 +19284,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F462" t="inlineStr"/>
-      <c r="G462" t="inlineStr"/>
-      <c r="H462" t="inlineStr"/>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
@@ -19365,9 +19311,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F463" t="inlineStr"/>
-      <c r="G463" t="inlineStr"/>
-      <c r="H463" t="inlineStr"/>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
@@ -19395,9 +19338,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Olivan Javier (Officer) plans to sell 1,692 shares (~$1.02M) on/after 08/10/2026</t>
         </is>
       </c>
-      <c r="F464" t="inlineStr"/>
-      <c r="G464" t="inlineStr"/>
-      <c r="H464" t="inlineStr"/>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -19425,9 +19365,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F465" t="inlineStr"/>
-      <c r="G465" t="inlineStr"/>
-      <c r="H465" t="inlineStr"/>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
@@ -19455,9 +19392,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F466" t="inlineStr"/>
-      <c r="G466" t="inlineStr"/>
-      <c r="H466" t="inlineStr"/>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
@@ -19485,9 +19419,6 @@
           <t>[MATERIAL] Material event disclosure</t>
         </is>
       </c>
-      <c r="F467" t="inlineStr"/>
-      <c r="G467" t="inlineStr"/>
-      <c r="H467" t="inlineStr"/>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
@@ -19515,9 +19446,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F468" t="inlineStr"/>
-      <c r="G468" t="inlineStr"/>
-      <c r="H468" t="inlineStr"/>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
@@ -19545,9 +19473,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F469" t="inlineStr"/>
-      <c r="G469" t="inlineStr"/>
-      <c r="H469" t="inlineStr"/>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
@@ -19575,9 +19500,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F470" t="inlineStr"/>
-      <c r="G470" t="inlineStr"/>
-      <c r="H470" t="inlineStr"/>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
@@ -19605,9 +19527,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F471" t="inlineStr"/>
-      <c r="G471" t="inlineStr"/>
-      <c r="H471" t="inlineStr"/>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -19635,9 +19554,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F472" t="inlineStr"/>
-      <c r="G472" t="inlineStr"/>
-      <c r="H472" t="inlineStr"/>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
@@ -19665,9 +19581,6 @@
           <t>[MATERIAL] Update to 5%+ passive owner disclosure</t>
         </is>
       </c>
-      <c r="F473" t="inlineStr"/>
-      <c r="G473" t="inlineStr"/>
-      <c r="H473" t="inlineStr"/>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
@@ -19695,9 +19608,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F474" t="inlineStr"/>
-      <c r="G474" t="inlineStr"/>
-      <c r="H474" t="inlineStr"/>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
@@ -19725,9 +19635,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F475" t="inlineStr"/>
-      <c r="G475" t="inlineStr"/>
-      <c r="H475" t="inlineStr"/>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
@@ -19755,9 +19662,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F476" t="inlineStr"/>
-      <c r="G476" t="inlineStr"/>
-      <c r="H476" t="inlineStr"/>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
@@ -19785,9 +19689,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F477" t="inlineStr"/>
-      <c r="G477" t="inlineStr"/>
-      <c r="H477" t="inlineStr"/>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
@@ -19815,9 +19716,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F478" t="inlineStr"/>
-      <c r="G478" t="inlineStr"/>
-      <c r="H478" t="inlineStr"/>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
@@ -19845,9 +19743,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F479" t="inlineStr"/>
-      <c r="G479" t="inlineStr"/>
-      <c r="H479" t="inlineStr"/>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -19875,9 +19770,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F480" t="inlineStr"/>
-      <c r="G480" t="inlineStr"/>
-      <c r="H480" t="inlineStr"/>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
@@ -19905,9 +19797,6 @@
           <t>[ROUTINE] Insider trade — Roelof Botha (Director) other: 461,106 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F481" t="inlineStr"/>
-      <c r="G481" t="inlineStr"/>
-      <c r="H481" t="inlineStr"/>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
@@ -19935,9 +19824,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F482" t="inlineStr"/>
-      <c r="G482" t="inlineStr"/>
-      <c r="H482" t="inlineStr"/>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
@@ -19965,9 +19851,6 @@
           <t>[ROUTINE] Insider trade — Neumann Spencer Adam (Chief Financial Officer) sold 9,248 shares @ $75.79 ($700.9K) on 2026-08-10</t>
         </is>
       </c>
-      <c r="F483" t="inlineStr"/>
-      <c r="G483" t="inlineStr"/>
-      <c r="H483" t="inlineStr"/>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
@@ -19995,9 +19878,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Neumann Spencer (Officer) plans to sell 9,248 shares (~$700.9K) on/after 08/10/2026</t>
         </is>
       </c>
-      <c r="F484" t="inlineStr"/>
-      <c r="G484" t="inlineStr"/>
-      <c r="H484" t="inlineStr"/>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
@@ -20025,9 +19905,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F485" t="inlineStr"/>
-      <c r="G485" t="inlineStr"/>
-      <c r="H485" t="inlineStr"/>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
@@ -20055,9 +19932,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F486" t="inlineStr"/>
-      <c r="G486" t="inlineStr"/>
-      <c r="H486" t="inlineStr"/>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
@@ -20085,9 +19959,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F487" t="inlineStr"/>
-      <c r="G487" t="inlineStr"/>
-      <c r="H487" t="inlineStr"/>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
@@ -20115,9 +19986,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F488" t="inlineStr"/>
-      <c r="G488" t="inlineStr"/>
-      <c r="H488" t="inlineStr"/>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
@@ -20145,9 +20013,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F489" t="inlineStr"/>
-      <c r="G489" t="inlineStr"/>
-      <c r="H489" t="inlineStr"/>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
@@ -20175,9 +20040,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Morin Brit (Director) plans to sell 15,582 shares (~$1.01M) on/after 08/10/2026</t>
         </is>
       </c>
-      <c r="F490" t="inlineStr"/>
-      <c r="G490" t="inlineStr"/>
-      <c r="H490" t="inlineStr"/>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
@@ -20205,9 +20067,6 @@
           <t>[MATERIAL] Material event disclosure</t>
         </is>
       </c>
-      <c r="F491" t="inlineStr"/>
-      <c r="G491" t="inlineStr"/>
-      <c r="H491" t="inlineStr"/>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
@@ -20235,9 +20094,6 @@
           <t>[MATERIAL] Quarterly report</t>
         </is>
       </c>
-      <c r="F492" t="inlineStr"/>
-      <c r="G492" t="inlineStr"/>
-      <c r="H492" t="inlineStr"/>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -20265,9 +20121,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F493" t="inlineStr"/>
-      <c r="G493" t="inlineStr"/>
-      <c r="H493" t="inlineStr"/>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
@@ -20295,9 +20148,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F494" t="inlineStr"/>
-      <c r="G494" t="inlineStr"/>
-      <c r="H494" t="inlineStr"/>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -20325,9 +20175,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F495" t="inlineStr"/>
-      <c r="G495" t="inlineStr"/>
-      <c r="H495" t="inlineStr"/>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
@@ -20355,9 +20202,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F496" t="inlineStr"/>
-      <c r="G496" t="inlineStr"/>
-      <c r="H496" t="inlineStr"/>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
@@ -20385,9 +20229,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F497" t="inlineStr"/>
-      <c r="G497" t="inlineStr"/>
-      <c r="H497" t="inlineStr"/>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -20415,9 +20256,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F498" t="inlineStr"/>
-      <c r="G498" t="inlineStr"/>
-      <c r="H498" t="inlineStr"/>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -20445,9 +20283,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F499" t="inlineStr"/>
-      <c r="G499" t="inlineStr"/>
-      <c r="H499" t="inlineStr"/>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
@@ -20475,9 +20310,6 @@
           <t>[ROUTINE] Insider trade</t>
         </is>
       </c>
-      <c r="F500" t="inlineStr"/>
-      <c r="G500" t="inlineStr"/>
-      <c r="H500" t="inlineStr"/>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
@@ -20505,9 +20337,6 @@
           <t>[ROUTINE] Insider trade</t>
         </is>
       </c>
-      <c r="F501" t="inlineStr"/>
-      <c r="G501" t="inlineStr"/>
-      <c r="H501" t="inlineStr"/>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
@@ -20535,9 +20364,6 @@
           <t>[ROUTINE] Insider trade</t>
         </is>
       </c>
-      <c r="F502" t="inlineStr"/>
-      <c r="G502" t="inlineStr"/>
-      <c r="H502" t="inlineStr"/>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
@@ -20565,9 +20391,6 @@
           <t>[ROUTINE] Insider trade</t>
         </is>
       </c>
-      <c r="F503" t="inlineStr"/>
-      <c r="G503" t="inlineStr"/>
-      <c r="H503" t="inlineStr"/>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
@@ -20595,9 +20418,6 @@
           <t>[UNKNOWN] Form S-3ASR</t>
         </is>
       </c>
-      <c r="F504" t="inlineStr"/>
-      <c r="G504" t="inlineStr"/>
-      <c r="H504" t="inlineStr"/>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
@@ -20625,9 +20445,6 @@
           <t>[UNKNOWN] Form 425</t>
         </is>
       </c>
-      <c r="F505" t="inlineStr"/>
-      <c r="G505" t="inlineStr"/>
-      <c r="H505" t="inlineStr"/>
     </row>
     <row r="506">
       <c r="A506" t="inlineStr">
@@ -20655,9 +20472,6 @@
           <t>[UNKNOWN] Form 8-K/A</t>
         </is>
       </c>
-      <c r="F506" t="inlineStr"/>
-      <c r="G506" t="inlineStr"/>
-      <c r="H506" t="inlineStr"/>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
@@ -20685,9 +20499,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F507" t="inlineStr"/>
-      <c r="G507" t="inlineStr"/>
-      <c r="H507" t="inlineStr"/>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
@@ -20715,9 +20526,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F508" t="inlineStr"/>
-      <c r="G508" t="inlineStr"/>
-      <c r="H508" t="inlineStr"/>
     </row>
     <row r="509">
       <c r="A509" t="inlineStr">
@@ -20745,9 +20553,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F509" t="inlineStr"/>
-      <c r="G509" t="inlineStr"/>
-      <c r="H509" t="inlineStr"/>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
@@ -20775,9 +20580,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F510" t="inlineStr"/>
-      <c r="G510" t="inlineStr"/>
-      <c r="H510" t="inlineStr"/>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
@@ -20805,9 +20607,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F511" t="inlineStr"/>
-      <c r="G511" t="inlineStr"/>
-      <c r="H511" t="inlineStr"/>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
@@ -20835,9 +20634,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F512" t="inlineStr"/>
-      <c r="G512" t="inlineStr"/>
-      <c r="H512" t="inlineStr"/>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
@@ -20865,9 +20661,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F513" t="inlineStr"/>
-      <c r="G513" t="inlineStr"/>
-      <c r="H513" t="inlineStr"/>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
@@ -20895,9 +20688,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F514" t="inlineStr"/>
-      <c r="G514" t="inlineStr"/>
-      <c r="H514" t="inlineStr"/>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
@@ -20925,9 +20715,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F515" t="inlineStr"/>
-      <c r="G515" t="inlineStr"/>
-      <c r="H515" t="inlineStr"/>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
@@ -20955,9 +20742,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — H. Strauss Zelnick (Officer) plans to sell 40,000 shares (~$10.14M) on/after 08/10/2026</t>
         </is>
       </c>
-      <c r="F516" t="inlineStr"/>
-      <c r="G516" t="inlineStr"/>
-      <c r="H516" t="inlineStr"/>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
@@ -20985,9 +20769,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F517" t="inlineStr"/>
-      <c r="G517" t="inlineStr"/>
-      <c r="H517" t="inlineStr"/>
     </row>
     <row r="518">
       <c r="A518" t="inlineStr">
@@ -21015,9 +20796,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F518" t="inlineStr"/>
-      <c r="G518" t="inlineStr"/>
-      <c r="H518" t="inlineStr"/>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
@@ -21045,9 +20823,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F519" t="inlineStr"/>
-      <c r="G519" t="inlineStr"/>
-      <c r="H519" t="inlineStr"/>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
@@ -21075,9 +20850,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F520" t="inlineStr"/>
-      <c r="G520" t="inlineStr"/>
-      <c r="H520" t="inlineStr"/>
     </row>
     <row r="521">
       <c r="A521" t="inlineStr">
@@ -21105,9 +20877,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F521" t="inlineStr"/>
-      <c r="G521" t="inlineStr"/>
-      <c r="H521" t="inlineStr"/>
     </row>
     <row r="522">
       <c r="A522" t="inlineStr">
@@ -21135,9 +20904,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F522" t="inlineStr"/>
-      <c r="G522" t="inlineStr"/>
-      <c r="H522" t="inlineStr"/>
     </row>
     <row r="523">
       <c r="A523" t="inlineStr">
@@ -21165,9 +20931,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F523" t="inlineStr"/>
-      <c r="G523" t="inlineStr"/>
-      <c r="H523" t="inlineStr"/>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
@@ -21195,9 +20958,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F524" t="inlineStr"/>
-      <c r="G524" t="inlineStr"/>
-      <c r="H524" t="inlineStr"/>
     </row>
     <row r="525">
       <c r="A525" t="inlineStr">
@@ -21225,9 +20985,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F525" t="inlineStr"/>
-      <c r="G525" t="inlineStr"/>
-      <c r="H525" t="inlineStr"/>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
@@ -21255,9 +21012,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F526" t="inlineStr"/>
-      <c r="G526" t="inlineStr"/>
-      <c r="H526" t="inlineStr"/>
     </row>
     <row r="527">
       <c r="A527" t="inlineStr">
@@ -21285,9 +21039,6 @@
           <t>[ROUTINE] Insider trade — Sarowitz Steven I (Director) sold 11,136 shares @ $150.81 ($1.68M) on 2026-08-06</t>
         </is>
       </c>
-      <c r="F527" t="inlineStr"/>
-      <c r="G527" t="inlineStr"/>
-      <c r="H527" t="inlineStr"/>
     </row>
     <row r="528">
       <c r="A528" t="inlineStr">
@@ -21315,9 +21066,1416 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F528" t="inlineStr"/>
-      <c r="G528" t="inlineStr"/>
-      <c r="H528" t="inlineStr"/>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>GRMN</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Garmin Ltd.</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1121788/000101410826000045/xslF345X06/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Jonathan Burrell (Director) gift: 90,000 Registered Shares on 2026-08-10</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr"/>
+      <c r="G529" t="inlineStr"/>
+      <c r="H529" t="inlineStr"/>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>https://www.lyft.com/blog</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr"/>
+      <c r="G530" t="inlineStr"/>
+      <c r="H530" t="inlineStr"/>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Lyft, Inc.</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1759509/000197349526000005/xslF345X06/form4-08112026_100831.xml</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Whiteside Janey (Director) sold 14,220 shares @ $17.00 ($241.7K) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr"/>
+      <c r="G531" t="inlineStr"/>
+      <c r="H531" t="inlineStr"/>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>EXPE</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Expedia Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>https://careers.expediagroup.com</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr"/>
+      <c r="G532" t="inlineStr"/>
+      <c r="H532" t="inlineStr"/>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>BKNG</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Booking Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/content/terms.html</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr"/>
+      <c r="G533" t="inlineStr"/>
+      <c r="H533" t="inlineStr"/>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>https://careers.airbnb.com</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr"/>
+      <c r="G534" t="inlineStr"/>
+      <c r="H534" t="inlineStr"/>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1559720/000119312526345333/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Chesky Brian (CEO and Chairman) sold 20,000 shares @ $173.61 ($3.47M) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr"/>
+      <c r="G535" t="inlineStr"/>
+      <c r="H535" t="inlineStr"/>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1559720/000119312526345326/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Chesky Brian (CEO and Chairman) sold 200,000 shares @ $174.79 ($34.96M) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr"/>
+      <c r="G536" t="inlineStr"/>
+      <c r="H536" t="inlineStr"/>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1559720/000119312526345316/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Blecharczyk Nathan (Chief Strategy Officer) sold 531,000 shares @ $174.41 ($92.61M) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr"/>
+      <c r="G537" t="inlineStr"/>
+      <c r="H537" t="inlineStr"/>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Airbnb, Inc.</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1559720/000119312526345303/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Kenneth I Chenault (Director) sold 8,346 shares @ $170.00 ($1.42M) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr"/>
+      <c r="G538" t="inlineStr"/>
+      <c r="H538" t="inlineStr"/>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>CHH</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Choice Hotels International, Inc.</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>https://media.choicehotels.com</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr"/>
+      <c r="G539" t="inlineStr"/>
+      <c r="H539" t="inlineStr"/>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>https://blog.google</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr"/>
+      <c r="G540" t="inlineStr"/>
+      <c r="H540" t="inlineStr"/>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1652044/000119312526345383/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Sergey Brin (Director) C: 673,200 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr"/>
+      <c r="G541" t="inlineStr"/>
+      <c r="H541" t="inlineStr"/>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1564408/000180678426000003/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Coffey Kelly (Director) granted 46,905 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr"/>
+      <c r="G542" t="inlineStr"/>
+      <c r="H542" t="inlineStr"/>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1564408/000187456626000003/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Vargas Fidel (Director) granted 46,905 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr"/>
+      <c r="G543" t="inlineStr"/>
+      <c r="H543" t="inlineStr"/>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1564408/000169932326000002/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Coles Joanna (Director) granted 46,905 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr"/>
+      <c r="G544" t="inlineStr"/>
+      <c r="H544" t="inlineStr"/>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1564408/000175091326000003/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Lanzone James (Director) granted 46,905 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr"/>
+      <c r="G545" t="inlineStr"/>
+      <c r="H545" t="inlineStr"/>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1564408/000213702426000012/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Wood Luke (Director) granted 46,905 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr"/>
+      <c r="G546" t="inlineStr"/>
+      <c r="H546" t="inlineStr"/>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1564408/000127335726000003/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Scott D Miller (Director) granted 46,905 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr"/>
+      <c r="G547" t="inlineStr"/>
+      <c r="H547" t="inlineStr"/>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1564408/000174331726000003/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Spence Patrick (Director) granted 46,905 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr"/>
+      <c r="G548" t="inlineStr"/>
+      <c r="H548" t="inlineStr"/>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1564408/000160611526000006/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Lynton Michael (Director) granted 46,905 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr"/>
+      <c r="G549" t="inlineStr"/>
+      <c r="H549" t="inlineStr"/>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1564408/000183277826000003/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Jenkins Elizabeth (Director) granted 46,905 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr"/>
+      <c r="G550" t="inlineStr"/>
+      <c r="H550" t="inlineStr"/>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1564408/000174798926000003/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Thorpe Poppy (Director) granted 46,905 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr"/>
+      <c r="G551" t="inlineStr"/>
+      <c r="H551" t="inlineStr"/>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1564408/000172739626000007/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Morrow Rebecca (Chief Accounting Officer) granted 65,081 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr"/>
+      <c r="G552" t="inlineStr"/>
+      <c r="H552" t="inlineStr"/>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>SNAP</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Snap Inc.</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1564408/000165473326000010/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Matthew Blake Mcrae (Director) granted 46,905 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr"/>
+      <c r="G553" t="inlineStr"/>
+      <c r="H553" t="inlineStr"/>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>PINS</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Pinterest, Inc.</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1506293/000192109426000830/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Silbermann Benjamin (Director) plans to sell 46,875 shares (~$1.12M) on/after 08/11/2026</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr"/>
+      <c r="G554" t="inlineStr"/>
+      <c r="H554" t="inlineStr"/>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>PINS</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Pinterest, Inc.</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1506293/000192109426000829/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Brown Claude Leonard (Officer) plans to sell 12,240 shares (~$292.3K) on/after 08/11/2026</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr"/>
+      <c r="G555" t="inlineStr"/>
+      <c r="H555" t="inlineStr"/>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Reddit, Inc.</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>https://redditinc.com/careers</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr"/>
+      <c r="G556" t="inlineStr"/>
+      <c r="H556" t="inlineStr"/>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>AppLovin Corporation</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>https://www.applovin.com/blog/</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr"/>
+      <c r="G557" t="inlineStr"/>
+      <c r="H557" t="inlineStr"/>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Unity Software Inc.</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>https://careers.unity.com</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr"/>
+      <c r="G558" t="inlineStr"/>
+      <c r="H558" t="inlineStr"/>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Unity Software Inc.</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1810806/000197640826000716/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Dovrat Shlomo (Former Director) plans to sell 50,000 shares (~$2.15M) on/after 08/11/2026</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr"/>
+      <c r="G559" t="inlineStr"/>
+      <c r="H559" t="inlineStr"/>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Unity Software Inc.</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1810806/000119312526344792/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Durban Egon (Director) other: 21,537 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr"/>
+      <c r="G560" t="inlineStr"/>
+      <c r="H560" t="inlineStr"/>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>https://www.spotify.com/premium</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr"/>
+      <c r="G561" t="inlineStr"/>
+      <c r="H561" t="inlineStr"/>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Spotify Technology S.A.</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>https://www.lifeatspotify.com</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr"/>
+      <c r="G562" t="inlineStr"/>
+      <c r="H562" t="inlineStr"/>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>https://www.disneyplus.com/welcome</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr"/>
+      <c r="G563" t="inlineStr"/>
+      <c r="H563" t="inlineStr"/>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>https://thewaltdisneycompany.com/news/</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr"/>
+      <c r="G564" t="inlineStr"/>
+      <c r="H564" t="inlineStr"/>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>https://jobs.disneycareers.com</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr"/>
+      <c r="G565" t="inlineStr"/>
+      <c r="H565" t="inlineStr"/>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Fox Corporation</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>https://foxcareers.com</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr"/>
+      <c r="G566" t="inlineStr"/>
+      <c r="H566" t="inlineStr"/>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>WMG</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Warner Music Group Corp.</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1319161/000119312526344951/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>[ROUTINE] New insider — initial ownership statement</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr"/>
+      <c r="G567" t="inlineStr"/>
+      <c r="H567" t="inlineStr"/>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>LYV</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Live Nation Entertainment, Inc.</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>https://investors.livenationentertainment.com</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr"/>
+      <c r="G568" t="inlineStr"/>
+      <c r="H568" t="inlineStr"/>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Take-Two Interactive Software, Inc.</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>https://ir.take2games.com</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr"/>
+      <c r="G569" t="inlineStr"/>
+      <c r="H569" t="inlineStr"/>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Take-Two Interactive Software, Inc.</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/946581/000094658126000069/xslF345X06/form4.xml</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Strauss Zelnick (Chairman, CEO) sold 40,000 shares @ $252.64 ($10.11M) on 2026-08-10</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr"/>
+      <c r="G570" t="inlineStr"/>
+      <c r="H570" t="inlineStr"/>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>RBLX</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Roblox Corporation</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1315098/000183498826000008/xslF345X06/form4-08112026_080826.xml</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Lee Anthony P (Director) gift: 100,000 shares on 2026-08-10</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr"/>
+      <c r="G571" t="inlineStr"/>
+      <c r="H571" t="inlineStr"/>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Intuit Inc.</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>https://investors.intuit.com</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr"/>
+      <c r="G572" t="inlineStr"/>
+      <c r="H572" t="inlineStr"/>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>PAYC</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Paycom Software, Inc.</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1590955/000119312526345730/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Boelte Craig E. (Director) gift: 1,000 shares on 2026-08-10</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr"/>
+      <c r="G573" t="inlineStr"/>
+      <c r="H573" t="inlineStr"/>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>PCTY</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Paylocity Holding Corporation</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1591698/000159787026000004/xslF345X06/wk-form4_1786478595.xml</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Sarowitz Steven I (Director) sold 32,972 shares @ $152.48 ($5.03M) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr"/>
+      <c r="G574" t="inlineStr"/>
+      <c r="H574" t="inlineStr"/>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>CDW Corporation</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1402057/000140205726000068/xslF345X06/wk-form4_1786479982.xml</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Elizabeth H. Connelly (See Remarks) sold 26,695 shares @ $137.62 ($3.67M) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr"/>
+      <c r="G575" t="inlineStr"/>
+      <c r="H575" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=ARMK,CVNA,HQY,VRSK run 2026-08-12T13:17Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -6853,7 +6853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H575"/>
+  <dimension ref="A1:H581"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -21093,9 +21093,6 @@
           <t>[ROUTINE] Insider trade — Jonathan Burrell (Director) gift: 90,000 Registered Shares on 2026-08-10</t>
         </is>
       </c>
-      <c r="F529" t="inlineStr"/>
-      <c r="G529" t="inlineStr"/>
-      <c r="H529" t="inlineStr"/>
     </row>
     <row r="530">
       <c r="A530" t="inlineStr">
@@ -21123,9 +21120,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F530" t="inlineStr"/>
-      <c r="G530" t="inlineStr"/>
-      <c r="H530" t="inlineStr"/>
     </row>
     <row r="531">
       <c r="A531" t="inlineStr">
@@ -21153,9 +21147,6 @@
           <t>[ROUTINE] Insider trade — Whiteside Janey (Director) sold 14,220 shares @ $17.00 ($241.7K) on 2026-08-07</t>
         </is>
       </c>
-      <c r="F531" t="inlineStr"/>
-      <c r="G531" t="inlineStr"/>
-      <c r="H531" t="inlineStr"/>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
@@ -21183,9 +21174,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F532" t="inlineStr"/>
-      <c r="G532" t="inlineStr"/>
-      <c r="H532" t="inlineStr"/>
     </row>
     <row r="533">
       <c r="A533" t="inlineStr">
@@ -21213,9 +21201,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F533" t="inlineStr"/>
-      <c r="G533" t="inlineStr"/>
-      <c r="H533" t="inlineStr"/>
     </row>
     <row r="534">
       <c r="A534" t="inlineStr">
@@ -21243,9 +21228,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F534" t="inlineStr"/>
-      <c r="G534" t="inlineStr"/>
-      <c r="H534" t="inlineStr"/>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
@@ -21273,9 +21255,6 @@
           <t>[ROUTINE] Insider trade — Chesky Brian (CEO and Chairman) sold 20,000 shares @ $173.61 ($3.47M) on 2026-08-07</t>
         </is>
       </c>
-      <c r="F535" t="inlineStr"/>
-      <c r="G535" t="inlineStr"/>
-      <c r="H535" t="inlineStr"/>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
@@ -21303,9 +21282,6 @@
           <t>[ROUTINE] Insider trade — Chesky Brian (CEO and Chairman) sold 200,000 shares @ $174.79 ($34.96M) on 2026-08-07</t>
         </is>
       </c>
-      <c r="F536" t="inlineStr"/>
-      <c r="G536" t="inlineStr"/>
-      <c r="H536" t="inlineStr"/>
     </row>
     <row r="537">
       <c r="A537" t="inlineStr">
@@ -21333,9 +21309,6 @@
           <t>[ROUTINE] Insider trade — Blecharczyk Nathan (Chief Strategy Officer) sold 531,000 shares @ $174.41 ($92.61M) on 2026-08-07</t>
         </is>
       </c>
-      <c r="F537" t="inlineStr"/>
-      <c r="G537" t="inlineStr"/>
-      <c r="H537" t="inlineStr"/>
     </row>
     <row r="538">
       <c r="A538" t="inlineStr">
@@ -21363,9 +21336,6 @@
           <t>[ROUTINE] Insider trade — Kenneth I Chenault (Director) sold 8,346 shares @ $170.00 ($1.42M) on 2026-08-07</t>
         </is>
       </c>
-      <c r="F538" t="inlineStr"/>
-      <c r="G538" t="inlineStr"/>
-      <c r="H538" t="inlineStr"/>
     </row>
     <row r="539">
       <c r="A539" t="inlineStr">
@@ -21393,9 +21363,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F539" t="inlineStr"/>
-      <c r="G539" t="inlineStr"/>
-      <c r="H539" t="inlineStr"/>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
@@ -21423,9 +21390,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F540" t="inlineStr"/>
-      <c r="G540" t="inlineStr"/>
-      <c r="H540" t="inlineStr"/>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
@@ -21453,9 +21417,6 @@
           <t>[ROUTINE] Insider trade — Sergey Brin (Director) C: 673,200 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F541" t="inlineStr"/>
-      <c r="G541" t="inlineStr"/>
-      <c r="H541" t="inlineStr"/>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
@@ -21483,9 +21444,6 @@
           <t>[ROUTINE] Insider trade — Coffey Kelly (Director) granted 46,905 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F542" t="inlineStr"/>
-      <c r="G542" t="inlineStr"/>
-      <c r="H542" t="inlineStr"/>
     </row>
     <row r="543">
       <c r="A543" t="inlineStr">
@@ -21513,9 +21471,6 @@
           <t>[ROUTINE] Insider trade — Vargas Fidel (Director) granted 46,905 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F543" t="inlineStr"/>
-      <c r="G543" t="inlineStr"/>
-      <c r="H543" t="inlineStr"/>
     </row>
     <row r="544">
       <c r="A544" t="inlineStr">
@@ -21543,9 +21498,6 @@
           <t>[ROUTINE] Insider trade — Coles Joanna (Director) granted 46,905 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F544" t="inlineStr"/>
-      <c r="G544" t="inlineStr"/>
-      <c r="H544" t="inlineStr"/>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
@@ -21573,9 +21525,6 @@
           <t>[ROUTINE] Insider trade — Lanzone James (Director) granted 46,905 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F545" t="inlineStr"/>
-      <c r="G545" t="inlineStr"/>
-      <c r="H545" t="inlineStr"/>
     </row>
     <row r="546">
       <c r="A546" t="inlineStr">
@@ -21603,9 +21552,6 @@
           <t>[ROUTINE] Insider trade — Wood Luke (Director) granted 46,905 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F546" t="inlineStr"/>
-      <c r="G546" t="inlineStr"/>
-      <c r="H546" t="inlineStr"/>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
@@ -21633,9 +21579,6 @@
           <t>[ROUTINE] Insider trade — Scott D Miller (Director) granted 46,905 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F547" t="inlineStr"/>
-      <c r="G547" t="inlineStr"/>
-      <c r="H547" t="inlineStr"/>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
@@ -21663,9 +21606,6 @@
           <t>[ROUTINE] Insider trade — Spence Patrick (Director) granted 46,905 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F548" t="inlineStr"/>
-      <c r="G548" t="inlineStr"/>
-      <c r="H548" t="inlineStr"/>
     </row>
     <row r="549">
       <c r="A549" t="inlineStr">
@@ -21693,9 +21633,6 @@
           <t>[ROUTINE] Insider trade — Lynton Michael (Director) granted 46,905 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F549" t="inlineStr"/>
-      <c r="G549" t="inlineStr"/>
-      <c r="H549" t="inlineStr"/>
     </row>
     <row r="550">
       <c r="A550" t="inlineStr">
@@ -21723,9 +21660,6 @@
           <t>[ROUTINE] Insider trade — Jenkins Elizabeth (Director) granted 46,905 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F550" t="inlineStr"/>
-      <c r="G550" t="inlineStr"/>
-      <c r="H550" t="inlineStr"/>
     </row>
     <row r="551">
       <c r="A551" t="inlineStr">
@@ -21753,9 +21687,6 @@
           <t>[ROUTINE] Insider trade — Thorpe Poppy (Director) granted 46,905 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F551" t="inlineStr"/>
-      <c r="G551" t="inlineStr"/>
-      <c r="H551" t="inlineStr"/>
     </row>
     <row r="552">
       <c r="A552" t="inlineStr">
@@ -21783,9 +21714,6 @@
           <t>[ROUTINE] Insider trade — Morrow Rebecca (Chief Accounting Officer) granted 65,081 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F552" t="inlineStr"/>
-      <c r="G552" t="inlineStr"/>
-      <c r="H552" t="inlineStr"/>
     </row>
     <row r="553">
       <c r="A553" t="inlineStr">
@@ -21813,9 +21741,6 @@
           <t>[ROUTINE] Insider trade — Matthew Blake Mcrae (Director) granted 46,905 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F553" t="inlineStr"/>
-      <c r="G553" t="inlineStr"/>
-      <c r="H553" t="inlineStr"/>
     </row>
     <row r="554">
       <c r="A554" t="inlineStr">
@@ -21843,9 +21768,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Silbermann Benjamin (Director) plans to sell 46,875 shares (~$1.12M) on/after 08/11/2026</t>
         </is>
       </c>
-      <c r="F554" t="inlineStr"/>
-      <c r="G554" t="inlineStr"/>
-      <c r="H554" t="inlineStr"/>
     </row>
     <row r="555">
       <c r="A555" t="inlineStr">
@@ -21873,9 +21795,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Brown Claude Leonard (Officer) plans to sell 12,240 shares (~$292.3K) on/after 08/11/2026</t>
         </is>
       </c>
-      <c r="F555" t="inlineStr"/>
-      <c r="G555" t="inlineStr"/>
-      <c r="H555" t="inlineStr"/>
     </row>
     <row r="556">
       <c r="A556" t="inlineStr">
@@ -21903,9 +21822,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F556" t="inlineStr"/>
-      <c r="G556" t="inlineStr"/>
-      <c r="H556" t="inlineStr"/>
     </row>
     <row r="557">
       <c r="A557" t="inlineStr">
@@ -21933,9 +21849,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F557" t="inlineStr"/>
-      <c r="G557" t="inlineStr"/>
-      <c r="H557" t="inlineStr"/>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr">
@@ -21963,9 +21876,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F558" t="inlineStr"/>
-      <c r="G558" t="inlineStr"/>
-      <c r="H558" t="inlineStr"/>
     </row>
     <row r="559">
       <c r="A559" t="inlineStr">
@@ -21993,9 +21903,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Dovrat Shlomo (Former Director) plans to sell 50,000 shares (~$2.15M) on/after 08/11/2026</t>
         </is>
       </c>
-      <c r="F559" t="inlineStr"/>
-      <c r="G559" t="inlineStr"/>
-      <c r="H559" t="inlineStr"/>
     </row>
     <row r="560">
       <c r="A560" t="inlineStr">
@@ -22023,9 +21930,6 @@
           <t>[ROUTINE] Insider trade — Durban Egon (Director) other: 21,537 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F560" t="inlineStr"/>
-      <c r="G560" t="inlineStr"/>
-      <c r="H560" t="inlineStr"/>
     </row>
     <row r="561">
       <c r="A561" t="inlineStr">
@@ -22053,9 +21957,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F561" t="inlineStr"/>
-      <c r="G561" t="inlineStr"/>
-      <c r="H561" t="inlineStr"/>
     </row>
     <row r="562">
       <c r="A562" t="inlineStr">
@@ -22083,9 +21984,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F562" t="inlineStr"/>
-      <c r="G562" t="inlineStr"/>
-      <c r="H562" t="inlineStr"/>
     </row>
     <row r="563">
       <c r="A563" t="inlineStr">
@@ -22113,9 +22011,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F563" t="inlineStr"/>
-      <c r="G563" t="inlineStr"/>
-      <c r="H563" t="inlineStr"/>
     </row>
     <row r="564">
       <c r="A564" t="inlineStr">
@@ -22143,9 +22038,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F564" t="inlineStr"/>
-      <c r="G564" t="inlineStr"/>
-      <c r="H564" t="inlineStr"/>
     </row>
     <row r="565">
       <c r="A565" t="inlineStr">
@@ -22173,9 +22065,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F565" t="inlineStr"/>
-      <c r="G565" t="inlineStr"/>
-      <c r="H565" t="inlineStr"/>
     </row>
     <row r="566">
       <c r="A566" t="inlineStr">
@@ -22203,9 +22092,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F566" t="inlineStr"/>
-      <c r="G566" t="inlineStr"/>
-      <c r="H566" t="inlineStr"/>
     </row>
     <row r="567">
       <c r="A567" t="inlineStr">
@@ -22233,9 +22119,6 @@
           <t>[ROUTINE] New insider — initial ownership statement</t>
         </is>
       </c>
-      <c r="F567" t="inlineStr"/>
-      <c r="G567" t="inlineStr"/>
-      <c r="H567" t="inlineStr"/>
     </row>
     <row r="568">
       <c r="A568" t="inlineStr">
@@ -22263,9 +22146,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F568" t="inlineStr"/>
-      <c r="G568" t="inlineStr"/>
-      <c r="H568" t="inlineStr"/>
     </row>
     <row r="569">
       <c r="A569" t="inlineStr">
@@ -22293,9 +22173,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F569" t="inlineStr"/>
-      <c r="G569" t="inlineStr"/>
-      <c r="H569" t="inlineStr"/>
     </row>
     <row r="570">
       <c r="A570" t="inlineStr">
@@ -22323,9 +22200,6 @@
           <t>[ROUTINE] Insider trade — Strauss Zelnick (Chairman, CEO) sold 40,000 shares @ $252.64 ($10.11M) on 2026-08-10</t>
         </is>
       </c>
-      <c r="F570" t="inlineStr"/>
-      <c r="G570" t="inlineStr"/>
-      <c r="H570" t="inlineStr"/>
     </row>
     <row r="571">
       <c r="A571" t="inlineStr">
@@ -22353,9 +22227,6 @@
           <t>[ROUTINE] Insider trade — Lee Anthony P (Director) gift: 100,000 shares on 2026-08-10</t>
         </is>
       </c>
-      <c r="F571" t="inlineStr"/>
-      <c r="G571" t="inlineStr"/>
-      <c r="H571" t="inlineStr"/>
     </row>
     <row r="572">
       <c r="A572" t="inlineStr">
@@ -22383,9 +22254,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F572" t="inlineStr"/>
-      <c r="G572" t="inlineStr"/>
-      <c r="H572" t="inlineStr"/>
     </row>
     <row r="573">
       <c r="A573" t="inlineStr">
@@ -22413,9 +22281,6 @@
           <t>[ROUTINE] Insider trade — Boelte Craig E. (Director) gift: 1,000 shares on 2026-08-10</t>
         </is>
       </c>
-      <c r="F573" t="inlineStr"/>
-      <c r="G573" t="inlineStr"/>
-      <c r="H573" t="inlineStr"/>
     </row>
     <row r="574">
       <c r="A574" t="inlineStr">
@@ -22443,9 +22308,6 @@
           <t>[ROUTINE] Insider trade — Sarowitz Steven I (Director) sold 32,972 shares @ $152.48 ($5.03M) on 2026-08-07</t>
         </is>
       </c>
-      <c r="F574" t="inlineStr"/>
-      <c r="G574" t="inlineStr"/>
-      <c r="H574" t="inlineStr"/>
     </row>
     <row r="575">
       <c r="A575" t="inlineStr">
@@ -22473,9 +22335,186 @@
           <t>[ROUTINE] Insider trade — Elizabeth H. Connelly (See Remarks) sold 26,695 shares @ $137.62 ($3.67M) on 2026-08-07</t>
         </is>
       </c>
-      <c r="F575" t="inlineStr"/>
-      <c r="G575" t="inlineStr"/>
-      <c r="H575" t="inlineStr"/>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>VRSK</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Verisk Analytics, Inc.</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>https://investor.verisk.com</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr"/>
+      <c r="G576" t="inlineStr"/>
+      <c r="H576" t="inlineStr"/>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>CVNA</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Carvana Co.</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>https://investors.carvana.com</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr"/>
+      <c r="G577" t="inlineStr"/>
+      <c r="H577" t="inlineStr"/>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>ARMK</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Aramark</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>https://careers.aramark.com</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr"/>
+      <c r="G578" t="inlineStr"/>
+      <c r="H578" t="inlineStr"/>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>ARMK</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Aramark</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1584509/000170255126000011/xslF345X06/wk-form3_1786480868.xml</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>[ROUTINE] New insider — initial ownership statement</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr"/>
+      <c r="G579" t="inlineStr"/>
+      <c r="H579" t="inlineStr"/>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>ARMK</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Aramark</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1584509/000158450926000122/cik0-20260703.htm</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Quarterly report</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr"/>
+      <c r="G580" t="inlineStr"/>
+      <c r="H580" t="inlineStr"/>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>ARMK</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Aramark</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1584509/000158450926000118/cik0-20260811.htm</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Material event disclosure</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr"/>
+      <c r="G581" t="inlineStr"/>
+      <c r="H581" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tier=high run 2026-08-12T13:25Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -6853,7 +6853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H581"/>
+  <dimension ref="A1:H623"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -22362,9 +22362,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F576" t="inlineStr"/>
-      <c r="G576" t="inlineStr"/>
-      <c r="H576" t="inlineStr"/>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
@@ -22392,9 +22389,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F577" t="inlineStr"/>
-      <c r="G577" t="inlineStr"/>
-      <c r="H577" t="inlineStr"/>
     </row>
     <row r="578">
       <c r="A578" t="inlineStr">
@@ -22422,9 +22416,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F578" t="inlineStr"/>
-      <c r="G578" t="inlineStr"/>
-      <c r="H578" t="inlineStr"/>
     </row>
     <row r="579">
       <c r="A579" t="inlineStr">
@@ -22452,9 +22443,6 @@
           <t>[ROUTINE] New insider — initial ownership statement</t>
         </is>
       </c>
-      <c r="F579" t="inlineStr"/>
-      <c r="G579" t="inlineStr"/>
-      <c r="H579" t="inlineStr"/>
     </row>
     <row r="580">
       <c r="A580" t="inlineStr">
@@ -22482,9 +22470,6 @@
           <t>[MATERIAL] Quarterly report</t>
         </is>
       </c>
-      <c r="F580" t="inlineStr"/>
-      <c r="G580" t="inlineStr"/>
-      <c r="H580" t="inlineStr"/>
     </row>
     <row r="581">
       <c r="A581" t="inlineStr">
@@ -22512,9 +22497,1266 @@
           <t>[MATERIAL] Material event disclosure</t>
         </is>
       </c>
-      <c r="F581" t="inlineStr"/>
-      <c r="G581" t="inlineStr"/>
-      <c r="H581" t="inlineStr"/>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/legal/terms</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr"/>
+      <c r="G582" t="inlineStr"/>
+      <c r="H582" t="inlineStr"/>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/pricing</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr"/>
+      <c r="G583" t="inlineStr"/>
+      <c r="H583" t="inlineStr"/>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>https://news.shopify.com</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr"/>
+      <c r="G584" t="inlineStr"/>
+      <c r="H584" t="inlineStr"/>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>https://investors.shopify.com</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr"/>
+      <c r="G585" t="inlineStr"/>
+      <c r="H585" t="inlineStr"/>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Shopify Inc.</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/careers</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr"/>
+      <c r="G586" t="inlineStr"/>
+      <c r="H586" t="inlineStr"/>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>ETSY</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Etsy Inc.</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>https://investors.etsy.com</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr"/>
+      <c r="G587" t="inlineStr"/>
+      <c r="H587" t="inlineStr"/>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>ETSY</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Etsy Inc.</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1370637/000088698226000342/xslSCHEDULE_13G_X02/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Update to 5%+ passive owner disclosure</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr"/>
+      <c r="G588" t="inlineStr"/>
+      <c r="H588" t="inlineStr"/>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>ETSY</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Etsy Inc.</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1370637/000196922326000868/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Colburn Richard Edward III (Officer) plans to sell 8,252 shares (~$694.9K) on/after 08/10/2026</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr"/>
+      <c r="G589" t="inlineStr"/>
+      <c r="H589" t="inlineStr"/>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Duolingo Inc.</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>https://careers.duolingo.com/jobs/8687677002?gh_jid=8687677002</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>New senior role: Director of Growth Marketing Strategy</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr"/>
+      <c r="G590" t="inlineStr"/>
+      <c r="H590" t="inlineStr"/>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Duolingo Inc.</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>https://careers.duolingo.com/jobs/8691257002?gh_jid=8691257002</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>New senior role: Director of Sourcing</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr"/>
+      <c r="G591" t="inlineStr"/>
+      <c r="H591" t="inlineStr"/>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Duolingo Inc.</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>https://careers.duolingo.com/jobs/8590178002?gh_jid=8590178002</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>New senior role: Head of Talent Management Programs and PMO</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr"/>
+      <c r="G592" t="inlineStr"/>
+      <c r="H592" t="inlineStr"/>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Duolingo Inc.</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>https://careers.duolingo.com/jobs/8616695002?gh_jid=8616695002</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>New senior role: Senior Director of Engineering, Math</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr"/>
+      <c r="G593" t="inlineStr"/>
+      <c r="H593" t="inlineStr"/>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Duolingo Inc.</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>https://careers.duolingo.com/jobs/8584465002?gh_jid=8584465002</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>New senior role: Senior Director of Engineering, New Subjects</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr"/>
+      <c r="G594" t="inlineStr"/>
+      <c r="H594" t="inlineStr"/>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Duolingo Inc.</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/duolingo</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>35 new non-senior roles posted</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr"/>
+      <c r="G595" t="inlineStr"/>
+      <c r="H595" t="inlineStr"/>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Duolingo Inc.</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>https://blog.duolingo.com/</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr"/>
+      <c r="G596" t="inlineStr"/>
+      <c r="H596" t="inlineStr"/>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Duolingo Inc.</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1562088/000162828026055015/duol-20260810.htm</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Material event disclosure</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr"/>
+      <c r="G597" t="inlineStr"/>
+      <c r="H597" t="inlineStr"/>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>BILL</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>BILL Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>https://www.bill.com/leadership</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr"/>
+      <c r="G598" t="inlineStr"/>
+      <c r="H598" t="inlineStr"/>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>BILL</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>BILL Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>https://www.bill.com/product/pricing</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr"/>
+      <c r="G599" t="inlineStr"/>
+      <c r="H599" t="inlineStr"/>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>BILL</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>BILL Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>https://www.bill.com/press-release</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr"/>
+      <c r="G600" t="inlineStr"/>
+      <c r="H600" t="inlineStr"/>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>BILL</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>BILL Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>https://investor.bill.com</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr"/>
+      <c r="G601" t="inlineStr"/>
+      <c r="H601" t="inlineStr"/>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>BILL</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>BILL Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>https://www.bill.com/careers</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>careers: change detected</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr"/>
+      <c r="G602" t="inlineStr"/>
+      <c r="H602" t="inlineStr"/>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>https://careers.toasttab.com/jobs?gh_jid=7743831</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>New senior role: Director of International Program Management</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr"/>
+      <c r="G603" t="inlineStr"/>
+      <c r="H603" t="inlineStr"/>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>https://careers.toasttab.com/jobs?gh_jid=7777850</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>New senior role: Director of International Program Management</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr"/>
+      <c r="G604" t="inlineStr"/>
+      <c r="H604" t="inlineStr"/>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>https://careers.toasttab.com/jobs?gh_jid=7996612</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>New senior role: Director of Product Management, Enterprise</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr"/>
+      <c r="G605" t="inlineStr"/>
+      <c r="H605" t="inlineStr"/>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>https://careers.toasttab.com/jobs?gh_jid=7838464</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>New senior role: Vice President, Enterprise Sales</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr"/>
+      <c r="G606" t="inlineStr"/>
+      <c r="H606" t="inlineStr"/>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/toast</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>250 new non-senior roles posted</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr"/>
+      <c r="G607" t="inlineStr"/>
+      <c r="H607" t="inlineStr"/>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>https://pos.toasttab.com/terms-of-service</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr"/>
+      <c r="G608" t="inlineStr"/>
+      <c r="H608" t="inlineStr"/>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>https://pos.toasttab.com/pricing</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr"/>
+      <c r="G609" t="inlineStr"/>
+      <c r="H609" t="inlineStr"/>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>https://investors.toasttab.com</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr"/>
+      <c r="G610" t="inlineStr"/>
+      <c r="H610" t="inlineStr"/>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1650164/000195917326005905/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Vassil Jonathan (Officer) plans to sell 13,797 shares (~$496.9K) on/after 08/11/2026</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr"/>
+      <c r="G611" t="inlineStr"/>
+      <c r="H611" t="inlineStr"/>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1650164/000165016426000178/xslF345X06/wk-form4_1786480258.xml</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Narang Aman (CEO) sold 161,948 shares @ $35.31 ($5.72M) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr"/>
+      <c r="G612" t="inlineStr"/>
+      <c r="H612" t="inlineStr"/>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1650164/000165016426000177/xslF345X06/wk-form4_1786480226.xml</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Gomez Elena (President, CFO) sold 7,924 shares @ $35.30 ($279.7K) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr"/>
+      <c r="G613" t="inlineStr"/>
+      <c r="H613" t="inlineStr"/>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1650164/000195917326005860/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Narang Aman (Officer) plans to sell 119,843 shares (~$4.24M) on/after 08/10/2026</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr"/>
+      <c r="G614" t="inlineStr"/>
+      <c r="H614" t="inlineStr"/>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Toast Inc.</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1650164/000195917326005851/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Gomez Elena (Officer) plans to sell 5,761 shares (~$203.8K) on/after 08/10/2026</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr"/>
+      <c r="G615" t="inlineStr"/>
+      <c r="H615" t="inlineStr"/>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/robinhood/jobs/7839130?t=gh_src=&amp;gh_jid=7839130</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>New senior role: Chief of Staff, Brokerage Product</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr"/>
+      <c r="G616" t="inlineStr"/>
+      <c r="H616" t="inlineStr"/>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/robinhood/jobs/8088954?t=gh_src=&amp;gh_jid=8088954</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>New senior role: Director of Accounting</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr"/>
+      <c r="G617" t="inlineStr"/>
+      <c r="H617" t="inlineStr"/>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/robinhood/jobs/8039695?t=gh_src=&amp;gh_jid=8039695</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>New senior role: Senior Director of Income Tax</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr"/>
+      <c r="G618" t="inlineStr"/>
+      <c r="H618" t="inlineStr"/>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/robinhood</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>95 new non-senior roles posted</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr"/>
+      <c r="G619" t="inlineStr"/>
+      <c r="H619" t="inlineStr"/>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>https://cdn.robinhood.com/assets/robinhood/legal/Robinhood-Customer-Agreement.pdf</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr"/>
+      <c r="G620" t="inlineStr"/>
+      <c r="H620" t="inlineStr"/>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>https://robinhood.com/us/en/support/articles/trading-fees-on-robinhood/</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr"/>
+      <c r="G621" t="inlineStr"/>
+      <c r="H621" t="inlineStr"/>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>https://newsroom.aboutrobinhood.com</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr"/>
+      <c r="G622" t="inlineStr"/>
+      <c r="H622" t="inlineStr"/>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Robinhood Markets Inc.</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1783879/000178387926000124/xslF345X06/wk-form4_1786481261.xml</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Robinhood Markets, Inc. (10%+ owner) sold 18,365 shares @ $28.10 ($516.1K) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr"/>
+      <c r="G623" t="inlineStr"/>
+      <c r="H623" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=CART,DASH run 2026-08-12T15:01Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -6853,7 +6853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H623"/>
+  <dimension ref="A1:H639"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -22524,9 +22524,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F582" t="inlineStr"/>
-      <c r="G582" t="inlineStr"/>
-      <c r="H582" t="inlineStr"/>
     </row>
     <row r="583">
       <c r="A583" t="inlineStr">
@@ -22554,9 +22551,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F583" t="inlineStr"/>
-      <c r="G583" t="inlineStr"/>
-      <c r="H583" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" t="inlineStr">
@@ -22584,9 +22578,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F584" t="inlineStr"/>
-      <c r="G584" t="inlineStr"/>
-      <c r="H584" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" t="inlineStr">
@@ -22614,9 +22605,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F585" t="inlineStr"/>
-      <c r="G585" t="inlineStr"/>
-      <c r="H585" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" t="inlineStr">
@@ -22644,9 +22632,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F586" t="inlineStr"/>
-      <c r="G586" t="inlineStr"/>
-      <c r="H586" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" t="inlineStr">
@@ -22674,9 +22659,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F587" t="inlineStr"/>
-      <c r="G587" t="inlineStr"/>
-      <c r="H587" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" t="inlineStr">
@@ -22704,9 +22686,6 @@
           <t>[MATERIAL] Update to 5%+ passive owner disclosure</t>
         </is>
       </c>
-      <c r="F588" t="inlineStr"/>
-      <c r="G588" t="inlineStr"/>
-      <c r="H588" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" t="inlineStr">
@@ -22734,9 +22713,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Colburn Richard Edward III (Officer) plans to sell 8,252 shares (~$694.9K) on/after 08/10/2026</t>
         </is>
       </c>
-      <c r="F589" t="inlineStr"/>
-      <c r="G589" t="inlineStr"/>
-      <c r="H589" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" t="inlineStr">
@@ -22764,9 +22740,6 @@
           <t>New senior role: Director of Growth Marketing Strategy</t>
         </is>
       </c>
-      <c r="F590" t="inlineStr"/>
-      <c r="G590" t="inlineStr"/>
-      <c r="H590" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" t="inlineStr">
@@ -22794,9 +22767,6 @@
           <t>New senior role: Director of Sourcing</t>
         </is>
       </c>
-      <c r="F591" t="inlineStr"/>
-      <c r="G591" t="inlineStr"/>
-      <c r="H591" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" t="inlineStr">
@@ -22824,9 +22794,6 @@
           <t>New senior role: Head of Talent Management Programs and PMO</t>
         </is>
       </c>
-      <c r="F592" t="inlineStr"/>
-      <c r="G592" t="inlineStr"/>
-      <c r="H592" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" t="inlineStr">
@@ -22854,9 +22821,6 @@
           <t>New senior role: Senior Director of Engineering, Math</t>
         </is>
       </c>
-      <c r="F593" t="inlineStr"/>
-      <c r="G593" t="inlineStr"/>
-      <c r="H593" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" t="inlineStr">
@@ -22884,9 +22848,6 @@
           <t>New senior role: Senior Director of Engineering, New Subjects</t>
         </is>
       </c>
-      <c r="F594" t="inlineStr"/>
-      <c r="G594" t="inlineStr"/>
-      <c r="H594" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" t="inlineStr">
@@ -22914,9 +22875,6 @@
           <t>35 new non-senior roles posted</t>
         </is>
       </c>
-      <c r="F595" t="inlineStr"/>
-      <c r="G595" t="inlineStr"/>
-      <c r="H595" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" t="inlineStr">
@@ -22944,9 +22902,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F596" t="inlineStr"/>
-      <c r="G596" t="inlineStr"/>
-      <c r="H596" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" t="inlineStr">
@@ -22974,9 +22929,6 @@
           <t>[MATERIAL] Material event disclosure</t>
         </is>
       </c>
-      <c r="F597" t="inlineStr"/>
-      <c r="G597" t="inlineStr"/>
-      <c r="H597" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" t="inlineStr">
@@ -23004,9 +22956,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F598" t="inlineStr"/>
-      <c r="G598" t="inlineStr"/>
-      <c r="H598" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" t="inlineStr">
@@ -23034,9 +22983,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F599" t="inlineStr"/>
-      <c r="G599" t="inlineStr"/>
-      <c r="H599" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" t="inlineStr">
@@ -23064,9 +23010,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F600" t="inlineStr"/>
-      <c r="G600" t="inlineStr"/>
-      <c r="H600" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" t="inlineStr">
@@ -23094,9 +23037,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F601" t="inlineStr"/>
-      <c r="G601" t="inlineStr"/>
-      <c r="H601" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" t="inlineStr">
@@ -23124,9 +23064,6 @@
           <t>careers: change detected</t>
         </is>
       </c>
-      <c r="F602" t="inlineStr"/>
-      <c r="G602" t="inlineStr"/>
-      <c r="H602" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" t="inlineStr">
@@ -23154,9 +23091,6 @@
           <t>New senior role: Director of International Program Management</t>
         </is>
       </c>
-      <c r="F603" t="inlineStr"/>
-      <c r="G603" t="inlineStr"/>
-      <c r="H603" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
@@ -23184,9 +23118,6 @@
           <t>New senior role: Director of International Program Management</t>
         </is>
       </c>
-      <c r="F604" t="inlineStr"/>
-      <c r="G604" t="inlineStr"/>
-      <c r="H604" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
@@ -23214,9 +23145,6 @@
           <t>New senior role: Director of Product Management, Enterprise</t>
         </is>
       </c>
-      <c r="F605" t="inlineStr"/>
-      <c r="G605" t="inlineStr"/>
-      <c r="H605" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" t="inlineStr">
@@ -23244,9 +23172,6 @@
           <t>New senior role: Vice President, Enterprise Sales</t>
         </is>
       </c>
-      <c r="F606" t="inlineStr"/>
-      <c r="G606" t="inlineStr"/>
-      <c r="H606" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
@@ -23274,9 +23199,6 @@
           <t>250 new non-senior roles posted</t>
         </is>
       </c>
-      <c r="F607" t="inlineStr"/>
-      <c r="G607" t="inlineStr"/>
-      <c r="H607" t="inlineStr"/>
     </row>
     <row r="608">
       <c r="A608" t="inlineStr">
@@ -23304,9 +23226,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F608" t="inlineStr"/>
-      <c r="G608" t="inlineStr"/>
-      <c r="H608" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" t="inlineStr">
@@ -23334,9 +23253,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F609" t="inlineStr"/>
-      <c r="G609" t="inlineStr"/>
-      <c r="H609" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
@@ -23364,9 +23280,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F610" t="inlineStr"/>
-      <c r="G610" t="inlineStr"/>
-      <c r="H610" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr">
@@ -23394,9 +23307,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Vassil Jonathan (Officer) plans to sell 13,797 shares (~$496.9K) on/after 08/11/2026</t>
         </is>
       </c>
-      <c r="F611" t="inlineStr"/>
-      <c r="G611" t="inlineStr"/>
-      <c r="H611" t="inlineStr"/>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
@@ -23424,9 +23334,6 @@
           <t>[ROUTINE] Insider trade — Narang Aman (CEO) sold 161,948 shares @ $35.31 ($5.72M) on 2026-08-07</t>
         </is>
       </c>
-      <c r="F612" t="inlineStr"/>
-      <c r="G612" t="inlineStr"/>
-      <c r="H612" t="inlineStr"/>
     </row>
     <row r="613">
       <c r="A613" t="inlineStr">
@@ -23454,9 +23361,6 @@
           <t>[ROUTINE] Insider trade — Gomez Elena (President, CFO) sold 7,924 shares @ $35.30 ($279.7K) on 2026-08-07</t>
         </is>
       </c>
-      <c r="F613" t="inlineStr"/>
-      <c r="G613" t="inlineStr"/>
-      <c r="H613" t="inlineStr"/>
     </row>
     <row r="614">
       <c r="A614" t="inlineStr">
@@ -23484,9 +23388,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Narang Aman (Officer) plans to sell 119,843 shares (~$4.24M) on/after 08/10/2026</t>
         </is>
       </c>
-      <c r="F614" t="inlineStr"/>
-      <c r="G614" t="inlineStr"/>
-      <c r="H614" t="inlineStr"/>
     </row>
     <row r="615">
       <c r="A615" t="inlineStr">
@@ -23514,9 +23415,6 @@
           <t>[ROUTINE] Notice of proposed insider sale — Gomez Elena (Officer) plans to sell 5,761 shares (~$203.8K) on/after 08/10/2026</t>
         </is>
       </c>
-      <c r="F615" t="inlineStr"/>
-      <c r="G615" t="inlineStr"/>
-      <c r="H615" t="inlineStr"/>
     </row>
     <row r="616">
       <c r="A616" t="inlineStr">
@@ -23544,9 +23442,6 @@
           <t>New senior role: Chief of Staff, Brokerage Product</t>
         </is>
       </c>
-      <c r="F616" t="inlineStr"/>
-      <c r="G616" t="inlineStr"/>
-      <c r="H616" t="inlineStr"/>
     </row>
     <row r="617">
       <c r="A617" t="inlineStr">
@@ -23574,9 +23469,6 @@
           <t>New senior role: Director of Accounting</t>
         </is>
       </c>
-      <c r="F617" t="inlineStr"/>
-      <c r="G617" t="inlineStr"/>
-      <c r="H617" t="inlineStr"/>
     </row>
     <row r="618">
       <c r="A618" t="inlineStr">
@@ -23604,9 +23496,6 @@
           <t>New senior role: Senior Director of Income Tax</t>
         </is>
       </c>
-      <c r="F618" t="inlineStr"/>
-      <c r="G618" t="inlineStr"/>
-      <c r="H618" t="inlineStr"/>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr">
@@ -23634,9 +23523,6 @@
           <t>95 new non-senior roles posted</t>
         </is>
       </c>
-      <c r="F619" t="inlineStr"/>
-      <c r="G619" t="inlineStr"/>
-      <c r="H619" t="inlineStr"/>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
@@ -23664,9 +23550,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F620" t="inlineStr"/>
-      <c r="G620" t="inlineStr"/>
-      <c r="H620" t="inlineStr"/>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
@@ -23694,9 +23577,6 @@
           <t>pricing: change detected</t>
         </is>
       </c>
-      <c r="F621" t="inlineStr"/>
-      <c r="G621" t="inlineStr"/>
-      <c r="H621" t="inlineStr"/>
     </row>
     <row r="622">
       <c r="A622" t="inlineStr">
@@ -23724,9 +23604,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F622" t="inlineStr"/>
-      <c r="G622" t="inlineStr"/>
-      <c r="H622" t="inlineStr"/>
     </row>
     <row r="623">
       <c r="A623" t="inlineStr">
@@ -23754,9 +23631,486 @@
           <t>[ROUTINE] Insider trade — Robinhood Markets, Inc. (10%+ owner) sold 18,365 shares @ $28.10 ($516.1K) on 2026-08-07</t>
         </is>
       </c>
-      <c r="F623" t="inlineStr"/>
-      <c r="G623" t="inlineStr"/>
-      <c r="H623" t="inlineStr"/>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>https://help.doordash.com/consumers/s/terms-of-service</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr"/>
+      <c r="G624" t="inlineStr"/>
+      <c r="H624" t="inlineStr"/>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com/governance/management/default.aspx</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>management_team: change detected</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr"/>
+      <c r="G625" t="inlineStr"/>
+      <c r="H625" t="inlineStr"/>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>https://about.doordash.com/en-us/news</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr"/>
+      <c r="G626" t="inlineStr"/>
+      <c r="H626" t="inlineStr"/>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>https://ir.doordash.com</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>investor_relations: change detected</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr"/>
+      <c r="G627" t="inlineStr"/>
+      <c r="H627" t="inlineStr"/>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000179033026000005/xslF345X06/form4.xml</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Lin Alfred (Director) other: 7,030,715 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr"/>
+      <c r="G628" t="inlineStr"/>
+      <c r="H628" t="inlineStr"/>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000114036126032238/ny20079824x1_pre14c.htm</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>[UNKNOWN] Form PRE 14C</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr"/>
+      <c r="G629" t="inlineStr"/>
+      <c r="H629" t="inlineStr"/>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000114036126032235/ef20079912_8k.htm</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>[MATERIAL] Material event disclosure</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr"/>
+      <c r="G630" t="inlineStr"/>
+      <c r="H630" t="inlineStr"/>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183261426000025/xslF345X06/form4-08112026_040804.xml</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Tang Stanley (Director) other: 10,361 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr"/>
+      <c r="G631" t="inlineStr"/>
+      <c r="H631" t="inlineStr"/>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183261726000007/xslF345X06/form4-08112026_040802.xml</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Xu Tony (CHIEF EXECUTIVE OFFICER) other: 8,159 shares on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr"/>
+      <c r="G632" t="inlineStr"/>
+      <c r="H632" t="inlineStr"/>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>DoorDash Inc.</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1792789/000183239026000019/xslF345X06/form4-08102026_040802.xml</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Fang Andy (Director) sold 15,000 shares @ $215.00 ($3.23M) on 2026-08-06</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr"/>
+      <c r="G633" t="inlineStr"/>
+      <c r="H633" t="inlineStr"/>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>https://instacart.careers/job/?gh_jid=8112136</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>New senior role: Chief of Staff, Online Grocery</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr"/>
+      <c r="G634" t="inlineStr"/>
+      <c r="H634" t="inlineStr"/>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>https://instacart.careers/job/?gh_jid=8112138</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>New senior role: Chief of Staff, Online Grocery</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr"/>
+      <c r="G635" t="inlineStr"/>
+      <c r="H635" t="inlineStr"/>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>https://instacart.careers/job/?gh_jid=7871823</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>New senior role: Director of Customer Success</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr"/>
+      <c r="G636" t="inlineStr"/>
+      <c r="H636" t="inlineStr"/>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/instacart</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>43 new non-senior roles posted</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr"/>
+      <c r="G637" t="inlineStr"/>
+      <c r="H637" t="inlineStr"/>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/company/newsroom</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>newsroom: change detected</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr"/>
+      <c r="G638" t="inlineStr"/>
+      <c r="H638" t="inlineStr"/>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1579091/000208293026000012/xslF345X06/wk-form4_1786478742.xml</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Rogers Chris (President and CEO) sold 4,933 shares @ $50.00 ($246.7K) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr"/>
+      <c r="G639" t="inlineStr"/>
+      <c r="H639" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monitor: tickers=AFRM,APPF,CART,COMP,CSGP,DASH,DAVE,EBAY,ENVA,GDDY,GLBE,MTCH,ONON,PYPL,RH,RKT,SEZL,SGI,UPST,W,WIX,WSM,XYZ,Z run 2026-08-12T17:27Z
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -6853,7 +6853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H639"/>
+  <dimension ref="A1:H661"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -23658,9 +23658,6 @@
           <t>terms: change detected</t>
         </is>
       </c>
-      <c r="F624" t="inlineStr"/>
-      <c r="G624" t="inlineStr"/>
-      <c r="H624" t="inlineStr"/>
     </row>
     <row r="625">
       <c r="A625" t="inlineStr">
@@ -23688,9 +23685,6 @@
           <t>management_team: change detected</t>
         </is>
       </c>
-      <c r="F625" t="inlineStr"/>
-      <c r="G625" t="inlineStr"/>
-      <c r="H625" t="inlineStr"/>
     </row>
     <row r="626">
       <c r="A626" t="inlineStr">
@@ -23718,9 +23712,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F626" t="inlineStr"/>
-      <c r="G626" t="inlineStr"/>
-      <c r="H626" t="inlineStr"/>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr">
@@ -23748,9 +23739,6 @@
           <t>investor_relations: change detected</t>
         </is>
       </c>
-      <c r="F627" t="inlineStr"/>
-      <c r="G627" t="inlineStr"/>
-      <c r="H627" t="inlineStr"/>
     </row>
     <row r="628">
       <c r="A628" t="inlineStr">
@@ -23778,9 +23766,6 @@
           <t>[ROUTINE] Insider trade — Lin Alfred (Director) other: 7,030,715 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F628" t="inlineStr"/>
-      <c r="G628" t="inlineStr"/>
-      <c r="H628" t="inlineStr"/>
     </row>
     <row r="629">
       <c r="A629" t="inlineStr">
@@ -23808,9 +23793,6 @@
           <t>[UNKNOWN] Form PRE 14C</t>
         </is>
       </c>
-      <c r="F629" t="inlineStr"/>
-      <c r="G629" t="inlineStr"/>
-      <c r="H629" t="inlineStr"/>
     </row>
     <row r="630">
       <c r="A630" t="inlineStr">
@@ -23838,9 +23820,6 @@
           <t>[MATERIAL] Material event disclosure</t>
         </is>
       </c>
-      <c r="F630" t="inlineStr"/>
-      <c r="G630" t="inlineStr"/>
-      <c r="H630" t="inlineStr"/>
     </row>
     <row r="631">
       <c r="A631" t="inlineStr">
@@ -23868,9 +23847,6 @@
           <t>[ROUTINE] Insider trade — Tang Stanley (Director) other: 10,361 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F631" t="inlineStr"/>
-      <c r="G631" t="inlineStr"/>
-      <c r="H631" t="inlineStr"/>
     </row>
     <row r="632">
       <c r="A632" t="inlineStr">
@@ -23898,9 +23874,6 @@
           <t>[ROUTINE] Insider trade — Xu Tony (CHIEF EXECUTIVE OFFICER) other: 8,159 shares on 2026-08-07</t>
         </is>
       </c>
-      <c r="F632" t="inlineStr"/>
-      <c r="G632" t="inlineStr"/>
-      <c r="H632" t="inlineStr"/>
     </row>
     <row r="633">
       <c r="A633" t="inlineStr">
@@ -23928,9 +23901,6 @@
           <t>[ROUTINE] Insider trade — Fang Andy (Director) sold 15,000 shares @ $215.00 ($3.23M) on 2026-08-06</t>
         </is>
       </c>
-      <c r="F633" t="inlineStr"/>
-      <c r="G633" t="inlineStr"/>
-      <c r="H633" t="inlineStr"/>
     </row>
     <row r="634">
       <c r="A634" t="inlineStr">
@@ -23958,9 +23928,6 @@
           <t>New senior role: Chief of Staff, Online Grocery</t>
         </is>
       </c>
-      <c r="F634" t="inlineStr"/>
-      <c r="G634" t="inlineStr"/>
-      <c r="H634" t="inlineStr"/>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr">
@@ -23988,9 +23955,6 @@
           <t>New senior role: Chief of Staff, Online Grocery</t>
         </is>
       </c>
-      <c r="F635" t="inlineStr"/>
-      <c r="G635" t="inlineStr"/>
-      <c r="H635" t="inlineStr"/>
     </row>
     <row r="636">
       <c r="A636" t="inlineStr">
@@ -24018,9 +23982,6 @@
           <t>New senior role: Director of Customer Success</t>
         </is>
       </c>
-      <c r="F636" t="inlineStr"/>
-      <c r="G636" t="inlineStr"/>
-      <c r="H636" t="inlineStr"/>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
@@ -24048,9 +24009,6 @@
           <t>43 new non-senior roles posted</t>
         </is>
       </c>
-      <c r="F637" t="inlineStr"/>
-      <c r="G637" t="inlineStr"/>
-      <c r="H637" t="inlineStr"/>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr">
@@ -24078,9 +24036,6 @@
           <t>newsroom: change detected</t>
         </is>
       </c>
-      <c r="F638" t="inlineStr"/>
-      <c r="G638" t="inlineStr"/>
-      <c r="H638" t="inlineStr"/>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
@@ -24108,9 +24063,666 @@
           <t>[ROUTINE] Insider trade — Rogers Chris (President and CEO) sold 4,933 shares @ $50.00 ($246.7K) on 2026-08-07</t>
         </is>
       </c>
-      <c r="F639" t="inlineStr"/>
-      <c r="G639" t="inlineStr"/>
-      <c r="H639" t="inlineStr"/>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/press-room/home/post/wix-launches-symphony-by-wix-a-new-standalone-multi-agent-system-built-for-smbs</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>newsroom: Wix Launches Symphony by Wix, a New Standalone Multi-Agent System Built for SMBs</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr"/>
+      <c r="G640" t="inlineStr"/>
+      <c r="H640" t="inlineStr"/>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>https://support.wix.com/en/article/terms-of-use</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>terms: change detected</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr"/>
+      <c r="G641" t="inlineStr"/>
+      <c r="H641" t="inlineStr"/>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>WIX</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Wix.com Ltd.</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>https://www.wix.com/upgrade/website</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>pricing: change detected</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr"/>
+      <c r="G642" t="inlineStr"/>
+      <c r="H642" t="inlineStr"/>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>GLBE</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Global-E Online Ltd.</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1835963/000117891326004050/zk2635930.htm</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>[UNKNOWN] Form 6-K</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr"/>
+      <c r="G643" t="inlineStr"/>
+      <c r="H643" t="inlineStr"/>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>GLBE</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Global-E Online Ltd.</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1835963/000119312526343811/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Schlachet Amir (CEO) sold 322 shares @ $42.07 ($13.5K) on 2026-08-10</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr"/>
+      <c r="G644" t="inlineStr"/>
+      <c r="H644" t="inlineStr"/>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>GLBE</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Global-E Online Ltd.</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1835963/000119312526342619/xslF345X06/ownership.xml</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Schlachet Amir (CEO) sold 100,000 shares @ $42.20 ($4.22M) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr"/>
+      <c r="G645" t="inlineStr"/>
+      <c r="H645" t="inlineStr"/>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>eBay Inc.</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1065088/000106508826000181/xslF345X06/form4.xml</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Rebecca Spencer (VP, Chief Accounting Officer) sold 5,190 shares @ $107.79 ($559.4K) on 2026-08-10</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr"/>
+      <c r="G646" t="inlineStr"/>
+      <c r="H646" t="inlineStr"/>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Wayfair Inc.</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1616707/000195917326005813/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Shah Niraj (Officer) plans to sell 6,000 shares (~$636.0K) on/after 08/10/2026</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr"/>
+      <c r="G647" t="inlineStr"/>
+      <c r="H647" t="inlineStr"/>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Wayfair Inc.</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1616707/000195917326005812/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Conine Steven (Officer) plans to sell 6,000 shares (~$636.0K) on/after 08/10/2026</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr"/>
+      <c r="G648" t="inlineStr"/>
+      <c r="H648" t="inlineStr"/>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Maplebear Inc. (Instacart)</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/instacart</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>1 new non-senior roles posted</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr"/>
+      <c r="G649" t="inlineStr"/>
+      <c r="H649" t="inlineStr"/>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Zillow Group Inc.</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1617640/000192109426000831/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Cormier Thielke Claire (Director) plans to sell 1,187 shares (~$39.3K) on/after 08/11/2026</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr"/>
+      <c r="G650" t="inlineStr"/>
+      <c r="H650" t="inlineStr"/>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>CSGP</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>CoStar Group Inc.</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1057352/000147276226000012/xslF345X06/wk-form4_1786392398.xml</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Cann Cynthia Cammett (Chief Accounting Officer) sold 4,788 shares @ $30.78 ($147.4K) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr"/>
+      <c r="G651" t="inlineStr"/>
+      <c r="H651" t="inlineStr"/>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>CSGP</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>CoStar Group Inc.</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1057352/000135168926000005/xslF345X06/wk-form4_1786392390.xml</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Hill John W (Director) sold 3,500 shares @ $30.21 ($105.7K) on 2026-08-05</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr"/>
+      <c r="G652" t="inlineStr"/>
+      <c r="H652" t="inlineStr"/>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>APPF</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>AppFolio Inc.</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1433195/000195004726007950/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Pickering Evan (Officer) plans to sell 141 shares (~$28.1K) on/after 08/11/2026</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr"/>
+      <c r="G653" t="inlineStr"/>
+      <c r="H653" t="inlineStr"/>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>APPF</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>AppFolio Inc.</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1433195/000093833326000012/xslF345X06/form4-08102026_090836.xml</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Maurice J Duca (10%+ owner) sold 5,809 shares @ $198.44 ($1.15M) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr"/>
+      <c r="G654" t="inlineStr"/>
+      <c r="H654" t="inlineStr"/>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>APPF</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>AppFolio Inc.</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1433195/000093833326000011/xslF345X06/form4-08102026_090853.xml</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Maurice J Duca (10%+ owner) sold 15,591 shares @ $194.65 ($3.03M) on 2026-08-06</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr"/>
+      <c r="G655" t="inlineStr"/>
+      <c r="H655" t="inlineStr"/>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>APPF</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>AppFolio Inc.</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1433195/000195004726007880/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — Rigler Don (Officer) plans to sell 300 shares (~$59.6K) on/after 08/10/2026</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr"/>
+      <c r="G656" t="inlineStr"/>
+      <c r="H656" t="inlineStr"/>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Block Inc. (fmr. Square)</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1512673/000162828026055837/xslF345X06/wk-form4_1786485228.xml</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Eisen Anthony Mathew (Director) sold 18,000 shares @ $78.73 ($1.42M) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr"/>
+      <c r="G657" t="inlineStr"/>
+      <c r="H657" t="inlineStr"/>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Block Inc. (fmr. Square)</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1512673/000195004726007931/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — M Eisen Anthony (Director) plans to sell 6,000 shares (~$472.9K) on/after 08/11/2026</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr"/>
+      <c r="G658" t="inlineStr"/>
+      <c r="H658" t="inlineStr"/>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Block Inc. (fmr. Square)</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1512673/000195004726007863/xsl144X01/primary_doc.xml</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Notice of proposed insider sale — M Eisen Anthony (Director) plans to sell 6,000 shares (~$470.8K) on/after 08/10/2026</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr"/>
+      <c r="G659" t="inlineStr"/>
+      <c r="H659" t="inlineStr"/>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>WSM</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Williams-Sonoma Inc.</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/719955/000071995526000196/xslF345X06/form4.xml</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>[ROUTINE] Insider trade — Yearout Karalyn (EVP CHIEF TALENT OFFICER) sold 522 shares @ $246.39 ($128.6K) on 2026-08-07</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr"/>
+      <c r="G660" t="inlineStr"/>
+      <c r="H660" t="inlineStr"/>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>ONON</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>On Holding AG</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1858985/000185898526000018/onholdingag-20260630.htm</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>[UNKNOWN] Form 6-K</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr"/>
+      <c r="G661" t="inlineStr"/>
+      <c r="H661" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix medium-tier URLs — verified content, blank SPA/dead pages
Mechanical probe over the IP-independent medium-tier failures (dead hosts +
404s). Verified each candidate actually yields extractable text, not just a
200. 10 confirmed real (WSM IR+careers, SEZL mgmt+news, ENVA news, SGI
news+terms, W news, MTCH news+careers); 4 JS-only pages blanked (UPST/terms,
GLBE/careers, ENVA/careers, W/terms); 3 non-existent pricing pages blanked
(DASH, W, SGI). 6 IR-platform sites left for the CI re-verify to judge.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -888,11 +888,7 @@
           <t>https://investors.global-e.com/corporate-governance/management-team</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>https://www.global-e.com/careers/</t>
-        </is>
-      </c>
+      <c r="G4" s="4" t="n"/>
       <c r="H4" s="4" t="inlineStr">
         <is>
           <t>https://www.global-e.com/platform/</t>
@@ -1138,7 +1134,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.wayfair.com/media-room/</t>
+          <t>https://investor.wayfair.com/news</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -1151,16 +1147,8 @@
           <t>https://www.aboutwayfair.com/careers</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>https://partners.wayfair.com/</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>https://www.wayfair.com/terms-conditions/</t>
-        </is>
-      </c>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="inlineStr">
         <is>
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=W</t>
@@ -1409,11 +1397,7 @@
           <t>https://careers.doordash.com</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>https://merchants.doordash.com/en-us/products/merchant-pricing</t>
-        </is>
-      </c>
+      <c r="H10" s="4" t="n"/>
       <c r="I10" s="4" t="inlineStr">
         <is>
           <t>https://help.doordash.com/consumers/s/terms-of-service</t>
@@ -1659,7 +1643,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://ir.mtch.com/investor-relations/news-events/news-events/default.aspx</t>
+          <t>https://mtch.com/news</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -1669,7 +1653,7 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.mtch.com</t>
+          <t>https://mtch.com/careers</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -2605,12 +2589,12 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://www.sezzle.com/blog</t>
+          <t>https://sezzle.com/news</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>https://investors.sezzle.com/leadership/default.aspx</t>
+          <t>https://sezzle.com/governance/leadership</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -2686,7 +2670,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>https://ir.dave.com</t>
+          <t>https://investors.dave.com</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -3139,11 +3123,7 @@
           <t>https://www.upstart.com/</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>https://www.upstart.com/terms</t>
-        </is>
-      </c>
+      <c r="I30" s="4" t="n"/>
       <c r="J30" s="4" t="inlineStr">
         <is>
           <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=UPST</t>
@@ -3288,7 +3268,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>https://ir.williams-sonoma.com</t>
+          <t>https://ir.williams-sonomainc.com</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -3303,7 +3283,7 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>https://careers.williams-sonoma.com</t>
+          <t>https://www.williams-sonoma.com/careers</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -3379,7 +3359,7 @@
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>https://somnigroup.com/newsroom/default.aspx</t>
+          <t>https://www.somnigroup.com/news</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
@@ -3392,14 +3372,10 @@
           <t>https://somnigroup.com/careers/default.aspx</t>
         </is>
       </c>
-      <c r="H33" s="7" t="inlineStr">
-        <is>
-          <t>https://www.tempurpedic.com/shop-mattresses/</t>
-        </is>
-      </c>
+      <c r="H33" s="7" t="n"/>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>https://somnigroup.com/legal/default.aspx</t>
+          <t>https://www.somnigroup.com/terms</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
@@ -3465,7 +3441,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://ir.enova.com/news-events/news-releases/default.aspx</t>
+          <t>https://www.enova.com/newsroom</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -3473,11 +3449,7 @@
           <t>https://ir.enova.com/corporate-governance/leadership-team/default.aspx</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>https://www.enova.com/careers/</t>
-        </is>
-      </c>
+      <c r="G34" s="4" t="n"/>
       <c r="H34" s="4" t="inlineStr">
         <is>
           <t>https://www.enova.com/brands/</t>
@@ -6248,600 +6220,593 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId613"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6853,7 +6818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H661"/>
+  <dimension ref="A1:H639"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -24063,666 +24028,6 @@
           <t>[ROUTINE] Insider trade — Rogers Chris (President and CEO) sold 4,933 shares @ $50.00 ($246.7K) on 2026-08-07</t>
         </is>
       </c>
-    </row>
-    <row r="640">
-      <c r="A640" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B640" t="inlineStr">
-        <is>
-          <t>WIX</t>
-        </is>
-      </c>
-      <c r="C640" t="inlineStr">
-        <is>
-          <t>Wix.com Ltd.</t>
-        </is>
-      </c>
-      <c r="D640" t="inlineStr">
-        <is>
-          <t>https://www.wix.com/press-room/home/post/wix-launches-symphony-by-wix-a-new-standalone-multi-agent-system-built-for-smbs</t>
-        </is>
-      </c>
-      <c r="E640" t="inlineStr">
-        <is>
-          <t>newsroom: Wix Launches Symphony by Wix, a New Standalone Multi-Agent System Built for SMBs</t>
-        </is>
-      </c>
-      <c r="F640" t="inlineStr"/>
-      <c r="G640" t="inlineStr"/>
-      <c r="H640" t="inlineStr"/>
-    </row>
-    <row r="641">
-      <c r="A641" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B641" t="inlineStr">
-        <is>
-          <t>WIX</t>
-        </is>
-      </c>
-      <c r="C641" t="inlineStr">
-        <is>
-          <t>Wix.com Ltd.</t>
-        </is>
-      </c>
-      <c r="D641" t="inlineStr">
-        <is>
-          <t>https://support.wix.com/en/article/terms-of-use</t>
-        </is>
-      </c>
-      <c r="E641" t="inlineStr">
-        <is>
-          <t>terms: change detected</t>
-        </is>
-      </c>
-      <c r="F641" t="inlineStr"/>
-      <c r="G641" t="inlineStr"/>
-      <c r="H641" t="inlineStr"/>
-    </row>
-    <row r="642">
-      <c r="A642" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B642" t="inlineStr">
-        <is>
-          <t>WIX</t>
-        </is>
-      </c>
-      <c r="C642" t="inlineStr">
-        <is>
-          <t>Wix.com Ltd.</t>
-        </is>
-      </c>
-      <c r="D642" t="inlineStr">
-        <is>
-          <t>https://www.wix.com/upgrade/website</t>
-        </is>
-      </c>
-      <c r="E642" t="inlineStr">
-        <is>
-          <t>pricing: change detected</t>
-        </is>
-      </c>
-      <c r="F642" t="inlineStr"/>
-      <c r="G642" t="inlineStr"/>
-      <c r="H642" t="inlineStr"/>
-    </row>
-    <row r="643">
-      <c r="A643" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B643" t="inlineStr">
-        <is>
-          <t>GLBE</t>
-        </is>
-      </c>
-      <c r="C643" t="inlineStr">
-        <is>
-          <t>Global-E Online Ltd.</t>
-        </is>
-      </c>
-      <c r="D643" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1835963/000117891326004050/zk2635930.htm</t>
-        </is>
-      </c>
-      <c r="E643" t="inlineStr">
-        <is>
-          <t>[UNKNOWN] Form 6-K</t>
-        </is>
-      </c>
-      <c r="F643" t="inlineStr"/>
-      <c r="G643" t="inlineStr"/>
-      <c r="H643" t="inlineStr"/>
-    </row>
-    <row r="644">
-      <c r="A644" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B644" t="inlineStr">
-        <is>
-          <t>GLBE</t>
-        </is>
-      </c>
-      <c r="C644" t="inlineStr">
-        <is>
-          <t>Global-E Online Ltd.</t>
-        </is>
-      </c>
-      <c r="D644" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1835963/000119312526343811/xslF345X06/ownership.xml</t>
-        </is>
-      </c>
-      <c r="E644" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Insider trade — Schlachet Amir (CEO) sold 322 shares @ $42.07 ($13.5K) on 2026-08-10</t>
-        </is>
-      </c>
-      <c r="F644" t="inlineStr"/>
-      <c r="G644" t="inlineStr"/>
-      <c r="H644" t="inlineStr"/>
-    </row>
-    <row r="645">
-      <c r="A645" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B645" t="inlineStr">
-        <is>
-          <t>GLBE</t>
-        </is>
-      </c>
-      <c r="C645" t="inlineStr">
-        <is>
-          <t>Global-E Online Ltd.</t>
-        </is>
-      </c>
-      <c r="D645" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1835963/000119312526342619/xslF345X06/ownership.xml</t>
-        </is>
-      </c>
-      <c r="E645" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Insider trade — Schlachet Amir (CEO) sold 100,000 shares @ $42.20 ($4.22M) on 2026-08-07</t>
-        </is>
-      </c>
-      <c r="F645" t="inlineStr"/>
-      <c r="G645" t="inlineStr"/>
-      <c r="H645" t="inlineStr"/>
-    </row>
-    <row r="646">
-      <c r="A646" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B646" t="inlineStr">
-        <is>
-          <t>EBAY</t>
-        </is>
-      </c>
-      <c r="C646" t="inlineStr">
-        <is>
-          <t>eBay Inc.</t>
-        </is>
-      </c>
-      <c r="D646" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1065088/000106508826000181/xslF345X06/form4.xml</t>
-        </is>
-      </c>
-      <c r="E646" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Insider trade — Rebecca Spencer (VP, Chief Accounting Officer) sold 5,190 shares @ $107.79 ($559.4K) on 2026-08-10</t>
-        </is>
-      </c>
-      <c r="F646" t="inlineStr"/>
-      <c r="G646" t="inlineStr"/>
-      <c r="H646" t="inlineStr"/>
-    </row>
-    <row r="647">
-      <c r="A647" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B647" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="C647" t="inlineStr">
-        <is>
-          <t>Wayfair Inc.</t>
-        </is>
-      </c>
-      <c r="D647" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1616707/000195917326005813/xsl144X01/primary_doc.xml</t>
-        </is>
-      </c>
-      <c r="E647" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Notice of proposed insider sale — Shah Niraj (Officer) plans to sell 6,000 shares (~$636.0K) on/after 08/10/2026</t>
-        </is>
-      </c>
-      <c r="F647" t="inlineStr"/>
-      <c r="G647" t="inlineStr"/>
-      <c r="H647" t="inlineStr"/>
-    </row>
-    <row r="648">
-      <c r="A648" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B648" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="C648" t="inlineStr">
-        <is>
-          <t>Wayfair Inc.</t>
-        </is>
-      </c>
-      <c r="D648" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1616707/000195917326005812/xsl144X01/primary_doc.xml</t>
-        </is>
-      </c>
-      <c r="E648" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Notice of proposed insider sale — Conine Steven (Officer) plans to sell 6,000 shares (~$636.0K) on/after 08/10/2026</t>
-        </is>
-      </c>
-      <c r="F648" t="inlineStr"/>
-      <c r="G648" t="inlineStr"/>
-      <c r="H648" t="inlineStr"/>
-    </row>
-    <row r="649">
-      <c r="A649" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B649" t="inlineStr">
-        <is>
-          <t>CART</t>
-        </is>
-      </c>
-      <c r="C649" t="inlineStr">
-        <is>
-          <t>Maplebear Inc. (Instacart)</t>
-        </is>
-      </c>
-      <c r="D649" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/instacart</t>
-        </is>
-      </c>
-      <c r="E649" t="inlineStr">
-        <is>
-          <t>1 new non-senior roles posted</t>
-        </is>
-      </c>
-      <c r="F649" t="inlineStr"/>
-      <c r="G649" t="inlineStr"/>
-      <c r="H649" t="inlineStr"/>
-    </row>
-    <row r="650">
-      <c r="A650" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B650" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="C650" t="inlineStr">
-        <is>
-          <t>Zillow Group Inc.</t>
-        </is>
-      </c>
-      <c r="D650" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1617640/000192109426000831/xsl144X01/primary_doc.xml</t>
-        </is>
-      </c>
-      <c r="E650" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Notice of proposed insider sale — Cormier Thielke Claire (Director) plans to sell 1,187 shares (~$39.3K) on/after 08/11/2026</t>
-        </is>
-      </c>
-      <c r="F650" t="inlineStr"/>
-      <c r="G650" t="inlineStr"/>
-      <c r="H650" t="inlineStr"/>
-    </row>
-    <row r="651">
-      <c r="A651" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B651" t="inlineStr">
-        <is>
-          <t>CSGP</t>
-        </is>
-      </c>
-      <c r="C651" t="inlineStr">
-        <is>
-          <t>CoStar Group Inc.</t>
-        </is>
-      </c>
-      <c r="D651" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1057352/000147276226000012/xslF345X06/wk-form4_1786392398.xml</t>
-        </is>
-      </c>
-      <c r="E651" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Insider trade — Cann Cynthia Cammett (Chief Accounting Officer) sold 4,788 shares @ $30.78 ($147.4K) on 2026-08-07</t>
-        </is>
-      </c>
-      <c r="F651" t="inlineStr"/>
-      <c r="G651" t="inlineStr"/>
-      <c r="H651" t="inlineStr"/>
-    </row>
-    <row r="652">
-      <c r="A652" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B652" t="inlineStr">
-        <is>
-          <t>CSGP</t>
-        </is>
-      </c>
-      <c r="C652" t="inlineStr">
-        <is>
-          <t>CoStar Group Inc.</t>
-        </is>
-      </c>
-      <c r="D652" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1057352/000135168926000005/xslF345X06/wk-form4_1786392390.xml</t>
-        </is>
-      </c>
-      <c r="E652" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Insider trade — Hill John W (Director) sold 3,500 shares @ $30.21 ($105.7K) on 2026-08-05</t>
-        </is>
-      </c>
-      <c r="F652" t="inlineStr"/>
-      <c r="G652" t="inlineStr"/>
-      <c r="H652" t="inlineStr"/>
-    </row>
-    <row r="653">
-      <c r="A653" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B653" t="inlineStr">
-        <is>
-          <t>APPF</t>
-        </is>
-      </c>
-      <c r="C653" t="inlineStr">
-        <is>
-          <t>AppFolio Inc.</t>
-        </is>
-      </c>
-      <c r="D653" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1433195/000195004726007950/xsl144X01/primary_doc.xml</t>
-        </is>
-      </c>
-      <c r="E653" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Notice of proposed insider sale — Pickering Evan (Officer) plans to sell 141 shares (~$28.1K) on/after 08/11/2026</t>
-        </is>
-      </c>
-      <c r="F653" t="inlineStr"/>
-      <c r="G653" t="inlineStr"/>
-      <c r="H653" t="inlineStr"/>
-    </row>
-    <row r="654">
-      <c r="A654" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B654" t="inlineStr">
-        <is>
-          <t>APPF</t>
-        </is>
-      </c>
-      <c r="C654" t="inlineStr">
-        <is>
-          <t>AppFolio Inc.</t>
-        </is>
-      </c>
-      <c r="D654" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1433195/000093833326000012/xslF345X06/form4-08102026_090836.xml</t>
-        </is>
-      </c>
-      <c r="E654" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Insider trade — Maurice J Duca (10%+ owner) sold 5,809 shares @ $198.44 ($1.15M) on 2026-08-07</t>
-        </is>
-      </c>
-      <c r="F654" t="inlineStr"/>
-      <c r="G654" t="inlineStr"/>
-      <c r="H654" t="inlineStr"/>
-    </row>
-    <row r="655">
-      <c r="A655" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B655" t="inlineStr">
-        <is>
-          <t>APPF</t>
-        </is>
-      </c>
-      <c r="C655" t="inlineStr">
-        <is>
-          <t>AppFolio Inc.</t>
-        </is>
-      </c>
-      <c r="D655" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1433195/000093833326000011/xslF345X06/form4-08102026_090853.xml</t>
-        </is>
-      </c>
-      <c r="E655" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Insider trade — Maurice J Duca (10%+ owner) sold 15,591 shares @ $194.65 ($3.03M) on 2026-08-06</t>
-        </is>
-      </c>
-      <c r="F655" t="inlineStr"/>
-      <c r="G655" t="inlineStr"/>
-      <c r="H655" t="inlineStr"/>
-    </row>
-    <row r="656">
-      <c r="A656" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B656" t="inlineStr">
-        <is>
-          <t>APPF</t>
-        </is>
-      </c>
-      <c r="C656" t="inlineStr">
-        <is>
-          <t>AppFolio Inc.</t>
-        </is>
-      </c>
-      <c r="D656" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1433195/000195004726007880/xsl144X01/primary_doc.xml</t>
-        </is>
-      </c>
-      <c r="E656" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Notice of proposed insider sale — Rigler Don (Officer) plans to sell 300 shares (~$59.6K) on/after 08/10/2026</t>
-        </is>
-      </c>
-      <c r="F656" t="inlineStr"/>
-      <c r="G656" t="inlineStr"/>
-      <c r="H656" t="inlineStr"/>
-    </row>
-    <row r="657">
-      <c r="A657" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B657" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C657" t="inlineStr">
-        <is>
-          <t>Block Inc. (fmr. Square)</t>
-        </is>
-      </c>
-      <c r="D657" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1512673/000162828026055837/xslF345X06/wk-form4_1786485228.xml</t>
-        </is>
-      </c>
-      <c r="E657" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Insider trade — Eisen Anthony Mathew (Director) sold 18,000 shares @ $78.73 ($1.42M) on 2026-08-07</t>
-        </is>
-      </c>
-      <c r="F657" t="inlineStr"/>
-      <c r="G657" t="inlineStr"/>
-      <c r="H657" t="inlineStr"/>
-    </row>
-    <row r="658">
-      <c r="A658" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B658" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C658" t="inlineStr">
-        <is>
-          <t>Block Inc. (fmr. Square)</t>
-        </is>
-      </c>
-      <c r="D658" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1512673/000195004726007931/xsl144X01/primary_doc.xml</t>
-        </is>
-      </c>
-      <c r="E658" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Notice of proposed insider sale — M Eisen Anthony (Director) plans to sell 6,000 shares (~$472.9K) on/after 08/11/2026</t>
-        </is>
-      </c>
-      <c r="F658" t="inlineStr"/>
-      <c r="G658" t="inlineStr"/>
-      <c r="H658" t="inlineStr"/>
-    </row>
-    <row r="659">
-      <c r="A659" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B659" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C659" t="inlineStr">
-        <is>
-          <t>Block Inc. (fmr. Square)</t>
-        </is>
-      </c>
-      <c r="D659" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1512673/000195004726007863/xsl144X01/primary_doc.xml</t>
-        </is>
-      </c>
-      <c r="E659" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Notice of proposed insider sale — M Eisen Anthony (Director) plans to sell 6,000 shares (~$470.8K) on/after 08/10/2026</t>
-        </is>
-      </c>
-      <c r="F659" t="inlineStr"/>
-      <c r="G659" t="inlineStr"/>
-      <c r="H659" t="inlineStr"/>
-    </row>
-    <row r="660">
-      <c r="A660" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B660" t="inlineStr">
-        <is>
-          <t>WSM</t>
-        </is>
-      </c>
-      <c r="C660" t="inlineStr">
-        <is>
-          <t>Williams-Sonoma Inc.</t>
-        </is>
-      </c>
-      <c r="D660" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/719955/000071995526000196/xslF345X06/form4.xml</t>
-        </is>
-      </c>
-      <c r="E660" t="inlineStr">
-        <is>
-          <t>[ROUTINE] Insider trade — Yearout Karalyn (EVP CHIEF TALENT OFFICER) sold 522 shares @ $246.39 ($128.6K) on 2026-08-07</t>
-        </is>
-      </c>
-      <c r="F660" t="inlineStr"/>
-      <c r="G660" t="inlineStr"/>
-      <c r="H660" t="inlineStr"/>
-    </row>
-    <row r="661">
-      <c r="A661" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B661" t="inlineStr">
-        <is>
-          <t>ONON</t>
-        </is>
-      </c>
-      <c r="C661" t="inlineStr">
-        <is>
-          <t>On Holding AG</t>
-        </is>
-      </c>
-      <c r="D661" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1858985/000185898526000018/onholdingag-20260630.htm</t>
-        </is>
-      </c>
-      <c r="E661" t="inlineStr">
-        <is>
-          <t>[UNKNOWN] Form 6-K</t>
-        </is>
-      </c>
-      <c r="F661" t="inlineStr"/>
-      <c r="G661" t="inlineStr"/>
-      <c r="H661" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Restructure coverage into two analyst lists (source of truth in xlsx)
- xlsx: new "Analyst" column assigns each name to 1 (41 names) or 2 (35).
  ARMK/CVNA/HQY/VRSK are in neither list → Active=FALSE (dropped).
- config_reader: read the Analyst column into Company.analyst.
- run.py: add --analyst {1,2} selector (filters by that column); blocked
  names (analyst 2 owns a few foreign ones) are skipped with a log line.
- monitor.yml: daily schedule now scrapes BOTH analysts and sends each their
  own digest — Analyst 1 → EMAIL_TO, Analyst 2 → EMAIL_TO_2 (soft-skips until
  that secret is set). Manual dispatch gains an `analyst` input.

Analyst 1 and 2 are disjoint, so per-name snapshots never collide.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/company_urls_jc.xlsx
+++ b/config/company_urls_jc.xlsx
@@ -547,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T81"/>
+  <dimension ref="A1:U81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -665,6 +665,11 @@
           <t>Pricing Selector</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Analyst</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="52" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -760,6 +765,11 @@
           <t>main</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -856,6 +866,11 @@
           <t>main</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="52" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -938,6 +953,11 @@
       <c r="R4" t="b">
         <v>1</v>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="52" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -1024,6 +1044,11 @@
       <c r="R5" t="b">
         <v>1</v>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -1109,6 +1134,11 @@
       </c>
       <c r="R6" t="b">
         <v>1</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="52" customHeight="1">
@@ -1188,6 +1218,11 @@
       <c r="R7" t="b">
         <v>1</v>
       </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1274,6 +1309,11 @@
       <c r="R8" t="b">
         <v>1</v>
       </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="52" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -1360,6 +1400,11 @@
       <c r="R9" t="b">
         <v>1</v>
       </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="52" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1442,6 +1487,11 @@
       <c r="R10" t="b">
         <v>1</v>
       </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="52" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1533,6 +1583,11 @@
           <t>main</t>
         </is>
       </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="52" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1619,6 +1674,11 @@
       <c r="R12" t="b">
         <v>1</v>
       </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="52" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1705,6 +1765,11 @@
       <c r="R13" t="b">
         <v>1</v>
       </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="52" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1791,6 +1856,11 @@
       <c r="R14" t="b">
         <v>1</v>
       </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="52" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1877,6 +1947,11 @@
       <c r="R15" t="b">
         <v>1</v>
       </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="52" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1963,6 +2038,11 @@
       <c r="R16" t="b">
         <v>1</v>
       </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="52" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -2049,6 +2129,11 @@
       <c r="R17" t="b">
         <v>1</v>
       </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="52" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -2135,6 +2220,11 @@
       <c r="R18" t="b">
         <v>1</v>
       </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="52" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
@@ -2221,6 +2311,11 @@
       <c r="R19" t="b">
         <v>1</v>
       </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="52" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -2307,6 +2402,11 @@
       <c r="R20" t="b">
         <v>1</v>
       </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="52" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -2393,6 +2493,11 @@
       <c r="R21" t="b">
         <v>1</v>
       </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="52" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -2479,6 +2584,11 @@
       <c r="R22" t="b">
         <v>1</v>
       </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="52" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -2565,6 +2675,11 @@
       <c r="R23" t="b">
         <v>1</v>
       </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="52" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -2651,6 +2766,11 @@
       <c r="R24" t="b">
         <v>1</v>
       </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="52" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -2737,6 +2857,11 @@
       <c r="R25" t="b">
         <v>1</v>
       </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="52" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -2823,6 +2948,11 @@
       <c r="R26" t="b">
         <v>1</v>
       </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="52" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -2909,6 +3039,11 @@
       <c r="R27" t="b">
         <v>1</v>
       </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="52" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -2995,6 +3130,11 @@
       <c r="R28" t="b">
         <v>1</v>
       </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="52" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -3081,6 +3221,11 @@
       <c r="R29" t="b">
         <v>1</v>
       </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="52" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -3163,6 +3308,11 @@
       <c r="R30" t="b">
         <v>1</v>
       </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="52" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -3249,6 +3399,11 @@
       <c r="R31" t="b">
         <v>1</v>
       </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="52" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -3335,6 +3490,11 @@
       <c r="R32" t="b">
         <v>1</v>
       </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="52" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -3417,6 +3577,11 @@
       <c r="R33" t="b">
         <v>1</v>
       </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="52" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -3499,6 +3664,11 @@
       <c r="R34" t="b">
         <v>1</v>
       </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="52" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -3585,6 +3755,11 @@
       <c r="R35" t="b">
         <v>1</v>
       </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="52" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -3671,6 +3846,11 @@
       <c r="R36" t="b">
         <v>1</v>
       </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3731,6 +3911,11 @@
       <c r="R37" t="b">
         <v>1</v>
       </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3796,6 +3981,11 @@
       <c r="R38" t="b">
         <v>1</v>
       </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3836,6 +4026,11 @@
       <c r="R39" t="b">
         <v>1</v>
       </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3906,6 +4101,11 @@
       <c r="R40" t="b">
         <v>1</v>
       </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3956,6 +4156,11 @@
       <c r="R41" t="b">
         <v>1</v>
       </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4021,6 +4226,11 @@
       <c r="R42" t="b">
         <v>1</v>
       </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4081,6 +4291,11 @@
       <c r="R43" t="b">
         <v>1</v>
       </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4146,6 +4361,11 @@
       <c r="R44" t="b">
         <v>1</v>
       </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4211,6 +4431,11 @@
       <c r="R45" t="b">
         <v>1</v>
       </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4269,7 +4494,7 @@
         </is>
       </c>
       <c r="R46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -4334,7 +4559,7 @@
         </is>
       </c>
       <c r="R47" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -4394,7 +4619,7 @@
         </is>
       </c>
       <c r="R48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -4454,7 +4679,7 @@
         </is>
       </c>
       <c r="R49" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -4511,6 +4736,11 @@
       <c r="R50" t="b">
         <v>1</v>
       </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4566,6 +4796,11 @@
       <c r="R51" t="b">
         <v>1</v>
       </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4626,6 +4861,11 @@
       <c r="R52" t="b">
         <v>1</v>
       </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4686,6 +4926,11 @@
       <c r="R53" t="b">
         <v>1</v>
       </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4746,6 +4991,11 @@
       <c r="R54" t="b">
         <v>1</v>
       </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4801,6 +5051,11 @@
       <c r="R55" t="b">
         <v>1</v>
       </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4861,6 +5116,11 @@
       <c r="R56" t="b">
         <v>1</v>
       </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4916,6 +5176,11 @@
       <c r="R57" t="b">
         <v>1</v>
       </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4971,6 +5236,11 @@
       <c r="R58" t="b">
         <v>1</v>
       </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5031,6 +5301,11 @@
       <c r="R59" t="b">
         <v>1</v>
       </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5091,6 +5366,11 @@
       <c r="R60" t="b">
         <v>1</v>
       </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5146,6 +5426,11 @@
       <c r="R61" t="b">
         <v>1</v>
       </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5181,6 +5466,11 @@
       <c r="R62" t="b">
         <v>1</v>
       </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5236,6 +5526,11 @@
       <c r="R63" t="b">
         <v>1</v>
       </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5296,6 +5591,11 @@
       <c r="R64" t="b">
         <v>1</v>
       </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5351,6 +5651,11 @@
       <c r="R65" t="b">
         <v>1</v>
       </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5401,6 +5706,11 @@
       <c r="R66" t="b">
         <v>1</v>
       </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5456,6 +5766,11 @@
       <c r="R67" t="b">
         <v>1</v>
       </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5511,6 +5826,11 @@
       <c r="R68" t="b">
         <v>1</v>
       </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5566,6 +5886,11 @@
       <c r="R69" t="b">
         <v>1</v>
       </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5601,6 +5926,11 @@
       <c r="R70" t="b">
         <v>1</v>
       </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5656,6 +5986,11 @@
       <c r="R71" t="b">
         <v>1</v>
       </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5711,6 +6046,11 @@
       <c r="R72" t="b">
         <v>1</v>
       </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5761,6 +6101,11 @@
       <c r="R73" t="b">
         <v>1</v>
       </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5816,6 +6161,11 @@
       <c r="R74" t="b">
         <v>1</v>
       </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5871,6 +6221,11 @@
       <c r="R75" t="b">
         <v>1</v>
       </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5931,6 +6286,11 @@
       <c r="R76" t="b">
         <v>1</v>
       </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5986,6 +6346,11 @@
       <c r="R77" t="b">
         <v>1</v>
       </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6041,6 +6406,11 @@
       <c r="R78" t="b">
         <v>1</v>
       </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6081,6 +6451,11 @@
       <c r="R79" t="b">
         <v>1</v>
       </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6136,6 +6511,11 @@
       <c r="R80" t="b">
         <v>1</v>
       </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6190,6 +6570,11 @@
       </c>
       <c r="R81" t="b">
         <v>1</v>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>